<commit_message>
Actualizacion de estatus y pendientes XD
</commit_message>
<xml_diff>
--- a/validaciones_Y_ChecklistDeRequerimeintos/Copia de CheckList_Estatus-001-V.1.5DEV (1).xlsx
+++ b/validaciones_Y_ChecklistDeRequerimeintos/Copia de CheckList_Estatus-001-V.1.5DEV (1).xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diego\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\isrra\OneDrive\Documentos\GitHub\integradoraTeampoderoso\validaciones_Y_ChecklistDeRequerimeintos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5C6173F-8E1D-4B33-9F4E-7A9EF3B4A6B6}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B7610F5-EC99-4A8D-9882-E5096C7A9C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="586" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20640" windowHeight="11040" tabRatio="586" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFECTOS" sheetId="4" r:id="rId1"/>
     <sheet name="CBS" sheetId="6" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DEFECTOS!$A$1:$M$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DEFECTOS!$A$1:$M$14</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -609,21 +609,21 @@
   <dxfs count="61">
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -698,17 +698,6 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -724,6 +713,43 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF7C80"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -746,52 +772,6 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9C0006"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9C0006"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9C0006"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9C0006"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -845,6 +825,38 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <color theme="9" tint="-0.499984740745262"/>
@@ -864,18 +876,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -925,18 +925,6 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color theme="0"/>
       </font>
       <fill>
@@ -948,6 +936,18 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1060,22 +1060,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF7C80"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1101,21 +1100,22 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
+        <b/>
+        <i val="0"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFF7C80"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1141,6 +1141,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <condense val="0"/>
@@ -1152,10 +1162,51 @@
       <font>
         <b/>
         <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF7C80"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1183,57 +1234,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2044,7 +2044,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>6415510</xdr:colOff>
+      <xdr:colOff>6419320</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>2592501</xdr:rowOff>
     </xdr:to>
@@ -2407,22 +2407,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:ATS2317"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15" style="26" customWidth="1"/>
-    <col min="2" max="2" width="100.42578125" style="13" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" style="8" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" style="8" customWidth="1"/>
-    <col min="7" max="7" width="19.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" style="8" customWidth="1"/>
-    <col min="9" max="9" width="20.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="24.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5703125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="23.42578125" style="3" customWidth="1"/>
-    <col min="13" max="13" width="21.42578125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="100.44140625" style="13" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.88671875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="18.44140625" style="8" customWidth="1"/>
+    <col min="7" max="7" width="19.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.44140625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="20.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.5546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="23.44140625" style="3" customWidth="1"/>
+    <col min="13" max="13" width="21.44140625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1215" s="5" customFormat="1" ht="111" customHeight="1">
@@ -2466,7 +2467,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:1215" s="23" customFormat="1" ht="207.6" customHeight="1">
+    <row r="2" spans="1:1215" s="23" customFormat="1" ht="207.6" hidden="1" customHeight="1">
       <c r="A2" s="24" t="s">
         <v>30</v>
       </c>
@@ -3701,7 +3702,7 @@
       <c r="ATR2"/>
       <c r="ATS2"/>
     </row>
-    <row r="3" spans="1:1215" ht="343.5" customHeight="1">
+    <row r="3" spans="1:1215" ht="343.5" hidden="1" customHeight="1">
       <c r="A3" s="24" t="s">
         <v>31</v>
       </c>
@@ -3924,7 +3925,7 @@
       <c r="HB3" s="15"/>
       <c r="HC3" s="15"/>
     </row>
-    <row r="4" spans="1:1215" ht="217.15" customHeight="1">
+    <row r="4" spans="1:1215" ht="217.2" customHeight="1">
       <c r="A4" s="24" t="s">
         <v>32</v>
       </c>
@@ -4147,7 +4148,7 @@
       <c r="HB4" s="15"/>
       <c r="HC4" s="15"/>
     </row>
-    <row r="5" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="5" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A5" s="24" t="s">
         <v>33</v>
       </c>
@@ -4370,7 +4371,7 @@
       <c r="HB5" s="15"/>
       <c r="HC5" s="15"/>
     </row>
-    <row r="6" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="6" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A6" s="24" t="s">
         <v>33</v>
       </c>
@@ -4593,7 +4594,7 @@
       <c r="HB6" s="15"/>
       <c r="HC6" s="15"/>
     </row>
-    <row r="7" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="7" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A7" s="24" t="s">
         <v>33</v>
       </c>
@@ -4816,7 +4817,7 @@
       <c r="HB7" s="15"/>
       <c r="HC7" s="15"/>
     </row>
-    <row r="8" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="8" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A8" s="24" t="s">
         <v>33</v>
       </c>
@@ -5039,7 +5040,7 @@
       <c r="HB8" s="15"/>
       <c r="HC8" s="15"/>
     </row>
-    <row r="9" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="9" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A9" s="24" t="s">
         <v>33</v>
       </c>
@@ -5262,7 +5263,7 @@
       <c r="HB9" s="15"/>
       <c r="HC9" s="15"/>
     </row>
-    <row r="10" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="10" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A10" s="24" t="s">
         <v>33</v>
       </c>
@@ -5485,7 +5486,7 @@
       <c r="HB10" s="15"/>
       <c r="HC10" s="15"/>
     </row>
-    <row r="11" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="11" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A11" s="24" t="s">
         <v>33</v>
       </c>
@@ -5708,7 +5709,7 @@
       <c r="HB11" s="15"/>
       <c r="HC11" s="15"/>
     </row>
-    <row r="12" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="12" spans="1:1215" ht="277.2" customHeight="1">
       <c r="A12" s="24" t="s">
         <v>33</v>
       </c>
@@ -5719,7 +5720,7 @@
         <v>14</v>
       </c>
       <c r="D12" s="34" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E12" s="29" t="s">
         <v>35</v>
@@ -5931,7 +5932,7 @@
       <c r="HB12" s="15"/>
       <c r="HC12" s="15"/>
     </row>
-    <row r="13" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="13" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A13" s="24" t="s">
         <v>33</v>
       </c>
@@ -6154,7 +6155,7 @@
       <c r="HB13" s="15"/>
       <c r="HC13" s="15"/>
     </row>
-    <row r="14" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="14" spans="1:1215" ht="277.2" customHeight="1">
       <c r="A14" s="24" t="s">
         <v>33</v>
       </c>
@@ -6165,7 +6166,7 @@
         <v>14</v>
       </c>
       <c r="D14" s="34" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E14" s="29" t="s">
         <v>35</v>
@@ -12275,1387 +12276,1393 @@
     <row r="1980" spans="1:2">
       <c r="A1980" s="2"/>
     </row>
-    <row r="1981" spans="1:2" ht="12.75">
+    <row r="1981" spans="1:2" ht="13.2">
       <c r="A1981" s="2"/>
       <c r="B1981" s="2"/>
     </row>
-    <row r="1982" spans="1:2" ht="12.75">
+    <row r="1982" spans="1:2" ht="13.2">
       <c r="A1982" s="2"/>
       <c r="B1982" s="2"/>
     </row>
-    <row r="1983" spans="1:2" ht="12.75">
+    <row r="1983" spans="1:2" ht="13.2">
       <c r="A1983" s="2"/>
       <c r="B1983" s="2"/>
     </row>
-    <row r="1984" spans="1:2" ht="12.75">
+    <row r="1984" spans="1:2" ht="13.2">
       <c r="A1984" s="2"/>
       <c r="B1984" s="2"/>
     </row>
-    <row r="1985" spans="1:2" ht="12.75">
+    <row r="1985" spans="1:2" ht="13.2">
       <c r="A1985" s="2"/>
       <c r="B1985" s="2"/>
     </row>
-    <row r="1986" spans="1:2" ht="12.75">
+    <row r="1986" spans="1:2" ht="13.2">
       <c r="A1986" s="2"/>
       <c r="B1986" s="2"/>
     </row>
-    <row r="1987" spans="1:2" ht="12.75">
+    <row r="1987" spans="1:2" ht="13.2">
       <c r="A1987" s="2"/>
       <c r="B1987" s="2"/>
     </row>
-    <row r="1988" spans="1:2" ht="12.75">
+    <row r="1988" spans="1:2" ht="13.2">
       <c r="A1988" s="2"/>
       <c r="B1988" s="2"/>
     </row>
-    <row r="1989" spans="1:2" ht="12.75">
+    <row r="1989" spans="1:2" ht="13.2">
       <c r="A1989" s="2"/>
       <c r="B1989" s="2"/>
     </row>
-    <row r="1990" spans="1:2" ht="12.75">
+    <row r="1990" spans="1:2" ht="13.2">
       <c r="A1990" s="2"/>
       <c r="B1990" s="2"/>
     </row>
-    <row r="1991" spans="1:2" ht="12.75">
+    <row r="1991" spans="1:2" ht="13.2">
       <c r="A1991" s="2"/>
       <c r="B1991" s="2"/>
     </row>
-    <row r="1992" spans="1:2" ht="12.75">
+    <row r="1992" spans="1:2" ht="13.2">
       <c r="A1992" s="2"/>
       <c r="B1992" s="2"/>
     </row>
-    <row r="1993" spans="1:2" ht="12.75">
+    <row r="1993" spans="1:2" ht="13.2">
       <c r="A1993" s="2"/>
       <c r="B1993" s="2"/>
     </row>
-    <row r="1994" spans="1:2" ht="12.75">
+    <row r="1994" spans="1:2" ht="13.2">
       <c r="A1994" s="2"/>
       <c r="B1994" s="2"/>
     </row>
-    <row r="1995" spans="1:2" ht="12.75">
+    <row r="1995" spans="1:2" ht="13.2">
       <c r="A1995" s="2"/>
       <c r="B1995" s="2"/>
     </row>
-    <row r="1996" spans="1:2" ht="12.75">
+    <row r="1996" spans="1:2" ht="13.2">
       <c r="A1996" s="2"/>
       <c r="B1996" s="2"/>
     </row>
-    <row r="1997" spans="1:2" ht="12.75">
+    <row r="1997" spans="1:2" ht="13.2">
       <c r="A1997" s="2"/>
       <c r="B1997" s="2"/>
     </row>
-    <row r="1998" spans="1:2" ht="12.75">
+    <row r="1998" spans="1:2" ht="13.2">
       <c r="A1998" s="2"/>
       <c r="B1998" s="2"/>
     </row>
-    <row r="1999" spans="1:2" ht="12.75">
+    <row r="1999" spans="1:2" ht="13.2">
       <c r="A1999" s="2"/>
       <c r="B1999" s="2"/>
     </row>
-    <row r="2000" spans="1:2" ht="12.75">
+    <row r="2000" spans="1:2" ht="13.2">
       <c r="A2000" s="2"/>
       <c r="B2000" s="2"/>
     </row>
-    <row r="2001" spans="1:2" ht="12.75">
+    <row r="2001" spans="1:2" ht="13.2">
       <c r="A2001" s="2"/>
       <c r="B2001" s="2"/>
     </row>
-    <row r="2002" spans="1:2" ht="12.75">
+    <row r="2002" spans="1:2" ht="13.2">
       <c r="A2002" s="2"/>
       <c r="B2002" s="2"/>
     </row>
-    <row r="2003" spans="1:2" ht="12.75">
+    <row r="2003" spans="1:2" ht="13.2">
       <c r="A2003" s="2"/>
       <c r="B2003" s="2"/>
     </row>
-    <row r="2004" spans="1:2" ht="12.75">
+    <row r="2004" spans="1:2" ht="13.2">
       <c r="A2004" s="2"/>
       <c r="B2004" s="2"/>
     </row>
-    <row r="2005" spans="1:2" ht="12.75">
+    <row r="2005" spans="1:2" ht="13.2">
       <c r="A2005" s="2"/>
       <c r="B2005" s="2"/>
     </row>
-    <row r="2006" spans="1:2" ht="12.75">
+    <row r="2006" spans="1:2" ht="13.2">
       <c r="A2006" s="2"/>
       <c r="B2006" s="2"/>
     </row>
-    <row r="2007" spans="1:2" ht="12.75">
+    <row r="2007" spans="1:2" ht="13.2">
       <c r="A2007" s="2"/>
       <c r="B2007" s="2"/>
     </row>
-    <row r="2008" spans="1:2" ht="12.75">
+    <row r="2008" spans="1:2" ht="13.2">
       <c r="A2008" s="2"/>
       <c r="B2008" s="2"/>
     </row>
-    <row r="2009" spans="1:2" ht="12.75">
+    <row r="2009" spans="1:2" ht="13.2">
       <c r="A2009" s="2"/>
       <c r="B2009" s="2"/>
     </row>
-    <row r="2010" spans="1:2" ht="12.75">
+    <row r="2010" spans="1:2" ht="13.2">
       <c r="A2010" s="2"/>
       <c r="B2010" s="2"/>
     </row>
-    <row r="2011" spans="1:2" ht="12.75">
+    <row r="2011" spans="1:2" ht="13.2">
       <c r="A2011" s="2"/>
       <c r="B2011" s="2"/>
     </row>
-    <row r="2012" spans="1:2" ht="12.75">
+    <row r="2012" spans="1:2" ht="13.2">
       <c r="A2012" s="2"/>
       <c r="B2012" s="2"/>
     </row>
-    <row r="2013" spans="1:2" ht="12.75">
+    <row r="2013" spans="1:2" ht="13.2">
       <c r="A2013" s="2"/>
       <c r="B2013" s="2"/>
     </row>
-    <row r="2014" spans="1:2" ht="12.75">
+    <row r="2014" spans="1:2" ht="13.2">
       <c r="A2014" s="2"/>
       <c r="B2014" s="2"/>
     </row>
-    <row r="2015" spans="1:2" ht="12.75">
+    <row r="2015" spans="1:2" ht="13.2">
       <c r="A2015" s="2"/>
       <c r="B2015" s="2"/>
     </row>
-    <row r="2016" spans="1:2" ht="12.75">
+    <row r="2016" spans="1:2" ht="13.2">
       <c r="A2016" s="2"/>
       <c r="B2016" s="2"/>
     </row>
-    <row r="2017" spans="1:2" ht="12.75">
+    <row r="2017" spans="1:2" ht="13.2">
       <c r="A2017" s="2"/>
       <c r="B2017" s="2"/>
     </row>
-    <row r="2018" spans="1:2" ht="12.75">
+    <row r="2018" spans="1:2" ht="13.2">
       <c r="A2018" s="2"/>
       <c r="B2018" s="2"/>
     </row>
-    <row r="2019" spans="1:2" ht="12.75">
+    <row r="2019" spans="1:2" ht="13.2">
       <c r="A2019" s="2"/>
       <c r="B2019" s="2"/>
     </row>
-    <row r="2020" spans="1:2" ht="12.75">
+    <row r="2020" spans="1:2" ht="13.2">
       <c r="A2020" s="2"/>
       <c r="B2020" s="2"/>
     </row>
-    <row r="2021" spans="1:2" ht="12.75">
+    <row r="2021" spans="1:2" ht="13.2">
       <c r="A2021" s="2"/>
       <c r="B2021" s="2"/>
     </row>
-    <row r="2022" spans="1:2" ht="12.75">
+    <row r="2022" spans="1:2" ht="13.2">
       <c r="A2022" s="2"/>
       <c r="B2022" s="2"/>
     </row>
-    <row r="2023" spans="1:2" ht="12.75">
+    <row r="2023" spans="1:2" ht="13.2">
       <c r="A2023" s="2"/>
       <c r="B2023" s="2"/>
     </row>
-    <row r="2024" spans="1:2" ht="12.75">
+    <row r="2024" spans="1:2" ht="13.2">
       <c r="A2024" s="2"/>
       <c r="B2024" s="2"/>
     </row>
-    <row r="2025" spans="1:2" ht="12.75">
+    <row r="2025" spans="1:2" ht="13.2">
       <c r="A2025" s="2"/>
       <c r="B2025" s="2"/>
     </row>
-    <row r="2026" spans="1:2" ht="12.75">
+    <row r="2026" spans="1:2" ht="13.2">
       <c r="A2026" s="2"/>
       <c r="B2026" s="2"/>
     </row>
-    <row r="2027" spans="1:2" ht="12.75">
+    <row r="2027" spans="1:2" ht="13.2">
       <c r="A2027" s="2"/>
       <c r="B2027" s="2"/>
     </row>
-    <row r="2028" spans="1:2" ht="12.75">
+    <row r="2028" spans="1:2" ht="13.2">
       <c r="A2028" s="2"/>
       <c r="B2028" s="2"/>
     </row>
-    <row r="2029" spans="1:2" ht="12.75">
+    <row r="2029" spans="1:2" ht="13.2">
       <c r="A2029" s="2"/>
       <c r="B2029" s="2"/>
     </row>
-    <row r="2030" spans="1:2" ht="12.75">
+    <row r="2030" spans="1:2" ht="13.2">
       <c r="A2030" s="2"/>
       <c r="B2030" s="2"/>
     </row>
-    <row r="2031" spans="1:2" ht="12.75">
+    <row r="2031" spans="1:2" ht="13.2">
       <c r="A2031" s="2"/>
       <c r="B2031" s="2"/>
     </row>
-    <row r="2032" spans="1:2" ht="12.75">
+    <row r="2032" spans="1:2" ht="13.2">
       <c r="A2032" s="2"/>
       <c r="B2032" s="2"/>
     </row>
-    <row r="2033" spans="1:2" ht="12.75">
+    <row r="2033" spans="1:2" ht="13.2">
       <c r="A2033" s="2"/>
       <c r="B2033" s="2"/>
     </row>
-    <row r="2034" spans="1:2" ht="12.75">
+    <row r="2034" spans="1:2" ht="13.2">
       <c r="A2034" s="2"/>
       <c r="B2034" s="2"/>
     </row>
-    <row r="2035" spans="1:2" ht="12.75">
+    <row r="2035" spans="1:2" ht="13.2">
       <c r="A2035" s="2"/>
       <c r="B2035" s="2"/>
     </row>
-    <row r="2036" spans="1:2" ht="12.75">
+    <row r="2036" spans="1:2" ht="13.2">
       <c r="A2036" s="2"/>
       <c r="B2036" s="2"/>
     </row>
-    <row r="2037" spans="1:2" ht="12.75">
+    <row r="2037" spans="1:2" ht="13.2">
       <c r="A2037" s="2"/>
       <c r="B2037" s="2"/>
     </row>
-    <row r="2038" spans="1:2" ht="12.75">
+    <row r="2038" spans="1:2" ht="13.2">
       <c r="A2038" s="2"/>
       <c r="B2038" s="2"/>
     </row>
-    <row r="2039" spans="1:2" ht="12.75">
+    <row r="2039" spans="1:2" ht="13.2">
       <c r="A2039" s="2"/>
       <c r="B2039" s="2"/>
     </row>
-    <row r="2040" spans="1:2" ht="12.75">
+    <row r="2040" spans="1:2" ht="13.2">
       <c r="A2040" s="2"/>
       <c r="B2040" s="2"/>
     </row>
-    <row r="2041" spans="1:2" ht="12.75">
+    <row r="2041" spans="1:2" ht="13.2">
       <c r="A2041" s="2"/>
       <c r="B2041" s="2"/>
     </row>
-    <row r="2042" spans="1:2" ht="12.75">
+    <row r="2042" spans="1:2" ht="13.2">
       <c r="A2042" s="2"/>
       <c r="B2042" s="2"/>
     </row>
-    <row r="2043" spans="1:2" ht="12.75">
+    <row r="2043" spans="1:2" ht="13.2">
       <c r="A2043" s="2"/>
       <c r="B2043" s="2"/>
     </row>
-    <row r="2044" spans="1:2" ht="12.75">
+    <row r="2044" spans="1:2" ht="13.2">
       <c r="A2044" s="2"/>
       <c r="B2044" s="2"/>
     </row>
-    <row r="2045" spans="1:2" ht="12.75">
+    <row r="2045" spans="1:2" ht="13.2">
       <c r="A2045" s="2"/>
       <c r="B2045" s="2"/>
     </row>
-    <row r="2046" spans="1:2" ht="12.75">
+    <row r="2046" spans="1:2" ht="13.2">
       <c r="A2046" s="2"/>
       <c r="B2046" s="2"/>
     </row>
-    <row r="2047" spans="1:2" ht="12.75">
+    <row r="2047" spans="1:2" ht="13.2">
       <c r="A2047" s="2"/>
       <c r="B2047" s="2"/>
     </row>
-    <row r="2048" spans="1:2" ht="12.75">
+    <row r="2048" spans="1:2" ht="13.2">
       <c r="A2048" s="2"/>
       <c r="B2048" s="2"/>
     </row>
-    <row r="2049" spans="1:2" ht="12.75">
+    <row r="2049" spans="1:2" ht="13.2">
       <c r="A2049" s="2"/>
       <c r="B2049" s="2"/>
     </row>
-    <row r="2050" spans="1:2" ht="12.75">
+    <row r="2050" spans="1:2" ht="13.2">
       <c r="A2050" s="2"/>
       <c r="B2050" s="2"/>
     </row>
-    <row r="2051" spans="1:2" ht="12.75">
+    <row r="2051" spans="1:2" ht="13.2">
       <c r="A2051" s="2"/>
       <c r="B2051" s="2"/>
     </row>
-    <row r="2052" spans="1:2" ht="12.75">
+    <row r="2052" spans="1:2" ht="13.2">
       <c r="A2052" s="2"/>
       <c r="B2052" s="2"/>
     </row>
-    <row r="2053" spans="1:2" ht="12.75">
+    <row r="2053" spans="1:2" ht="13.2">
       <c r="A2053" s="2"/>
       <c r="B2053" s="2"/>
     </row>
-    <row r="2054" spans="1:2" ht="12.75">
+    <row r="2054" spans="1:2" ht="13.2">
       <c r="A2054" s="2"/>
       <c r="B2054" s="2"/>
     </row>
-    <row r="2055" spans="1:2" ht="12.75">
+    <row r="2055" spans="1:2" ht="13.2">
       <c r="A2055" s="2"/>
       <c r="B2055" s="2"/>
     </row>
-    <row r="2056" spans="1:2" ht="12.75">
+    <row r="2056" spans="1:2" ht="13.2">
       <c r="A2056" s="2"/>
       <c r="B2056" s="2"/>
     </row>
-    <row r="2057" spans="1:2" ht="12.75">
+    <row r="2057" spans="1:2" ht="13.2">
       <c r="A2057" s="2"/>
       <c r="B2057" s="2"/>
     </row>
-    <row r="2058" spans="1:2" ht="12.75">
+    <row r="2058" spans="1:2" ht="13.2">
       <c r="A2058" s="2"/>
       <c r="B2058" s="2"/>
     </row>
-    <row r="2059" spans="1:2" ht="12.75">
+    <row r="2059" spans="1:2" ht="13.2">
       <c r="A2059" s="2"/>
       <c r="B2059" s="2"/>
     </row>
-    <row r="2060" spans="1:2" ht="12.75">
+    <row r="2060" spans="1:2" ht="13.2">
       <c r="A2060" s="2"/>
       <c r="B2060" s="2"/>
     </row>
-    <row r="2061" spans="1:2" ht="12.75">
+    <row r="2061" spans="1:2" ht="13.2">
       <c r="A2061" s="2"/>
       <c r="B2061" s="2"/>
     </row>
-    <row r="2062" spans="1:2" ht="12.75">
+    <row r="2062" spans="1:2" ht="13.2">
       <c r="A2062" s="2"/>
       <c r="B2062" s="2"/>
     </row>
-    <row r="2063" spans="1:2" ht="12.75">
+    <row r="2063" spans="1:2" ht="13.2">
       <c r="A2063" s="2"/>
       <c r="B2063" s="2"/>
     </row>
-    <row r="2064" spans="1:2" ht="12.75">
+    <row r="2064" spans="1:2" ht="13.2">
       <c r="A2064" s="2"/>
       <c r="B2064" s="2"/>
     </row>
-    <row r="2065" spans="1:2" ht="12.75">
+    <row r="2065" spans="1:2" ht="13.2">
       <c r="A2065" s="2"/>
       <c r="B2065" s="2"/>
     </row>
-    <row r="2066" spans="1:2" ht="12.75">
+    <row r="2066" spans="1:2" ht="13.2">
       <c r="A2066" s="2"/>
       <c r="B2066" s="2"/>
     </row>
-    <row r="2067" spans="1:2" ht="12.75">
+    <row r="2067" spans="1:2" ht="13.2">
       <c r="A2067" s="2"/>
       <c r="B2067" s="2"/>
     </row>
-    <row r="2068" spans="1:2" ht="12.75">
+    <row r="2068" spans="1:2" ht="13.2">
       <c r="A2068" s="2"/>
       <c r="B2068" s="2"/>
     </row>
-    <row r="2069" spans="1:2" ht="12.75">
+    <row r="2069" spans="1:2" ht="13.2">
       <c r="A2069" s="2"/>
       <c r="B2069" s="2"/>
     </row>
-    <row r="2070" spans="1:2" ht="12.75">
+    <row r="2070" spans="1:2" ht="13.2">
       <c r="A2070" s="2"/>
       <c r="B2070" s="2"/>
     </row>
-    <row r="2071" spans="1:2" ht="12.75">
+    <row r="2071" spans="1:2" ht="13.2">
       <c r="A2071" s="2"/>
       <c r="B2071" s="2"/>
     </row>
-    <row r="2072" spans="1:2" ht="12.75">
+    <row r="2072" spans="1:2" ht="13.2">
       <c r="A2072" s="2"/>
       <c r="B2072" s="2"/>
     </row>
-    <row r="2073" spans="1:2" ht="12.75">
+    <row r="2073" spans="1:2" ht="13.2">
       <c r="A2073" s="2"/>
       <c r="B2073" s="2"/>
     </row>
-    <row r="2074" spans="1:2" ht="12.75">
+    <row r="2074" spans="1:2" ht="13.2">
       <c r="A2074" s="2"/>
       <c r="B2074" s="2"/>
     </row>
-    <row r="2075" spans="1:2" ht="12.75">
+    <row r="2075" spans="1:2" ht="13.2">
       <c r="A2075" s="2"/>
       <c r="B2075" s="2"/>
     </row>
-    <row r="2076" spans="1:2" ht="12.75">
+    <row r="2076" spans="1:2" ht="13.2">
       <c r="A2076" s="2"/>
       <c r="B2076" s="2"/>
     </row>
-    <row r="2077" spans="1:2" ht="12.75">
+    <row r="2077" spans="1:2" ht="13.2">
       <c r="A2077" s="2"/>
       <c r="B2077" s="2"/>
     </row>
-    <row r="2078" spans="1:2" ht="12.75">
+    <row r="2078" spans="1:2" ht="13.2">
       <c r="A2078" s="2"/>
       <c r="B2078" s="2"/>
     </row>
-    <row r="2079" spans="1:2" ht="12.75">
+    <row r="2079" spans="1:2" ht="13.2">
       <c r="A2079" s="2"/>
       <c r="B2079" s="2"/>
     </row>
-    <row r="2080" spans="1:2" ht="12.75">
+    <row r="2080" spans="1:2" ht="13.2">
       <c r="A2080" s="2"/>
       <c r="B2080" s="2"/>
     </row>
-    <row r="2081" spans="1:2" ht="12.75">
+    <row r="2081" spans="1:2" ht="13.2">
       <c r="A2081" s="2"/>
       <c r="B2081" s="2"/>
     </row>
-    <row r="2082" spans="1:2" ht="12.75">
+    <row r="2082" spans="1:2" ht="13.2">
       <c r="A2082" s="2"/>
       <c r="B2082" s="2"/>
     </row>
-    <row r="2083" spans="1:2" ht="12.75">
+    <row r="2083" spans="1:2" ht="13.2">
       <c r="A2083" s="2"/>
       <c r="B2083" s="2"/>
     </row>
-    <row r="2084" spans="1:2" ht="12.75">
+    <row r="2084" spans="1:2" ht="13.2">
       <c r="A2084" s="2"/>
       <c r="B2084" s="2"/>
     </row>
-    <row r="2085" spans="1:2" ht="12.75">
+    <row r="2085" spans="1:2" ht="13.2">
       <c r="A2085" s="2"/>
       <c r="B2085" s="2"/>
     </row>
-    <row r="2086" spans="1:2" ht="12.75">
+    <row r="2086" spans="1:2" ht="13.2">
       <c r="A2086" s="2"/>
       <c r="B2086" s="2"/>
     </row>
-    <row r="2087" spans="1:2" ht="12.75">
+    <row r="2087" spans="1:2" ht="13.2">
       <c r="A2087" s="2"/>
       <c r="B2087" s="2"/>
     </row>
-    <row r="2088" spans="1:2" ht="12.75">
+    <row r="2088" spans="1:2" ht="13.2">
       <c r="A2088" s="2"/>
       <c r="B2088" s="2"/>
     </row>
-    <row r="2089" spans="1:2" ht="12.75">
+    <row r="2089" spans="1:2" ht="13.2">
       <c r="A2089" s="2"/>
       <c r="B2089" s="2"/>
     </row>
-    <row r="2090" spans="1:2" ht="12.75">
+    <row r="2090" spans="1:2" ht="13.2">
       <c r="A2090" s="2"/>
       <c r="B2090" s="2"/>
     </row>
-    <row r="2091" spans="1:2" ht="12.75">
+    <row r="2091" spans="1:2" ht="13.2">
       <c r="A2091" s="2"/>
       <c r="B2091" s="2"/>
     </row>
-    <row r="2092" spans="1:2" ht="12.75">
+    <row r="2092" spans="1:2" ht="13.2">
       <c r="A2092" s="2"/>
       <c r="B2092" s="2"/>
     </row>
-    <row r="2093" spans="1:2" ht="12.75">
+    <row r="2093" spans="1:2" ht="13.2">
       <c r="A2093" s="2"/>
       <c r="B2093" s="2"/>
     </row>
-    <row r="2094" spans="1:2" ht="12.75">
+    <row r="2094" spans="1:2" ht="13.2">
       <c r="A2094" s="2"/>
       <c r="B2094" s="2"/>
     </row>
-    <row r="2095" spans="1:2" ht="12.75">
+    <row r="2095" spans="1:2" ht="13.2">
       <c r="A2095" s="2"/>
       <c r="B2095" s="2"/>
     </row>
-    <row r="2096" spans="1:2" ht="12.75">
+    <row r="2096" spans="1:2" ht="13.2">
       <c r="A2096" s="2"/>
       <c r="B2096" s="2"/>
     </row>
-    <row r="2097" spans="1:2" ht="12.75">
+    <row r="2097" spans="1:2" ht="13.2">
       <c r="A2097" s="2"/>
       <c r="B2097" s="2"/>
     </row>
-    <row r="2098" spans="1:2" ht="12.75">
+    <row r="2098" spans="1:2" ht="13.2">
       <c r="A2098" s="2"/>
       <c r="B2098" s="2"/>
     </row>
-    <row r="2099" spans="1:2" ht="12.75">
+    <row r="2099" spans="1:2" ht="13.2">
       <c r="A2099" s="2"/>
       <c r="B2099" s="2"/>
     </row>
-    <row r="2100" spans="1:2" ht="12.75">
+    <row r="2100" spans="1:2" ht="13.2">
       <c r="A2100" s="2"/>
       <c r="B2100" s="2"/>
     </row>
-    <row r="2101" spans="1:2" ht="12.75">
+    <row r="2101" spans="1:2" ht="13.2">
       <c r="A2101" s="2"/>
       <c r="B2101" s="2"/>
     </row>
-    <row r="2102" spans="1:2" ht="12.75">
+    <row r="2102" spans="1:2" ht="13.2">
       <c r="A2102" s="2"/>
       <c r="B2102" s="2"/>
     </row>
-    <row r="2103" spans="1:2" ht="12.75">
+    <row r="2103" spans="1:2" ht="13.2">
       <c r="A2103" s="2"/>
       <c r="B2103" s="2"/>
     </row>
-    <row r="2104" spans="1:2" ht="12.75">
+    <row r="2104" spans="1:2" ht="13.2">
       <c r="A2104" s="2"/>
       <c r="B2104" s="2"/>
     </row>
-    <row r="2105" spans="1:2" ht="12.75">
+    <row r="2105" spans="1:2" ht="13.2">
       <c r="A2105" s="2"/>
       <c r="B2105" s="2"/>
     </row>
-    <row r="2106" spans="1:2" ht="12.75">
+    <row r="2106" spans="1:2" ht="13.2">
       <c r="A2106" s="2"/>
       <c r="B2106" s="2"/>
     </row>
-    <row r="2107" spans="1:2" ht="12.75">
+    <row r="2107" spans="1:2" ht="13.2">
       <c r="A2107" s="2"/>
       <c r="B2107" s="2"/>
     </row>
-    <row r="2108" spans="1:2" ht="12.75">
+    <row r="2108" spans="1:2" ht="13.2">
       <c r="A2108" s="2"/>
       <c r="B2108" s="2"/>
     </row>
-    <row r="2109" spans="1:2" ht="12.75">
+    <row r="2109" spans="1:2" ht="13.2">
       <c r="A2109" s="2"/>
       <c r="B2109" s="2"/>
     </row>
-    <row r="2110" spans="1:2" ht="12.75">
+    <row r="2110" spans="1:2" ht="13.2">
       <c r="A2110" s="2"/>
       <c r="B2110" s="2"/>
     </row>
-    <row r="2111" spans="1:2" ht="12.75">
+    <row r="2111" spans="1:2" ht="13.2">
       <c r="A2111" s="2"/>
       <c r="B2111" s="2"/>
     </row>
-    <row r="2112" spans="1:2" ht="12.75">
+    <row r="2112" spans="1:2" ht="13.2">
       <c r="A2112" s="2"/>
       <c r="B2112" s="2"/>
     </row>
-    <row r="2113" spans="1:2" ht="12.75">
+    <row r="2113" spans="1:2" ht="13.2">
       <c r="A2113" s="2"/>
       <c r="B2113" s="2"/>
     </row>
-    <row r="2114" spans="1:2" ht="12.75">
+    <row r="2114" spans="1:2" ht="13.2">
       <c r="A2114" s="2"/>
       <c r="B2114" s="2"/>
     </row>
-    <row r="2115" spans="1:2" ht="12.75">
+    <row r="2115" spans="1:2" ht="13.2">
       <c r="A2115" s="2"/>
       <c r="B2115" s="2"/>
     </row>
-    <row r="2116" spans="1:2" ht="12.75">
+    <row r="2116" spans="1:2" ht="13.2">
       <c r="A2116" s="2"/>
       <c r="B2116" s="2"/>
     </row>
-    <row r="2117" spans="1:2" ht="12.75">
+    <row r="2117" spans="1:2" ht="13.2">
       <c r="A2117" s="2"/>
       <c r="B2117" s="2"/>
     </row>
-    <row r="2118" spans="1:2" ht="12.75">
+    <row r="2118" spans="1:2" ht="13.2">
       <c r="A2118" s="2"/>
       <c r="B2118" s="2"/>
     </row>
-    <row r="2119" spans="1:2" ht="12.75">
+    <row r="2119" spans="1:2" ht="13.2">
       <c r="A2119" s="2"/>
       <c r="B2119" s="2"/>
     </row>
-    <row r="2120" spans="1:2" ht="12.75">
+    <row r="2120" spans="1:2" ht="13.2">
       <c r="A2120" s="2"/>
       <c r="B2120" s="2"/>
     </row>
-    <row r="2121" spans="1:2" ht="12.75">
+    <row r="2121" spans="1:2" ht="13.2">
       <c r="A2121" s="2"/>
       <c r="B2121" s="2"/>
     </row>
-    <row r="2122" spans="1:2" ht="12.75">
+    <row r="2122" spans="1:2" ht="13.2">
       <c r="A2122" s="2"/>
       <c r="B2122" s="2"/>
     </row>
-    <row r="2123" spans="1:2" ht="12.75">
+    <row r="2123" spans="1:2" ht="13.2">
       <c r="A2123" s="2"/>
       <c r="B2123" s="2"/>
     </row>
-    <row r="2124" spans="1:2" ht="12.75">
+    <row r="2124" spans="1:2" ht="13.2">
       <c r="A2124" s="2"/>
       <c r="B2124" s="2"/>
     </row>
-    <row r="2125" spans="1:2" ht="12.75">
+    <row r="2125" spans="1:2" ht="13.2">
       <c r="A2125" s="2"/>
       <c r="B2125" s="2"/>
     </row>
-    <row r="2126" spans="1:2" ht="12.75">
+    <row r="2126" spans="1:2" ht="13.2">
       <c r="A2126" s="2"/>
       <c r="B2126" s="2"/>
     </row>
-    <row r="2127" spans="1:2" ht="12.75">
+    <row r="2127" spans="1:2" ht="13.2">
       <c r="A2127" s="2"/>
       <c r="B2127" s="2"/>
     </row>
-    <row r="2128" spans="1:2" ht="12.75">
+    <row r="2128" spans="1:2" ht="13.2">
       <c r="A2128" s="2"/>
       <c r="B2128" s="2"/>
     </row>
-    <row r="2129" spans="1:2" ht="12.75">
+    <row r="2129" spans="1:2" ht="13.2">
       <c r="A2129" s="2"/>
       <c r="B2129" s="2"/>
     </row>
-    <row r="2130" spans="1:2" ht="12.75">
+    <row r="2130" spans="1:2" ht="13.2">
       <c r="A2130" s="2"/>
       <c r="B2130" s="2"/>
     </row>
-    <row r="2131" spans="1:2" ht="12.75">
+    <row r="2131" spans="1:2" ht="13.2">
       <c r="A2131" s="2"/>
       <c r="B2131" s="2"/>
     </row>
-    <row r="2132" spans="1:2" ht="12.75">
+    <row r="2132" spans="1:2" ht="13.2">
       <c r="A2132" s="2"/>
       <c r="B2132" s="2"/>
     </row>
-    <row r="2133" spans="1:2" ht="12.75">
+    <row r="2133" spans="1:2" ht="13.2">
       <c r="A2133" s="2"/>
       <c r="B2133" s="2"/>
     </row>
-    <row r="2134" spans="1:2" ht="12.75">
+    <row r="2134" spans="1:2" ht="13.2">
       <c r="A2134" s="2"/>
       <c r="B2134" s="2"/>
     </row>
-    <row r="2135" spans="1:2" ht="12.75">
+    <row r="2135" spans="1:2" ht="13.2">
       <c r="A2135" s="2"/>
       <c r="B2135" s="2"/>
     </row>
-    <row r="2136" spans="1:2" ht="12.75">
+    <row r="2136" spans="1:2" ht="13.2">
       <c r="A2136" s="2"/>
       <c r="B2136" s="2"/>
     </row>
-    <row r="2137" spans="1:2" ht="12.75">
+    <row r="2137" spans="1:2" ht="13.2">
       <c r="A2137" s="2"/>
       <c r="B2137" s="2"/>
     </row>
-    <row r="2138" spans="1:2" ht="12.75">
+    <row r="2138" spans="1:2" ht="13.2">
       <c r="A2138" s="2"/>
       <c r="B2138" s="2"/>
     </row>
-    <row r="2139" spans="1:2" ht="12.75">
+    <row r="2139" spans="1:2" ht="13.2">
       <c r="A2139" s="2"/>
       <c r="B2139" s="2"/>
     </row>
-    <row r="2140" spans="1:2" ht="12.75">
+    <row r="2140" spans="1:2" ht="13.2">
       <c r="A2140" s="2"/>
       <c r="B2140" s="2"/>
     </row>
-    <row r="2141" spans="1:2" ht="12.75">
+    <row r="2141" spans="1:2" ht="13.2">
       <c r="A2141" s="2"/>
       <c r="B2141" s="2"/>
     </row>
-    <row r="2142" spans="1:2" ht="12.75">
+    <row r="2142" spans="1:2" ht="13.2">
       <c r="A2142" s="2"/>
       <c r="B2142" s="2"/>
     </row>
-    <row r="2143" spans="1:2" ht="12.75">
+    <row r="2143" spans="1:2" ht="13.2">
       <c r="A2143" s="2"/>
       <c r="B2143" s="2"/>
     </row>
-    <row r="2144" spans="1:2" ht="12.75">
+    <row r="2144" spans="1:2" ht="13.2">
       <c r="A2144" s="2"/>
       <c r="B2144" s="2"/>
     </row>
-    <row r="2145" spans="1:2" ht="12.75">
+    <row r="2145" spans="1:2" ht="13.2">
       <c r="A2145" s="2"/>
       <c r="B2145" s="2"/>
     </row>
-    <row r="2146" spans="1:2" ht="12.75">
+    <row r="2146" spans="1:2" ht="13.2">
       <c r="A2146" s="2"/>
       <c r="B2146" s="2"/>
     </row>
-    <row r="2147" spans="1:2" ht="12.75">
+    <row r="2147" spans="1:2" ht="13.2">
       <c r="A2147" s="2"/>
       <c r="B2147" s="2"/>
     </row>
-    <row r="2148" spans="1:2" ht="12.75">
+    <row r="2148" spans="1:2" ht="13.2">
       <c r="A2148" s="2"/>
       <c r="B2148" s="2"/>
     </row>
-    <row r="2149" spans="1:2" ht="12.75">
+    <row r="2149" spans="1:2" ht="13.2">
       <c r="A2149" s="2"/>
       <c r="B2149" s="2"/>
     </row>
-    <row r="2150" spans="1:2" ht="12.75">
+    <row r="2150" spans="1:2" ht="13.2">
       <c r="A2150" s="2"/>
       <c r="B2150" s="2"/>
     </row>
-    <row r="2151" spans="1:2" ht="12.75">
+    <row r="2151" spans="1:2" ht="13.2">
       <c r="A2151" s="2"/>
       <c r="B2151" s="2"/>
     </row>
-    <row r="2152" spans="1:2" ht="12.75">
+    <row r="2152" spans="1:2" ht="13.2">
       <c r="A2152" s="2"/>
       <c r="B2152" s="2"/>
     </row>
-    <row r="2153" spans="1:2" ht="12.75">
+    <row r="2153" spans="1:2" ht="13.2">
       <c r="A2153" s="2"/>
       <c r="B2153" s="2"/>
     </row>
-    <row r="2154" spans="1:2" ht="12.75">
+    <row r="2154" spans="1:2" ht="13.2">
       <c r="A2154" s="2"/>
       <c r="B2154" s="2"/>
     </row>
-    <row r="2155" spans="1:2" ht="12.75">
+    <row r="2155" spans="1:2" ht="13.2">
       <c r="A2155" s="2"/>
       <c r="B2155" s="2"/>
     </row>
-    <row r="2156" spans="1:2" ht="12.75">
+    <row r="2156" spans="1:2" ht="13.2">
       <c r="A2156" s="2"/>
       <c r="B2156" s="2"/>
     </row>
-    <row r="2157" spans="1:2" ht="12.75">
+    <row r="2157" spans="1:2" ht="13.2">
       <c r="A2157" s="2"/>
       <c r="B2157" s="2"/>
     </row>
-    <row r="2158" spans="1:2" ht="12.75">
+    <row r="2158" spans="1:2" ht="13.2">
       <c r="A2158" s="2"/>
       <c r="B2158" s="2"/>
     </row>
-    <row r="2159" spans="1:2" ht="12.75">
+    <row r="2159" spans="1:2" ht="13.2">
       <c r="A2159" s="2"/>
       <c r="B2159" s="2"/>
     </row>
-    <row r="2160" spans="1:2" ht="12.75">
+    <row r="2160" spans="1:2" ht="13.2">
       <c r="A2160" s="2"/>
       <c r="B2160" s="2"/>
     </row>
-    <row r="2161" spans="1:2" ht="12.75">
+    <row r="2161" spans="1:2" ht="13.2">
       <c r="A2161" s="2"/>
       <c r="B2161" s="2"/>
     </row>
-    <row r="2162" spans="1:2" ht="12.75">
+    <row r="2162" spans="1:2" ht="13.2">
       <c r="A2162" s="2"/>
       <c r="B2162" s="2"/>
     </row>
-    <row r="2163" spans="1:2" ht="12.75">
+    <row r="2163" spans="1:2" ht="13.2">
       <c r="A2163" s="2"/>
       <c r="B2163" s="2"/>
     </row>
-    <row r="2164" spans="1:2" ht="12.75">
+    <row r="2164" spans="1:2" ht="13.2">
       <c r="A2164" s="2"/>
       <c r="B2164" s="2"/>
     </row>
-    <row r="2165" spans="1:2" ht="12.75">
+    <row r="2165" spans="1:2" ht="13.2">
       <c r="A2165" s="2"/>
       <c r="B2165" s="2"/>
     </row>
-    <row r="2166" spans="1:2" ht="12.75">
+    <row r="2166" spans="1:2" ht="13.2">
       <c r="A2166" s="2"/>
       <c r="B2166" s="2"/>
     </row>
-    <row r="2167" spans="1:2" ht="12.75">
+    <row r="2167" spans="1:2" ht="13.2">
       <c r="A2167" s="2"/>
       <c r="B2167" s="2"/>
     </row>
-    <row r="2168" spans="1:2" ht="12.75">
+    <row r="2168" spans="1:2" ht="13.2">
       <c r="A2168" s="2"/>
       <c r="B2168" s="2"/>
     </row>
-    <row r="2169" spans="1:2" ht="12.75">
+    <row r="2169" spans="1:2" ht="13.2">
       <c r="A2169" s="2"/>
       <c r="B2169" s="2"/>
     </row>
-    <row r="2170" spans="1:2" ht="12.75">
+    <row r="2170" spans="1:2" ht="13.2">
       <c r="A2170" s="2"/>
       <c r="B2170" s="2"/>
     </row>
-    <row r="2171" spans="1:2" ht="12.75">
+    <row r="2171" spans="1:2" ht="13.2">
       <c r="A2171" s="2"/>
       <c r="B2171" s="2"/>
     </row>
-    <row r="2172" spans="1:2" ht="12.75">
+    <row r="2172" spans="1:2" ht="13.2">
       <c r="A2172" s="2"/>
       <c r="B2172" s="2"/>
     </row>
-    <row r="2173" spans="1:2" ht="12.75">
+    <row r="2173" spans="1:2" ht="13.2">
       <c r="A2173" s="2"/>
       <c r="B2173" s="2"/>
     </row>
-    <row r="2174" spans="1:2" ht="12.75">
+    <row r="2174" spans="1:2" ht="13.2">
       <c r="A2174" s="2"/>
       <c r="B2174" s="2"/>
     </row>
-    <row r="2175" spans="1:2" ht="12.75">
+    <row r="2175" spans="1:2" ht="13.2">
       <c r="A2175" s="2"/>
       <c r="B2175" s="2"/>
     </row>
-    <row r="2176" spans="1:2" ht="12.75">
+    <row r="2176" spans="1:2" ht="13.2">
       <c r="A2176" s="2"/>
       <c r="B2176" s="2"/>
     </row>
-    <row r="2177" spans="1:2" ht="12.75">
+    <row r="2177" spans="1:2" ht="13.2">
       <c r="A2177" s="2"/>
       <c r="B2177" s="2"/>
     </row>
-    <row r="2178" spans="1:2" ht="12.75">
+    <row r="2178" spans="1:2" ht="13.2">
       <c r="A2178" s="2"/>
       <c r="B2178" s="2"/>
     </row>
-    <row r="2179" spans="1:2" ht="12.75">
+    <row r="2179" spans="1:2" ht="13.2">
       <c r="A2179" s="2"/>
       <c r="B2179" s="2"/>
     </row>
-    <row r="2180" spans="1:2" ht="12.75">
+    <row r="2180" spans="1:2" ht="13.2">
       <c r="A2180" s="2"/>
       <c r="B2180" s="2"/>
     </row>
-    <row r="2181" spans="1:2" ht="12.75">
+    <row r="2181" spans="1:2" ht="13.2">
       <c r="A2181" s="2"/>
       <c r="B2181" s="2"/>
     </row>
-    <row r="2182" spans="1:2" ht="12.75">
+    <row r="2182" spans="1:2" ht="13.2">
       <c r="A2182" s="2"/>
       <c r="B2182" s="2"/>
     </row>
-    <row r="2183" spans="1:2" ht="12.75">
+    <row r="2183" spans="1:2" ht="13.2">
       <c r="A2183" s="2"/>
       <c r="B2183" s="2"/>
     </row>
-    <row r="2184" spans="1:2" ht="12.75">
+    <row r="2184" spans="1:2" ht="13.2">
       <c r="A2184" s="2"/>
       <c r="B2184" s="2"/>
     </row>
-    <row r="2185" spans="1:2" ht="12.75">
+    <row r="2185" spans="1:2" ht="13.2">
       <c r="A2185" s="2"/>
       <c r="B2185" s="2"/>
     </row>
-    <row r="2186" spans="1:2" ht="12.75">
+    <row r="2186" spans="1:2" ht="13.2">
       <c r="A2186" s="2"/>
       <c r="B2186" s="2"/>
     </row>
-    <row r="2187" spans="1:2" ht="12.75">
+    <row r="2187" spans="1:2" ht="13.2">
       <c r="A2187" s="2"/>
       <c r="B2187" s="2"/>
     </row>
-    <row r="2188" spans="1:2" ht="12.75">
+    <row r="2188" spans="1:2" ht="13.2">
       <c r="A2188" s="2"/>
       <c r="B2188" s="2"/>
     </row>
-    <row r="2189" spans="1:2" ht="12.75">
+    <row r="2189" spans="1:2" ht="13.2">
       <c r="A2189" s="2"/>
       <c r="B2189" s="2"/>
     </row>
-    <row r="2190" spans="1:2" ht="12.75">
+    <row r="2190" spans="1:2" ht="13.2">
       <c r="A2190" s="2"/>
       <c r="B2190" s="2"/>
     </row>
-    <row r="2191" spans="1:2" ht="12.75">
+    <row r="2191" spans="1:2" ht="13.2">
       <c r="A2191" s="2"/>
       <c r="B2191" s="2"/>
     </row>
-    <row r="2192" spans="1:2" ht="12.75">
+    <row r="2192" spans="1:2" ht="13.2">
       <c r="A2192" s="2"/>
       <c r="B2192" s="2"/>
     </row>
-    <row r="2193" spans="1:2" ht="12.75">
+    <row r="2193" spans="1:2" ht="13.2">
       <c r="A2193" s="2"/>
       <c r="B2193" s="2"/>
     </row>
-    <row r="2194" spans="1:2" ht="12.75">
+    <row r="2194" spans="1:2" ht="13.2">
       <c r="A2194" s="2"/>
       <c r="B2194" s="2"/>
     </row>
-    <row r="2195" spans="1:2" ht="12.75">
+    <row r="2195" spans="1:2" ht="13.2">
       <c r="A2195" s="2"/>
       <c r="B2195" s="2"/>
     </row>
-    <row r="2196" spans="1:2" ht="12.75">
+    <row r="2196" spans="1:2" ht="13.2">
       <c r="A2196" s="2"/>
       <c r="B2196" s="2"/>
     </row>
-    <row r="2197" spans="1:2" ht="12.75">
+    <row r="2197" spans="1:2" ht="13.2">
       <c r="A2197" s="2"/>
       <c r="B2197" s="2"/>
     </row>
-    <row r="2198" spans="1:2" ht="12.75">
+    <row r="2198" spans="1:2" ht="13.2">
       <c r="A2198" s="2"/>
       <c r="B2198" s="2"/>
     </row>
-    <row r="2199" spans="1:2" ht="12.75">
+    <row r="2199" spans="1:2" ht="13.2">
       <c r="A2199" s="2"/>
       <c r="B2199" s="2"/>
     </row>
-    <row r="2200" spans="1:2" ht="12.75">
+    <row r="2200" spans="1:2" ht="13.2">
       <c r="A2200" s="2"/>
       <c r="B2200" s="2"/>
     </row>
-    <row r="2201" spans="1:2" ht="12.75">
+    <row r="2201" spans="1:2" ht="13.2">
       <c r="A2201" s="2"/>
       <c r="B2201" s="2"/>
     </row>
-    <row r="2202" spans="1:2" ht="12.75">
+    <row r="2202" spans="1:2" ht="13.2">
       <c r="A2202" s="2"/>
       <c r="B2202" s="2"/>
     </row>
-    <row r="2203" spans="1:2" ht="12.75">
+    <row r="2203" spans="1:2" ht="13.2">
       <c r="A2203" s="2"/>
       <c r="B2203" s="2"/>
     </row>
-    <row r="2204" spans="1:2" ht="12.75">
+    <row r="2204" spans="1:2" ht="13.2">
       <c r="A2204" s="2"/>
       <c r="B2204" s="2"/>
     </row>
-    <row r="2205" spans="1:2" ht="12.75">
+    <row r="2205" spans="1:2" ht="13.2">
       <c r="A2205" s="2"/>
       <c r="B2205" s="2"/>
     </row>
-    <row r="2206" spans="1:2" ht="12.75">
+    <row r="2206" spans="1:2" ht="13.2">
       <c r="A2206" s="2"/>
       <c r="B2206" s="2"/>
     </row>
-    <row r="2207" spans="1:2" ht="12.75">
+    <row r="2207" spans="1:2" ht="13.2">
       <c r="A2207" s="2"/>
       <c r="B2207" s="2"/>
     </row>
-    <row r="2208" spans="1:2" ht="12.75">
+    <row r="2208" spans="1:2" ht="13.2">
       <c r="A2208" s="2"/>
       <c r="B2208" s="2"/>
     </row>
-    <row r="2209" spans="1:2" ht="12.75">
+    <row r="2209" spans="1:2" ht="13.2">
       <c r="A2209" s="2"/>
       <c r="B2209" s="2"/>
     </row>
-    <row r="2210" spans="1:2" ht="12.75">
+    <row r="2210" spans="1:2" ht="13.2">
       <c r="A2210" s="2"/>
       <c r="B2210" s="2"/>
     </row>
-    <row r="2211" spans="1:2" ht="12.75">
+    <row r="2211" spans="1:2" ht="13.2">
       <c r="A2211" s="2"/>
       <c r="B2211" s="2"/>
     </row>
-    <row r="2212" spans="1:2" ht="12.75">
+    <row r="2212" spans="1:2" ht="13.2">
       <c r="A2212" s="2"/>
       <c r="B2212" s="2"/>
     </row>
-    <row r="2213" spans="1:2" ht="12.75">
+    <row r="2213" spans="1:2" ht="13.2">
       <c r="A2213" s="2"/>
       <c r="B2213" s="2"/>
     </row>
-    <row r="2214" spans="1:2" ht="12.75">
+    <row r="2214" spans="1:2" ht="13.2">
       <c r="A2214" s="2"/>
       <c r="B2214" s="2"/>
     </row>
-    <row r="2215" spans="1:2" ht="12.75">
+    <row r="2215" spans="1:2" ht="13.2">
       <c r="A2215" s="2"/>
       <c r="B2215" s="2"/>
     </row>
-    <row r="2216" spans="1:2" ht="12.75">
+    <row r="2216" spans="1:2" ht="13.2">
       <c r="A2216" s="2"/>
       <c r="B2216" s="2"/>
     </row>
-    <row r="2217" spans="1:2" ht="12.75">
+    <row r="2217" spans="1:2" ht="13.2">
       <c r="A2217" s="2"/>
       <c r="B2217" s="2"/>
     </row>
-    <row r="2218" spans="1:2" ht="12.75">
+    <row r="2218" spans="1:2" ht="13.2">
       <c r="A2218" s="2"/>
       <c r="B2218" s="2"/>
     </row>
-    <row r="2219" spans="1:2" ht="12.75">
+    <row r="2219" spans="1:2" ht="13.2">
       <c r="A2219" s="2"/>
       <c r="B2219" s="2"/>
     </row>
-    <row r="2220" spans="1:2" ht="12.75">
+    <row r="2220" spans="1:2" ht="13.2">
       <c r="A2220" s="2"/>
       <c r="B2220" s="2"/>
     </row>
-    <row r="2221" spans="1:2" ht="12.75">
+    <row r="2221" spans="1:2" ht="13.2">
       <c r="A2221" s="2"/>
       <c r="B2221" s="2"/>
     </row>
-    <row r="2222" spans="1:2" ht="12.75">
+    <row r="2222" spans="1:2" ht="13.2">
       <c r="A2222" s="2"/>
       <c r="B2222" s="2"/>
     </row>
-    <row r="2223" spans="1:2" ht="12.75">
+    <row r="2223" spans="1:2" ht="13.2">
       <c r="A2223" s="2"/>
       <c r="B2223" s="2"/>
     </row>
-    <row r="2224" spans="1:2" ht="12.75">
+    <row r="2224" spans="1:2" ht="13.2">
       <c r="A2224" s="2"/>
       <c r="B2224" s="2"/>
     </row>
-    <row r="2225" spans="1:2" ht="12.75">
+    <row r="2225" spans="1:2" ht="13.2">
       <c r="A2225" s="2"/>
       <c r="B2225" s="2"/>
     </row>
-    <row r="2226" spans="1:2" ht="12.75">
+    <row r="2226" spans="1:2" ht="13.2">
       <c r="A2226" s="2"/>
       <c r="B2226" s="2"/>
     </row>
-    <row r="2227" spans="1:2" ht="12.75">
+    <row r="2227" spans="1:2" ht="13.2">
       <c r="A2227" s="2"/>
       <c r="B2227" s="2"/>
     </row>
-    <row r="2228" spans="1:2" ht="12.75">
+    <row r="2228" spans="1:2" ht="13.2">
       <c r="A2228" s="2"/>
       <c r="B2228" s="2"/>
     </row>
-    <row r="2229" spans="1:2" ht="12.75">
+    <row r="2229" spans="1:2" ht="13.2">
       <c r="A2229" s="2"/>
       <c r="B2229" s="2"/>
     </row>
-    <row r="2230" spans="1:2" ht="12.75">
+    <row r="2230" spans="1:2" ht="13.2">
       <c r="A2230" s="2"/>
       <c r="B2230" s="2"/>
     </row>
-    <row r="2231" spans="1:2" ht="12.75">
+    <row r="2231" spans="1:2" ht="13.2">
       <c r="A2231" s="2"/>
       <c r="B2231" s="2"/>
     </row>
-    <row r="2232" spans="1:2" ht="12.75">
+    <row r="2232" spans="1:2" ht="13.2">
       <c r="A2232" s="2"/>
       <c r="B2232" s="2"/>
     </row>
-    <row r="2233" spans="1:2" ht="12.75">
+    <row r="2233" spans="1:2" ht="13.2">
       <c r="A2233" s="2"/>
       <c r="B2233" s="2"/>
     </row>
-    <row r="2234" spans="1:2" ht="12.75">
+    <row r="2234" spans="1:2" ht="13.2">
       <c r="A2234" s="2"/>
       <c r="B2234" s="2"/>
     </row>
-    <row r="2235" spans="1:2" ht="12.75">
+    <row r="2235" spans="1:2" ht="13.2">
       <c r="A2235" s="2"/>
       <c r="B2235" s="2"/>
     </row>
-    <row r="2236" spans="1:2" ht="12.75">
+    <row r="2236" spans="1:2" ht="13.2">
       <c r="A2236" s="2"/>
       <c r="B2236" s="2"/>
     </row>
-    <row r="2237" spans="1:2" ht="12.75">
+    <row r="2237" spans="1:2" ht="13.2">
       <c r="A2237" s="2"/>
       <c r="B2237" s="2"/>
     </row>
-    <row r="2238" spans="1:2" ht="12.75">
+    <row r="2238" spans="1:2" ht="13.2">
       <c r="A2238" s="2"/>
       <c r="B2238" s="2"/>
     </row>
-    <row r="2239" spans="1:2" ht="12.75">
+    <row r="2239" spans="1:2" ht="13.2">
       <c r="A2239" s="2"/>
       <c r="B2239" s="2"/>
     </row>
-    <row r="2240" spans="1:2" ht="12.75">
+    <row r="2240" spans="1:2" ht="13.2">
       <c r="A2240" s="2"/>
       <c r="B2240" s="2"/>
     </row>
-    <row r="2241" spans="1:2" ht="12.75">
+    <row r="2241" spans="1:2" ht="13.2">
       <c r="A2241" s="2"/>
       <c r="B2241" s="2"/>
     </row>
-    <row r="2242" spans="1:2" ht="12.75">
+    <row r="2242" spans="1:2" ht="13.2">
       <c r="A2242" s="2"/>
       <c r="B2242" s="2"/>
     </row>
-    <row r="2243" spans="1:2" ht="12.75">
+    <row r="2243" spans="1:2" ht="13.2">
       <c r="A2243" s="2"/>
       <c r="B2243" s="2"/>
     </row>
-    <row r="2244" spans="1:2" ht="12.75">
+    <row r="2244" spans="1:2" ht="13.2">
       <c r="A2244" s="2"/>
       <c r="B2244" s="2"/>
     </row>
-    <row r="2245" spans="1:2" ht="12.75">
+    <row r="2245" spans="1:2" ht="13.2">
       <c r="A2245" s="2"/>
       <c r="B2245" s="2"/>
     </row>
-    <row r="2246" spans="1:2" ht="12.75">
+    <row r="2246" spans="1:2" ht="13.2">
       <c r="A2246" s="2"/>
       <c r="B2246" s="2"/>
     </row>
-    <row r="2247" spans="1:2" ht="12.75">
+    <row r="2247" spans="1:2" ht="13.2">
       <c r="A2247" s="2"/>
       <c r="B2247" s="2"/>
     </row>
-    <row r="2248" spans="1:2" ht="12.75">
+    <row r="2248" spans="1:2" ht="13.2">
       <c r="A2248" s="2"/>
       <c r="B2248" s="2"/>
     </row>
-    <row r="2249" spans="1:2" ht="12.75">
+    <row r="2249" spans="1:2" ht="13.2">
       <c r="A2249" s="2"/>
       <c r="B2249" s="2"/>
     </row>
-    <row r="2250" spans="1:2" ht="12.75">
+    <row r="2250" spans="1:2" ht="13.2">
       <c r="A2250" s="2"/>
       <c r="B2250" s="2"/>
     </row>
-    <row r="2251" spans="1:2" ht="12.75">
+    <row r="2251" spans="1:2" ht="13.2">
       <c r="A2251" s="2"/>
       <c r="B2251" s="2"/>
     </row>
-    <row r="2252" spans="1:2" ht="12.75">
+    <row r="2252" spans="1:2" ht="13.2">
       <c r="A2252" s="2"/>
       <c r="B2252" s="2"/>
     </row>
-    <row r="2253" spans="1:2" ht="12.75">
+    <row r="2253" spans="1:2" ht="13.2">
       <c r="A2253" s="2"/>
       <c r="B2253" s="2"/>
     </row>
-    <row r="2254" spans="1:2" ht="12.75">
+    <row r="2254" spans="1:2" ht="13.2">
       <c r="A2254" s="2"/>
       <c r="B2254" s="2"/>
     </row>
-    <row r="2255" spans="1:2" ht="12.75">
+    <row r="2255" spans="1:2" ht="13.2">
       <c r="A2255" s="2"/>
       <c r="B2255" s="2"/>
     </row>
-    <row r="2256" spans="1:2" ht="12.75">
+    <row r="2256" spans="1:2" ht="13.2">
       <c r="A2256" s="2"/>
       <c r="B2256" s="2"/>
     </row>
-    <row r="2257" spans="1:2" ht="12.75">
+    <row r="2257" spans="1:2" ht="13.2">
       <c r="A2257" s="2"/>
       <c r="B2257" s="2"/>
     </row>
-    <row r="2258" spans="1:2" ht="12.75">
+    <row r="2258" spans="1:2" ht="13.2">
       <c r="A2258" s="2"/>
       <c r="B2258" s="2"/>
     </row>
-    <row r="2259" spans="1:2" ht="12.75">
+    <row r="2259" spans="1:2" ht="13.2">
       <c r="A2259" s="2"/>
       <c r="B2259" s="2"/>
     </row>
-    <row r="2260" spans="1:2" ht="12.75">
+    <row r="2260" spans="1:2" ht="13.2">
       <c r="A2260" s="2"/>
       <c r="B2260" s="2"/>
     </row>
-    <row r="2261" spans="1:2" ht="12.75">
+    <row r="2261" spans="1:2" ht="13.2">
       <c r="A2261" s="2"/>
       <c r="B2261" s="2"/>
     </row>
-    <row r="2262" spans="1:2" ht="12.75">
+    <row r="2262" spans="1:2" ht="13.2">
       <c r="A2262" s="2"/>
       <c r="B2262" s="2"/>
     </row>
-    <row r="2263" spans="1:2" ht="12.75">
+    <row r="2263" spans="1:2" ht="13.2">
       <c r="A2263" s="2"/>
       <c r="B2263" s="2"/>
     </row>
-    <row r="2264" spans="1:2" ht="12.75">
+    <row r="2264" spans="1:2" ht="13.2">
       <c r="A2264" s="2"/>
       <c r="B2264" s="2"/>
     </row>
-    <row r="2265" spans="1:2" ht="12.75">
+    <row r="2265" spans="1:2" ht="13.2">
       <c r="A2265" s="2"/>
       <c r="B2265" s="2"/>
     </row>
-    <row r="2266" spans="1:2" ht="12.75">
+    <row r="2266" spans="1:2" ht="13.2">
       <c r="A2266" s="2"/>
       <c r="B2266" s="2"/>
     </row>
-    <row r="2267" spans="1:2" ht="12.75">
+    <row r="2267" spans="1:2" ht="13.2">
       <c r="A2267" s="2"/>
       <c r="B2267" s="2"/>
     </row>
-    <row r="2268" spans="1:2" ht="12.75">
+    <row r="2268" spans="1:2" ht="13.2">
       <c r="A2268" s="2"/>
       <c r="B2268" s="2"/>
     </row>
-    <row r="2269" spans="1:2" ht="12.75">
+    <row r="2269" spans="1:2" ht="13.2">
       <c r="A2269" s="2"/>
       <c r="B2269" s="2"/>
     </row>
-    <row r="2270" spans="1:2" ht="12.75">
+    <row r="2270" spans="1:2" ht="13.2">
       <c r="A2270" s="2"/>
       <c r="B2270" s="2"/>
     </row>
-    <row r="2271" spans="1:2" ht="12.75">
+    <row r="2271" spans="1:2" ht="13.2">
       <c r="A2271" s="2"/>
       <c r="B2271" s="2"/>
     </row>
-    <row r="2272" spans="1:2" ht="12.75">
+    <row r="2272" spans="1:2" ht="13.2">
       <c r="A2272" s="2"/>
       <c r="B2272" s="2"/>
     </row>
-    <row r="2273" spans="1:2" ht="12.75">
+    <row r="2273" spans="1:2" ht="13.2">
       <c r="A2273" s="2"/>
       <c r="B2273" s="2"/>
     </row>
-    <row r="2274" spans="1:2" ht="12.75">
+    <row r="2274" spans="1:2" ht="13.2">
       <c r="A2274" s="2"/>
       <c r="B2274" s="2"/>
     </row>
-    <row r="2275" spans="1:2" ht="12.75">
+    <row r="2275" spans="1:2" ht="13.2">
       <c r="A2275" s="2"/>
       <c r="B2275" s="2"/>
     </row>
-    <row r="2276" spans="1:2" ht="12.75">
+    <row r="2276" spans="1:2" ht="13.2">
       <c r="A2276" s="2"/>
       <c r="B2276" s="2"/>
     </row>
-    <row r="2277" spans="1:2" ht="12.75">
+    <row r="2277" spans="1:2" ht="13.2">
       <c r="A2277" s="2"/>
       <c r="B2277" s="2"/>
     </row>
-    <row r="2278" spans="1:2" ht="12.75">
+    <row r="2278" spans="1:2" ht="13.2">
       <c r="A2278" s="2"/>
       <c r="B2278" s="2"/>
     </row>
-    <row r="2279" spans="1:2" ht="12.75">
+    <row r="2279" spans="1:2" ht="13.2">
       <c r="A2279" s="2"/>
       <c r="B2279" s="2"/>
     </row>
-    <row r="2280" spans="1:2" ht="12.75">
+    <row r="2280" spans="1:2" ht="13.2">
       <c r="A2280" s="2"/>
       <c r="B2280" s="2"/>
     </row>
-    <row r="2281" spans="1:2" ht="12.75">
+    <row r="2281" spans="1:2" ht="13.2">
       <c r="A2281" s="2"/>
       <c r="B2281" s="2"/>
     </row>
-    <row r="2282" spans="1:2" ht="12.75">
+    <row r="2282" spans="1:2" ht="13.2">
       <c r="A2282" s="2"/>
       <c r="B2282" s="2"/>
     </row>
-    <row r="2283" spans="1:2" ht="12.75">
+    <row r="2283" spans="1:2" ht="13.2">
       <c r="A2283" s="2"/>
       <c r="B2283" s="2"/>
     </row>
-    <row r="2284" spans="1:2" ht="12.75">
+    <row r="2284" spans="1:2" ht="13.2">
       <c r="A2284" s="2"/>
       <c r="B2284" s="2"/>
     </row>
-    <row r="2285" spans="1:2" ht="12.75">
+    <row r="2285" spans="1:2" ht="13.2">
       <c r="A2285" s="2"/>
       <c r="B2285" s="2"/>
     </row>
-    <row r="2286" spans="1:2" ht="12.75">
+    <row r="2286" spans="1:2" ht="13.2">
       <c r="A2286" s="2"/>
       <c r="B2286" s="2"/>
     </row>
-    <row r="2287" spans="1:2" ht="12.75">
+    <row r="2287" spans="1:2" ht="13.2">
       <c r="A2287" s="2"/>
       <c r="B2287" s="2"/>
     </row>
-    <row r="2288" spans="1:2" ht="12.75">
+    <row r="2288" spans="1:2" ht="13.2">
       <c r="A2288" s="2"/>
       <c r="B2288" s="2"/>
     </row>
-    <row r="2289" spans="1:2" ht="12.75">
+    <row r="2289" spans="1:2" ht="13.2">
       <c r="A2289" s="2"/>
       <c r="B2289" s="2"/>
     </row>
-    <row r="2290" spans="1:2" ht="12.75">
+    <row r="2290" spans="1:2" ht="13.2">
       <c r="A2290" s="2"/>
       <c r="B2290" s="2"/>
     </row>
-    <row r="2291" spans="1:2" ht="12.75">
+    <row r="2291" spans="1:2" ht="13.2">
       <c r="A2291" s="2"/>
       <c r="B2291" s="2"/>
     </row>
-    <row r="2292" spans="1:2" ht="12.75">
+    <row r="2292" spans="1:2" ht="13.2">
       <c r="A2292" s="2"/>
       <c r="B2292" s="2"/>
     </row>
-    <row r="2293" spans="1:2" ht="12.75">
+    <row r="2293" spans="1:2" ht="13.2">
       <c r="A2293" s="2"/>
       <c r="B2293" s="2"/>
     </row>
-    <row r="2294" spans="1:2" ht="12.75">
+    <row r="2294" spans="1:2" ht="13.2">
       <c r="A2294" s="2"/>
       <c r="B2294" s="2"/>
     </row>
-    <row r="2295" spans="1:2" ht="12.75">
+    <row r="2295" spans="1:2" ht="13.2">
       <c r="A2295" s="2"/>
       <c r="B2295" s="2"/>
     </row>
-    <row r="2296" spans="1:2" ht="12.75">
+    <row r="2296" spans="1:2" ht="13.2">
       <c r="A2296" s="2"/>
       <c r="B2296" s="2"/>
     </row>
-    <row r="2297" spans="1:2" ht="12.75">
+    <row r="2297" spans="1:2" ht="13.2">
       <c r="A2297" s="2"/>
       <c r="B2297" s="2"/>
     </row>
-    <row r="2298" spans="1:2" ht="12.75">
+    <row r="2298" spans="1:2" ht="13.2">
       <c r="A2298" s="2"/>
       <c r="B2298" s="2"/>
     </row>
-    <row r="2299" spans="1:2" ht="12.75">
+    <row r="2299" spans="1:2" ht="13.2">
       <c r="A2299" s="2"/>
       <c r="B2299" s="2"/>
     </row>
-    <row r="2300" spans="1:2" ht="12.75">
+    <row r="2300" spans="1:2" ht="13.2">
       <c r="A2300" s="2"/>
       <c r="B2300" s="2"/>
     </row>
-    <row r="2301" spans="1:2" ht="12.75">
+    <row r="2301" spans="1:2" ht="13.2">
       <c r="A2301" s="2"/>
       <c r="B2301" s="2"/>
     </row>
-    <row r="2302" spans="1:2" ht="12.75">
+    <row r="2302" spans="1:2" ht="13.2">
       <c r="A2302" s="2"/>
       <c r="B2302" s="2"/>
     </row>
-    <row r="2303" spans="1:2" ht="12.75">
+    <row r="2303" spans="1:2" ht="13.2">
       <c r="A2303" s="2"/>
       <c r="B2303" s="2"/>
     </row>
-    <row r="2304" spans="1:2" ht="12.75">
+    <row r="2304" spans="1:2" ht="13.2">
       <c r="A2304" s="2"/>
       <c r="B2304" s="2"/>
     </row>
-    <row r="2305" spans="1:2" ht="12.75">
+    <row r="2305" spans="1:2" ht="13.2">
       <c r="A2305" s="2"/>
       <c r="B2305" s="2"/>
     </row>
-    <row r="2306" spans="1:2" ht="12.75">
+    <row r="2306" spans="1:2" ht="13.2">
       <c r="A2306" s="2"/>
       <c r="B2306" s="2"/>
     </row>
-    <row r="2307" spans="1:2" ht="12.75">
+    <row r="2307" spans="1:2" ht="13.2">
       <c r="A2307" s="2"/>
       <c r="B2307" s="2"/>
     </row>
-    <row r="2308" spans="1:2" ht="12.75">
+    <row r="2308" spans="1:2" ht="13.2">
       <c r="A2308" s="2"/>
       <c r="B2308" s="2"/>
     </row>
-    <row r="2309" spans="1:2" ht="12.75">
+    <row r="2309" spans="1:2" ht="13.2">
       <c r="A2309" s="2"/>
       <c r="B2309" s="2"/>
     </row>
-    <row r="2310" spans="1:2" ht="12.75">
+    <row r="2310" spans="1:2" ht="13.2">
       <c r="A2310" s="2"/>
       <c r="B2310" s="2"/>
     </row>
-    <row r="2311" spans="1:2" ht="12.75">
+    <row r="2311" spans="1:2" ht="13.2">
       <c r="A2311" s="2"/>
       <c r="B2311" s="2"/>
     </row>
-    <row r="2312" spans="1:2" ht="12.75">
+    <row r="2312" spans="1:2" ht="13.2">
       <c r="A2312" s="2"/>
       <c r="B2312" s="2"/>
     </row>
-    <row r="2313" spans="1:2" ht="12.75">
+    <row r="2313" spans="1:2" ht="13.2">
       <c r="A2313" s="2"/>
       <c r="B2313" s="2"/>
     </row>
-    <row r="2314" spans="1:2" ht="12.75">
+    <row r="2314" spans="1:2" ht="13.2">
       <c r="A2314" s="2"/>
       <c r="B2314" s="2"/>
     </row>
-    <row r="2315" spans="1:2" ht="12.75">
+    <row r="2315" spans="1:2" ht="13.2">
       <c r="A2315" s="2"/>
       <c r="B2315" s="2"/>
     </row>
-    <row r="2316" spans="1:2" ht="12.75">
+    <row r="2316" spans="1:2" ht="13.2">
       <c r="A2316" s="2"/>
       <c r="B2316" s="2"/>
     </row>
-    <row r="2317" spans="1:2" ht="12.75">
+    <row r="2317" spans="1:2" ht="13.2">
       <c r="A2317" s="2"/>
       <c r="B2317" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M5" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:M14" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="ABIERTO"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="A1">
-    <cfRule type="containsText" dxfId="60" priority="711" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="60" priority="713" operator="containsText" text="ABIERTO">
+      <formula>NOT(ISERROR(SEARCH("ABIERTO",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="59" priority="718" operator="containsText" text="ABIERTO">
+      <formula>NOT(ISERROR(SEARCH("ABIERTO",A1)))</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="58" priority="719" stopIfTrue="1" operator="equal">
+      <formula>"OPEN"</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="57" priority="711" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="59" priority="712" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="56" priority="712" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="58" priority="713" operator="containsText" text="ABIERTO">
+    <cfRule type="cellIs" dxfId="55" priority="720" stopIfTrue="1" operator="equal">
+      <formula>"CLOSED"</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="54" priority="714" operator="containsText" text="CERRADO">
+      <formula>NOT(ISERROR(SEARCH("CERRADO",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="53" priority="715" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="57" priority="714" operator="containsText" text="CERRADO">
+    <cfRule type="cellIs" dxfId="52" priority="721" stopIfTrue="1" operator="equal">
+      <formula>"IN PROGRESS"</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="51" priority="717" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="56" priority="715" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="55" priority="717" operator="containsText" text="CERRADO">
-      <formula>NOT(ISERROR(SEARCH("CERRADO",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="54" priority="718" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",A1)))</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="53" priority="719" stopIfTrue="1" operator="equal">
-      <formula>"OPEN"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="720" stopIfTrue="1" operator="equal">
-      <formula>"CLOSED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="721" stopIfTrue="1" operator="equal">
-      <formula>"IN PROGRESS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1 D1 D15:D1048576">
@@ -13669,23 +13676,23 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1">
-    <cfRule type="containsText" dxfId="48" priority="1744" operator="containsText" text="EN PROGRESO">
-      <formula>NOT(ISERROR(SEARCH("EN PROGRESO",B1)))</formula>
+    <cfRule type="containsText" dxfId="48" priority="1748" operator="containsText" text="ABIERTO">
+      <formula>NOT(ISERROR(SEARCH("ABIERTO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="47" priority="1745" operator="containsText" text="EN PROGRESO">
-      <formula>NOT(ISERROR(SEARCH("EN PROGRESO",B1)))</formula>
+    <cfRule type="containsText" dxfId="47" priority="1747" operator="containsText" text="CERRADO">
+      <formula>NOT(ISERROR(SEARCH("CERRADO",B1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="46" priority="1746" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="45" priority="1747" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="45" priority="1749" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="44" priority="1748" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",B1)))</formula>
+    <cfRule type="containsText" dxfId="44" priority="1745" operator="containsText" text="EN PROGRESO">
+      <formula>NOT(ISERROR(SEARCH("EN PROGRESO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="43" priority="1749" operator="containsText" text="CERRADO">
-      <formula>NOT(ISERROR(SEARCH("CERRADO",B1)))</formula>
+    <cfRule type="containsText" dxfId="43" priority="1744" operator="containsText" text="EN PROGRESO">
+      <formula>NOT(ISERROR(SEARCH("EN PROGRESO",B1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="42" priority="1750" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",B1)))</formula>
@@ -13719,14 +13726,14 @@
     <cfRule type="containsText" dxfId="33" priority="343" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="32" priority="1852" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="32" priority="1857" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="31" priority="1853" operator="containsText" text="Showstopper ">
+    <cfRule type="containsText" dxfId="31" priority="1852" operator="containsText" text="ALTO">
+      <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="30" priority="1853" operator="containsText" text="Showstopper ">
       <formula>NOT(ISERROR(SEARCH("Showstopper ",C1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="1857" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="29" priority="1858" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
@@ -13742,62 +13749,62 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C14">
-    <cfRule type="containsText" dxfId="25" priority="1" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="2" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="23" priority="4" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="24" priority="4" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="23" priority="1" operator="containsText" text="ALTO">
+      <formula>NOT(ISERROR(SEARCH("ALTO",C2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15:C1048576">
-    <cfRule type="containsText" dxfId="22" priority="1289" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="22" priority="1293" operator="containsText" text="MEDIO">
+      <formula>NOT(ISERROR(SEARCH("MEDIO",C15)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="21" priority="1294" operator="containsText" text="ALTO">
+      <formula>NOT(ISERROR(SEARCH("ALTO",C15)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="20" priority="1289" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="1291" operator="containsText" text="SHOWSTOPPER">
+    <cfRule type="containsText" dxfId="19" priority="1291" operator="containsText" text="SHOWSTOPPER">
       <formula>NOT(ISERROR(SEARCH("SHOWSTOPPER",C15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="1292" operator="containsText" text="show">
+    <cfRule type="containsText" dxfId="18" priority="1292" operator="containsText" text="show">
       <formula>NOT(ISERROR(SEARCH("show",C15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="19" priority="1293" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="1294" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1 D15:D1048576">
-    <cfRule type="containsText" dxfId="17" priority="197" operator="containsText" text="NO APLICA">
-      <formula>NOT(ISERROR(SEARCH("NO APLICA",D1)))</formula>
+    <cfRule type="containsText" dxfId="17" priority="1769" operator="containsText" text="EN PROGRESO">
+      <formula>NOT(ISERROR(SEARCH("EN PROGRESO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="205" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="16" priority="1770" operator="containsText" text="EN PROGRESO">
+      <formula>NOT(ISERROR(SEARCH("EN PROGRESO",D1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="1771" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="1769" operator="containsText" text="EN PROGRESO">
-      <formula>NOT(ISERROR(SEARCH("EN PROGRESO",D1)))</formula>
+    <cfRule type="containsText" dxfId="14" priority="1772" operator="containsText" text="CERRADO">
+      <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="1770" operator="containsText" text="EN PROGRESO">
-      <formula>NOT(ISERROR(SEARCH("EN PROGRESO",D1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="1771" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="13" priority="205" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="1772" operator="containsText" text="CERRADO">
-      <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
+    <cfRule type="containsText" dxfId="12" priority="197" operator="containsText" text="NO APLICA">
+      <formula>NOT(ISERROR(SEARCH("NO APLICA",D1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="containsText" dxfId="11" priority="1730" operator="containsText" text="PENDIENTE">
+    <cfRule type="containsText" dxfId="11" priority="1851" operator="containsText" text="ABIERTO">
+      <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="1730" operator="containsText" text="PENDIENTE">
       <formula>NOT(ISERROR(SEARCH("PENDIENTE",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="1735" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="9" priority="1735" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="1851" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="8" priority="1854" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
@@ -13824,11 +13831,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D15:D1048576">
-    <cfRule type="containsText" dxfId="1" priority="1295" operator="containsText" text="PENDIENTE">
+    <cfRule type="containsText" dxfId="1" priority="1498" operator="containsText" text="CERRADO">
+      <formula>NOT(ISERROR(SEARCH("CERRADO",D15)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="1295" operator="containsText" text="PENDIENTE">
       <formula>NOT(ISERROR(SEARCH("PENDIENTE",D15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="1498" operator="containsText" text="CERRADO">
-      <formula>NOT(ISERROR(SEARCH("CERRADO",D15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
@@ -13870,12 +13877,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02A2ABB5-42B5-497D-950A-71A244302DF4}">
   <dimension ref="B1:J19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2"/>
   <cols>
-    <col min="2" max="2" width="24.42578125" customWidth="1"/>
-    <col min="3" max="3" width="31.42578125" customWidth="1"/>
-    <col min="4" max="4" width="46.42578125" customWidth="1"/>
-    <col min="5" max="5" width="26.42578125" customWidth="1"/>
+    <col min="2" max="2" width="24.44140625" customWidth="1"/>
+    <col min="3" max="3" width="31.44140625" customWidth="1"/>
+    <col min="4" max="4" width="46.44140625" customWidth="1"/>
+    <col min="5" max="5" width="26.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:10" s="1" customFormat="1" ht="55.35" customHeight="1">

</xml_diff>

<commit_message>
update incidencias para isra
</commit_message>
<xml_diff>
--- a/validaciones_Y_ChecklistDeRequerimeintos/Copia de CheckList_Estatus-001-V.1.5DEV (1).xlsx
+++ b/validaciones_Y_ChecklistDeRequerimeintos/Copia de CheckList_Estatus-001-V.1.5DEV (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ITZELPROYECTO\integradoraTeampoderoso\validaciones_Y_ChecklistDeRequerimeintos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFBB523A-A001-4458-B69C-607D5481EDF2}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49B5453A-FA3B-4AEF-8DE9-EB30EFC2F50E}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="586" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="60">
   <si>
     <t>Descripción</t>
   </si>
@@ -261,6 +261,18 @@
   <si>
     <t>PANTALLA:Admin
 No se permite cancelar una cita ya que al dar clic en el icono de tachesito no realiza ninguna accion, y añadir sus descripciones a los iconos. Eliminar y Editar, ademas de agregar alerta de cuando se edita la cita y cuando se elimina.</t>
+  </si>
+  <si>
+    <t>PANTALLA:Admin-Citas
+Inicializar el firltro de buscar en la seccion de nombre, actualmente inciia con numero.</t>
+  </si>
+  <si>
+    <t>PANTALLA:Admin-Citas
+Mostrar el campo de numero de telefono , abajito de el estatus de la cita</t>
+  </si>
+  <si>
+    <t>PANTALLA:Admin-Citas
+Limitar el agendamineto de citas con el mismo numero de telefono a 4 citas por día.</t>
   </si>
 </sst>
 </file>
@@ -636,7 +648,151 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
   </cellStyles>
-  <dxfs count="93">
+  <dxfs count="105">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="7" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -2845,6 +3001,142 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>312964</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>734785</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>5333340</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>1792208</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Imagen 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6276927C-4033-4A1E-B71C-97CC79ECD8B6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1319893" y="75084214"/>
+          <a:ext cx="5020376" cy="1057423"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>68035</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>830037</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>6594586</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>2516290</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="31" name="Imagen 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1992F649-7E8B-4BAA-B88F-B8B9AA6A79FF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1074964" y="78690108"/>
+          <a:ext cx="6526551" cy="1686253"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3088821</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>2326822</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3510642</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>2966358</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="34" name="Conector recto de flecha 33">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D7654438-B265-4538-BF47-4F4A679C3478}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm flipV="1">
+          <a:off x="4095750" y="80186893"/>
+          <a:ext cx="421821" cy="639536"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="9"/>
+        </a:solidFill>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
+          <a:headEnd type="none" w="med" len="med"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -8927,14 +9219,674 @@
       <c r="HB22" s="15"/>
       <c r="HC22" s="15"/>
     </row>
-    <row r="23" spans="1:211">
-      <c r="A23" s="28"/>
-    </row>
-    <row r="24" spans="1:211">
-      <c r="A24" s="28"/>
-    </row>
-    <row r="25" spans="1:211">
-      <c r="A25" s="28"/>
+    <row r="23" spans="1:211" ht="277.14999999999998" customHeight="1">
+      <c r="A23" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="39" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="F23" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="G23" s="20">
+        <v>45986</v>
+      </c>
+      <c r="H23" s="30"/>
+      <c r="I23" s="20">
+        <v>45960</v>
+      </c>
+      <c r="J23" s="20">
+        <v>45961</v>
+      </c>
+      <c r="K23" s="31"/>
+      <c r="L23" s="32"/>
+      <c r="M23" s="32"/>
+      <c r="V23" s="15"/>
+      <c r="W23" s="15"/>
+      <c r="X23" s="15"/>
+      <c r="Y23" s="15"/>
+      <c r="Z23" s="15"/>
+      <c r="AA23" s="15"/>
+      <c r="AB23" s="15"/>
+      <c r="AC23" s="15"/>
+      <c r="AD23" s="15"/>
+      <c r="AE23" s="15"/>
+      <c r="AF23" s="15"/>
+      <c r="AG23" s="15"/>
+      <c r="AH23" s="15"/>
+      <c r="AI23" s="15"/>
+      <c r="AJ23" s="15"/>
+      <c r="AK23" s="15"/>
+      <c r="AL23" s="15"/>
+      <c r="AM23" s="15"/>
+      <c r="AN23" s="15"/>
+      <c r="AO23" s="15"/>
+      <c r="AP23" s="15"/>
+      <c r="AQ23" s="15"/>
+      <c r="AR23" s="15"/>
+      <c r="AS23" s="15"/>
+      <c r="AT23" s="15"/>
+      <c r="AU23" s="15"/>
+      <c r="AV23" s="15"/>
+      <c r="AW23" s="15"/>
+      <c r="AX23" s="15"/>
+      <c r="AY23" s="15"/>
+      <c r="AZ23" s="15"/>
+      <c r="BA23" s="15"/>
+      <c r="BB23" s="15"/>
+      <c r="BC23" s="15"/>
+      <c r="BD23" s="15"/>
+      <c r="BE23" s="15"/>
+      <c r="BF23" s="15"/>
+      <c r="BG23" s="15"/>
+      <c r="BH23" s="15"/>
+      <c r="BI23" s="15"/>
+      <c r="BJ23" s="15"/>
+      <c r="BK23" s="15"/>
+      <c r="BL23" s="15"/>
+      <c r="BM23" s="15"/>
+      <c r="BN23" s="15"/>
+      <c r="BO23" s="15"/>
+      <c r="BP23" s="15"/>
+      <c r="BQ23" s="15"/>
+      <c r="BR23" s="15"/>
+      <c r="BS23" s="15"/>
+      <c r="BT23" s="15"/>
+      <c r="BU23" s="15"/>
+      <c r="BV23" s="15"/>
+      <c r="BW23" s="15"/>
+      <c r="BX23" s="15"/>
+      <c r="BY23" s="15"/>
+      <c r="BZ23" s="15"/>
+      <c r="CA23" s="15"/>
+      <c r="CB23" s="15"/>
+      <c r="CC23" s="15"/>
+      <c r="CD23" s="15"/>
+      <c r="CE23" s="15"/>
+      <c r="CF23" s="15"/>
+      <c r="CG23" s="15"/>
+      <c r="CH23" s="15"/>
+      <c r="CI23" s="15"/>
+      <c r="CJ23" s="15"/>
+      <c r="CK23" s="15"/>
+      <c r="CL23" s="15"/>
+      <c r="CM23" s="15"/>
+      <c r="CN23" s="15"/>
+      <c r="CO23" s="15"/>
+      <c r="CP23" s="15"/>
+      <c r="CQ23" s="15"/>
+      <c r="CR23" s="15"/>
+      <c r="CS23" s="15"/>
+      <c r="CT23" s="15"/>
+      <c r="CU23" s="15"/>
+      <c r="CV23" s="15"/>
+      <c r="CW23" s="15"/>
+      <c r="CX23" s="15"/>
+      <c r="CY23" s="15"/>
+      <c r="CZ23" s="15"/>
+      <c r="DA23" s="15"/>
+      <c r="DB23" s="15"/>
+      <c r="DC23" s="15"/>
+      <c r="DD23" s="15"/>
+      <c r="DE23" s="15"/>
+      <c r="DF23" s="15"/>
+      <c r="DG23" s="15"/>
+      <c r="DH23" s="15"/>
+      <c r="DI23" s="15"/>
+      <c r="DJ23" s="15"/>
+      <c r="DK23" s="15"/>
+      <c r="DL23" s="15"/>
+      <c r="DM23" s="15"/>
+      <c r="DN23" s="15"/>
+      <c r="DO23" s="15"/>
+      <c r="DP23" s="15"/>
+      <c r="DQ23" s="15"/>
+      <c r="DR23" s="15"/>
+      <c r="DS23" s="15"/>
+      <c r="DT23" s="15"/>
+      <c r="DU23" s="15"/>
+      <c r="DV23" s="15"/>
+      <c r="DW23" s="15"/>
+      <c r="DX23" s="15"/>
+      <c r="DY23" s="15"/>
+      <c r="DZ23" s="15"/>
+      <c r="EA23" s="15"/>
+      <c r="EB23" s="15"/>
+      <c r="EC23" s="15"/>
+      <c r="ED23" s="15"/>
+      <c r="EE23" s="15"/>
+      <c r="EF23" s="15"/>
+      <c r="EG23" s="15"/>
+      <c r="EH23" s="15"/>
+      <c r="EI23" s="15"/>
+      <c r="EJ23" s="15"/>
+      <c r="EK23" s="15"/>
+      <c r="EL23" s="15"/>
+      <c r="EM23" s="15"/>
+      <c r="EN23" s="15"/>
+      <c r="EO23" s="15"/>
+      <c r="EP23" s="15"/>
+      <c r="EQ23" s="15"/>
+      <c r="ER23" s="15"/>
+      <c r="ES23" s="15"/>
+      <c r="ET23" s="15"/>
+      <c r="EU23" s="15"/>
+      <c r="EV23" s="15"/>
+      <c r="EW23" s="15"/>
+      <c r="EX23" s="15"/>
+      <c r="EY23" s="15"/>
+      <c r="EZ23" s="15"/>
+      <c r="FA23" s="15"/>
+      <c r="FB23" s="15"/>
+      <c r="FC23" s="15"/>
+      <c r="FD23" s="15"/>
+      <c r="FE23" s="15"/>
+      <c r="FF23" s="15"/>
+      <c r="FG23" s="15"/>
+      <c r="FH23" s="15"/>
+      <c r="FI23" s="15"/>
+      <c r="FJ23" s="15"/>
+      <c r="FK23" s="15"/>
+      <c r="FL23" s="15"/>
+      <c r="FM23" s="15"/>
+      <c r="FN23" s="15"/>
+      <c r="FO23" s="15"/>
+      <c r="FP23" s="15"/>
+      <c r="FQ23" s="15"/>
+      <c r="FR23" s="15"/>
+      <c r="FS23" s="15"/>
+      <c r="FT23" s="15"/>
+      <c r="FU23" s="15"/>
+      <c r="FV23" s="15"/>
+      <c r="FW23" s="15"/>
+      <c r="FX23" s="15"/>
+      <c r="FY23" s="15"/>
+      <c r="FZ23" s="15"/>
+      <c r="GA23" s="15"/>
+      <c r="GB23" s="15"/>
+      <c r="GC23" s="15"/>
+      <c r="GD23" s="15"/>
+      <c r="GE23" s="15"/>
+      <c r="GF23" s="15"/>
+      <c r="GG23" s="15"/>
+      <c r="GH23" s="15"/>
+      <c r="GI23" s="15"/>
+      <c r="GJ23" s="15"/>
+      <c r="GK23" s="15"/>
+      <c r="GL23" s="15"/>
+      <c r="GM23" s="15"/>
+      <c r="GN23" s="15"/>
+      <c r="GO23" s="15"/>
+      <c r="GP23" s="15"/>
+      <c r="GQ23" s="15"/>
+      <c r="GR23" s="15"/>
+      <c r="GS23" s="15"/>
+      <c r="GT23" s="15"/>
+      <c r="GU23" s="15"/>
+      <c r="GV23" s="15"/>
+      <c r="GW23" s="15"/>
+      <c r="GX23" s="15"/>
+      <c r="GY23" s="15"/>
+      <c r="GZ23" s="15"/>
+      <c r="HA23" s="15"/>
+      <c r="HB23" s="15"/>
+      <c r="HC23" s="15"/>
+    </row>
+    <row r="24" spans="1:211" ht="277.14999999999998" customHeight="1">
+      <c r="A24" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="39" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="F24" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="G24" s="20">
+        <v>45986</v>
+      </c>
+      <c r="H24" s="30"/>
+      <c r="I24" s="20">
+        <v>45960</v>
+      </c>
+      <c r="J24" s="20">
+        <v>45961</v>
+      </c>
+      <c r="K24" s="31"/>
+      <c r="L24" s="32"/>
+      <c r="M24" s="32"/>
+      <c r="V24" s="15"/>
+      <c r="W24" s="15"/>
+      <c r="X24" s="15"/>
+      <c r="Y24" s="15"/>
+      <c r="Z24" s="15"/>
+      <c r="AA24" s="15"/>
+      <c r="AB24" s="15"/>
+      <c r="AC24" s="15"/>
+      <c r="AD24" s="15"/>
+      <c r="AE24" s="15"/>
+      <c r="AF24" s="15"/>
+      <c r="AG24" s="15"/>
+      <c r="AH24" s="15"/>
+      <c r="AI24" s="15"/>
+      <c r="AJ24" s="15"/>
+      <c r="AK24" s="15"/>
+      <c r="AL24" s="15"/>
+      <c r="AM24" s="15"/>
+      <c r="AN24" s="15"/>
+      <c r="AO24" s="15"/>
+      <c r="AP24" s="15"/>
+      <c r="AQ24" s="15"/>
+      <c r="AR24" s="15"/>
+      <c r="AS24" s="15"/>
+      <c r="AT24" s="15"/>
+      <c r="AU24" s="15"/>
+      <c r="AV24" s="15"/>
+      <c r="AW24" s="15"/>
+      <c r="AX24" s="15"/>
+      <c r="AY24" s="15"/>
+      <c r="AZ24" s="15"/>
+      <c r="BA24" s="15"/>
+      <c r="BB24" s="15"/>
+      <c r="BC24" s="15"/>
+      <c r="BD24" s="15"/>
+      <c r="BE24" s="15"/>
+      <c r="BF24" s="15"/>
+      <c r="BG24" s="15"/>
+      <c r="BH24" s="15"/>
+      <c r="BI24" s="15"/>
+      <c r="BJ24" s="15"/>
+      <c r="BK24" s="15"/>
+      <c r="BL24" s="15"/>
+      <c r="BM24" s="15"/>
+      <c r="BN24" s="15"/>
+      <c r="BO24" s="15"/>
+      <c r="BP24" s="15"/>
+      <c r="BQ24" s="15"/>
+      <c r="BR24" s="15"/>
+      <c r="BS24" s="15"/>
+      <c r="BT24" s="15"/>
+      <c r="BU24" s="15"/>
+      <c r="BV24" s="15"/>
+      <c r="BW24" s="15"/>
+      <c r="BX24" s="15"/>
+      <c r="BY24" s="15"/>
+      <c r="BZ24" s="15"/>
+      <c r="CA24" s="15"/>
+      <c r="CB24" s="15"/>
+      <c r="CC24" s="15"/>
+      <c r="CD24" s="15"/>
+      <c r="CE24" s="15"/>
+      <c r="CF24" s="15"/>
+      <c r="CG24" s="15"/>
+      <c r="CH24" s="15"/>
+      <c r="CI24" s="15"/>
+      <c r="CJ24" s="15"/>
+      <c r="CK24" s="15"/>
+      <c r="CL24" s="15"/>
+      <c r="CM24" s="15"/>
+      <c r="CN24" s="15"/>
+      <c r="CO24" s="15"/>
+      <c r="CP24" s="15"/>
+      <c r="CQ24" s="15"/>
+      <c r="CR24" s="15"/>
+      <c r="CS24" s="15"/>
+      <c r="CT24" s="15"/>
+      <c r="CU24" s="15"/>
+      <c r="CV24" s="15"/>
+      <c r="CW24" s="15"/>
+      <c r="CX24" s="15"/>
+      <c r="CY24" s="15"/>
+      <c r="CZ24" s="15"/>
+      <c r="DA24" s="15"/>
+      <c r="DB24" s="15"/>
+      <c r="DC24" s="15"/>
+      <c r="DD24" s="15"/>
+      <c r="DE24" s="15"/>
+      <c r="DF24" s="15"/>
+      <c r="DG24" s="15"/>
+      <c r="DH24" s="15"/>
+      <c r="DI24" s="15"/>
+      <c r="DJ24" s="15"/>
+      <c r="DK24" s="15"/>
+      <c r="DL24" s="15"/>
+      <c r="DM24" s="15"/>
+      <c r="DN24" s="15"/>
+      <c r="DO24" s="15"/>
+      <c r="DP24" s="15"/>
+      <c r="DQ24" s="15"/>
+      <c r="DR24" s="15"/>
+      <c r="DS24" s="15"/>
+      <c r="DT24" s="15"/>
+      <c r="DU24" s="15"/>
+      <c r="DV24" s="15"/>
+      <c r="DW24" s="15"/>
+      <c r="DX24" s="15"/>
+      <c r="DY24" s="15"/>
+      <c r="DZ24" s="15"/>
+      <c r="EA24" s="15"/>
+      <c r="EB24" s="15"/>
+      <c r="EC24" s="15"/>
+      <c r="ED24" s="15"/>
+      <c r="EE24" s="15"/>
+      <c r="EF24" s="15"/>
+      <c r="EG24" s="15"/>
+      <c r="EH24" s="15"/>
+      <c r="EI24" s="15"/>
+      <c r="EJ24" s="15"/>
+      <c r="EK24" s="15"/>
+      <c r="EL24" s="15"/>
+      <c r="EM24" s="15"/>
+      <c r="EN24" s="15"/>
+      <c r="EO24" s="15"/>
+      <c r="EP24" s="15"/>
+      <c r="EQ24" s="15"/>
+      <c r="ER24" s="15"/>
+      <c r="ES24" s="15"/>
+      <c r="ET24" s="15"/>
+      <c r="EU24" s="15"/>
+      <c r="EV24" s="15"/>
+      <c r="EW24" s="15"/>
+      <c r="EX24" s="15"/>
+      <c r="EY24" s="15"/>
+      <c r="EZ24" s="15"/>
+      <c r="FA24" s="15"/>
+      <c r="FB24" s="15"/>
+      <c r="FC24" s="15"/>
+      <c r="FD24" s="15"/>
+      <c r="FE24" s="15"/>
+      <c r="FF24" s="15"/>
+      <c r="FG24" s="15"/>
+      <c r="FH24" s="15"/>
+      <c r="FI24" s="15"/>
+      <c r="FJ24" s="15"/>
+      <c r="FK24" s="15"/>
+      <c r="FL24" s="15"/>
+      <c r="FM24" s="15"/>
+      <c r="FN24" s="15"/>
+      <c r="FO24" s="15"/>
+      <c r="FP24" s="15"/>
+      <c r="FQ24" s="15"/>
+      <c r="FR24" s="15"/>
+      <c r="FS24" s="15"/>
+      <c r="FT24" s="15"/>
+      <c r="FU24" s="15"/>
+      <c r="FV24" s="15"/>
+      <c r="FW24" s="15"/>
+      <c r="FX24" s="15"/>
+      <c r="FY24" s="15"/>
+      <c r="FZ24" s="15"/>
+      <c r="GA24" s="15"/>
+      <c r="GB24" s="15"/>
+      <c r="GC24" s="15"/>
+      <c r="GD24" s="15"/>
+      <c r="GE24" s="15"/>
+      <c r="GF24" s="15"/>
+      <c r="GG24" s="15"/>
+      <c r="GH24" s="15"/>
+      <c r="GI24" s="15"/>
+      <c r="GJ24" s="15"/>
+      <c r="GK24" s="15"/>
+      <c r="GL24" s="15"/>
+      <c r="GM24" s="15"/>
+      <c r="GN24" s="15"/>
+      <c r="GO24" s="15"/>
+      <c r="GP24" s="15"/>
+      <c r="GQ24" s="15"/>
+      <c r="GR24" s="15"/>
+      <c r="GS24" s="15"/>
+      <c r="GT24" s="15"/>
+      <c r="GU24" s="15"/>
+      <c r="GV24" s="15"/>
+      <c r="GW24" s="15"/>
+      <c r="GX24" s="15"/>
+      <c r="GY24" s="15"/>
+      <c r="GZ24" s="15"/>
+      <c r="HA24" s="15"/>
+      <c r="HB24" s="15"/>
+      <c r="HC24" s="15"/>
+    </row>
+    <row r="25" spans="1:211" ht="58.5" customHeight="1">
+      <c r="A25" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="39" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="E25" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="G25" s="20">
+        <v>45986</v>
+      </c>
+      <c r="H25" s="30"/>
+      <c r="I25" s="20">
+        <v>45960</v>
+      </c>
+      <c r="J25" s="20">
+        <v>45961</v>
+      </c>
+      <c r="K25" s="31"/>
+      <c r="L25" s="32"/>
+      <c r="M25" s="32"/>
+      <c r="V25" s="15"/>
+      <c r="W25" s="15"/>
+      <c r="X25" s="15"/>
+      <c r="Y25" s="15"/>
+      <c r="Z25" s="15"/>
+      <c r="AA25" s="15"/>
+      <c r="AB25" s="15"/>
+      <c r="AC25" s="15"/>
+      <c r="AD25" s="15"/>
+      <c r="AE25" s="15"/>
+      <c r="AF25" s="15"/>
+      <c r="AG25" s="15"/>
+      <c r="AH25" s="15"/>
+      <c r="AI25" s="15"/>
+      <c r="AJ25" s="15"/>
+      <c r="AK25" s="15"/>
+      <c r="AL25" s="15"/>
+      <c r="AM25" s="15"/>
+      <c r="AN25" s="15"/>
+      <c r="AO25" s="15"/>
+      <c r="AP25" s="15"/>
+      <c r="AQ25" s="15"/>
+      <c r="AR25" s="15"/>
+      <c r="AS25" s="15"/>
+      <c r="AT25" s="15"/>
+      <c r="AU25" s="15"/>
+      <c r="AV25" s="15"/>
+      <c r="AW25" s="15"/>
+      <c r="AX25" s="15"/>
+      <c r="AY25" s="15"/>
+      <c r="AZ25" s="15"/>
+      <c r="BA25" s="15"/>
+      <c r="BB25" s="15"/>
+      <c r="BC25" s="15"/>
+      <c r="BD25" s="15"/>
+      <c r="BE25" s="15"/>
+      <c r="BF25" s="15"/>
+      <c r="BG25" s="15"/>
+      <c r="BH25" s="15"/>
+      <c r="BI25" s="15"/>
+      <c r="BJ25" s="15"/>
+      <c r="BK25" s="15"/>
+      <c r="BL25" s="15"/>
+      <c r="BM25" s="15"/>
+      <c r="BN25" s="15"/>
+      <c r="BO25" s="15"/>
+      <c r="BP25" s="15"/>
+      <c r="BQ25" s="15"/>
+      <c r="BR25" s="15"/>
+      <c r="BS25" s="15"/>
+      <c r="BT25" s="15"/>
+      <c r="BU25" s="15"/>
+      <c r="BV25" s="15"/>
+      <c r="BW25" s="15"/>
+      <c r="BX25" s="15"/>
+      <c r="BY25" s="15"/>
+      <c r="BZ25" s="15"/>
+      <c r="CA25" s="15"/>
+      <c r="CB25" s="15"/>
+      <c r="CC25" s="15"/>
+      <c r="CD25" s="15"/>
+      <c r="CE25" s="15"/>
+      <c r="CF25" s="15"/>
+      <c r="CG25" s="15"/>
+      <c r="CH25" s="15"/>
+      <c r="CI25" s="15"/>
+      <c r="CJ25" s="15"/>
+      <c r="CK25" s="15"/>
+      <c r="CL25" s="15"/>
+      <c r="CM25" s="15"/>
+      <c r="CN25" s="15"/>
+      <c r="CO25" s="15"/>
+      <c r="CP25" s="15"/>
+      <c r="CQ25" s="15"/>
+      <c r="CR25" s="15"/>
+      <c r="CS25" s="15"/>
+      <c r="CT25" s="15"/>
+      <c r="CU25" s="15"/>
+      <c r="CV25" s="15"/>
+      <c r="CW25" s="15"/>
+      <c r="CX25" s="15"/>
+      <c r="CY25" s="15"/>
+      <c r="CZ25" s="15"/>
+      <c r="DA25" s="15"/>
+      <c r="DB25" s="15"/>
+      <c r="DC25" s="15"/>
+      <c r="DD25" s="15"/>
+      <c r="DE25" s="15"/>
+      <c r="DF25" s="15"/>
+      <c r="DG25" s="15"/>
+      <c r="DH25" s="15"/>
+      <c r="DI25" s="15"/>
+      <c r="DJ25" s="15"/>
+      <c r="DK25" s="15"/>
+      <c r="DL25" s="15"/>
+      <c r="DM25" s="15"/>
+      <c r="DN25" s="15"/>
+      <c r="DO25" s="15"/>
+      <c r="DP25" s="15"/>
+      <c r="DQ25" s="15"/>
+      <c r="DR25" s="15"/>
+      <c r="DS25" s="15"/>
+      <c r="DT25" s="15"/>
+      <c r="DU25" s="15"/>
+      <c r="DV25" s="15"/>
+      <c r="DW25" s="15"/>
+      <c r="DX25" s="15"/>
+      <c r="DY25" s="15"/>
+      <c r="DZ25" s="15"/>
+      <c r="EA25" s="15"/>
+      <c r="EB25" s="15"/>
+      <c r="EC25" s="15"/>
+      <c r="ED25" s="15"/>
+      <c r="EE25" s="15"/>
+      <c r="EF25" s="15"/>
+      <c r="EG25" s="15"/>
+      <c r="EH25" s="15"/>
+      <c r="EI25" s="15"/>
+      <c r="EJ25" s="15"/>
+      <c r="EK25" s="15"/>
+      <c r="EL25" s="15"/>
+      <c r="EM25" s="15"/>
+      <c r="EN25" s="15"/>
+      <c r="EO25" s="15"/>
+      <c r="EP25" s="15"/>
+      <c r="EQ25" s="15"/>
+      <c r="ER25" s="15"/>
+      <c r="ES25" s="15"/>
+      <c r="ET25" s="15"/>
+      <c r="EU25" s="15"/>
+      <c r="EV25" s="15"/>
+      <c r="EW25" s="15"/>
+      <c r="EX25" s="15"/>
+      <c r="EY25" s="15"/>
+      <c r="EZ25" s="15"/>
+      <c r="FA25" s="15"/>
+      <c r="FB25" s="15"/>
+      <c r="FC25" s="15"/>
+      <c r="FD25" s="15"/>
+      <c r="FE25" s="15"/>
+      <c r="FF25" s="15"/>
+      <c r="FG25" s="15"/>
+      <c r="FH25" s="15"/>
+      <c r="FI25" s="15"/>
+      <c r="FJ25" s="15"/>
+      <c r="FK25" s="15"/>
+      <c r="FL25" s="15"/>
+      <c r="FM25" s="15"/>
+      <c r="FN25" s="15"/>
+      <c r="FO25" s="15"/>
+      <c r="FP25" s="15"/>
+      <c r="FQ25" s="15"/>
+      <c r="FR25" s="15"/>
+      <c r="FS25" s="15"/>
+      <c r="FT25" s="15"/>
+      <c r="FU25" s="15"/>
+      <c r="FV25" s="15"/>
+      <c r="FW25" s="15"/>
+      <c r="FX25" s="15"/>
+      <c r="FY25" s="15"/>
+      <c r="FZ25" s="15"/>
+      <c r="GA25" s="15"/>
+      <c r="GB25" s="15"/>
+      <c r="GC25" s="15"/>
+      <c r="GD25" s="15"/>
+      <c r="GE25" s="15"/>
+      <c r="GF25" s="15"/>
+      <c r="GG25" s="15"/>
+      <c r="GH25" s="15"/>
+      <c r="GI25" s="15"/>
+      <c r="GJ25" s="15"/>
+      <c r="GK25" s="15"/>
+      <c r="GL25" s="15"/>
+      <c r="GM25" s="15"/>
+      <c r="GN25" s="15"/>
+      <c r="GO25" s="15"/>
+      <c r="GP25" s="15"/>
+      <c r="GQ25" s="15"/>
+      <c r="GR25" s="15"/>
+      <c r="GS25" s="15"/>
+      <c r="GT25" s="15"/>
+      <c r="GU25" s="15"/>
+      <c r="GV25" s="15"/>
+      <c r="GW25" s="15"/>
+      <c r="GX25" s="15"/>
+      <c r="GY25" s="15"/>
+      <c r="GZ25" s="15"/>
+      <c r="HA25" s="15"/>
+      <c r="HB25" s="15"/>
+      <c r="HC25" s="15"/>
     </row>
     <row r="26" spans="1:211">
       <c r="A26" s="28"/>
@@ -16153,347 +17105,395 @@
   <autoFilter ref="A1:M14" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="A1">
-    <cfRule type="containsText" dxfId="92" priority="745" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="104" priority="757" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="91" priority="750" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="103" priority="762" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",A1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="751" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="102" priority="763" stopIfTrue="1" operator="equal">
       <formula>"OPEN"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="89" priority="743" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="101" priority="755" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="88" priority="744" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="100" priority="756" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",A1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="87" priority="752" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="99" priority="764" stopIfTrue="1" operator="equal">
       <formula>"CLOSED"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="86" priority="746" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="98" priority="758" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="85" priority="747" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="97" priority="759" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",A1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="753" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="96" priority="765" stopIfTrue="1" operator="equal">
       <formula>"IN PROGRESS"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="83" priority="749" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="95" priority="761" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:B1 D1 D23:D1048576">
-    <cfRule type="containsText" dxfId="82" priority="748" operator="containsText" text="CERRADO">
+  <conditionalFormatting sqref="A1:B1 D1 D26:D1048576">
+    <cfRule type="containsText" dxfId="94" priority="760" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="containsText" dxfId="81" priority="396" operator="containsText" text="PENDIENTE">
+    <cfRule type="containsText" dxfId="93" priority="408" operator="containsText" text="PENDIENTE">
       <formula>NOT(ISERROR(SEARCH("PENDIENTE",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1">
-    <cfRule type="containsText" dxfId="80" priority="1780" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="92" priority="1792" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="79" priority="1779" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="91" priority="1791" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="78" priority="1778" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="90" priority="1790" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="77" priority="1781" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="89" priority="1793" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="76" priority="1777" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="88" priority="1789" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="75" priority="1776" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="87" priority="1788" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="74" priority="1782" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="86" priority="1794" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="73" priority="1783" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="85" priority="1795" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",B1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="1784" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="1796" stopIfTrue="1" operator="equal">
       <formula>"OPEN"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="71" priority="1785" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="1797" stopIfTrue="1" operator="equal">
       <formula>"CLOSED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="1786" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="82" priority="1798" stopIfTrue="1" operator="equal">
       <formula>"IN PROGRESS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="containsText" dxfId="69" priority="370" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="81" priority="382" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="68" priority="372" operator="containsText" text="SHOWSTOPPER">
+    <cfRule type="containsText" dxfId="80" priority="384" operator="containsText" text="SHOWSTOPPER">
       <formula>NOT(ISERROR(SEARCH("SHOWSTOPPER",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="67" priority="373" operator="containsText" text="show">
+    <cfRule type="containsText" dxfId="79" priority="385" operator="containsText" text="show">
       <formula>NOT(ISERROR(SEARCH("show",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="66" priority="374" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="78" priority="386" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="65" priority="375" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="77" priority="387" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="64" priority="1889" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="76" priority="1901" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="63" priority="1884" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="75" priority="1896" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="62" priority="1885" operator="containsText" text="Showstopper ">
+    <cfRule type="containsText" dxfId="74" priority="1897" operator="containsText" text="Showstopper ">
       <formula>NOT(ISERROR(SEARCH("Showstopper ",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="61" priority="1890" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="73" priority="1902" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="1891" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="1903" stopIfTrue="1" operator="equal">
       <formula>"Medio"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="59" priority="1892" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="71" priority="1904" stopIfTrue="1" operator="equal">
       <formula>"Bajo"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="1893" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="70" priority="1905" stopIfTrue="1" operator="equal">
       <formula>"Alto"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C14">
-    <cfRule type="containsText" dxfId="57" priority="34" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="69" priority="46" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="56" priority="36" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="68" priority="48" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="55" priority="33" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="67" priority="45" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C23:C1048576">
-    <cfRule type="containsText" dxfId="54" priority="1325" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C23)))</formula>
+  <conditionalFormatting sqref="C26:C1048576">
+    <cfRule type="containsText" dxfId="66" priority="1337" operator="containsText" text="MEDIO">
+      <formula>NOT(ISERROR(SEARCH("MEDIO",C26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="53" priority="1326" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C23)))</formula>
+    <cfRule type="containsText" dxfId="65" priority="1338" operator="containsText" text="ALTO">
+      <formula>NOT(ISERROR(SEARCH("ALTO",C26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="52" priority="1321" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C23)))</formula>
+    <cfRule type="containsText" dxfId="64" priority="1333" operator="containsText" text="BAJA">
+      <formula>NOT(ISERROR(SEARCH("BAJA",C26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="51" priority="1323" operator="containsText" text="SHOWSTOPPER">
-      <formula>NOT(ISERROR(SEARCH("SHOWSTOPPER",C23)))</formula>
+    <cfRule type="containsText" dxfId="63" priority="1335" operator="containsText" text="SHOWSTOPPER">
+      <formula>NOT(ISERROR(SEARCH("SHOWSTOPPER",C26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="50" priority="1324" operator="containsText" text="show">
-      <formula>NOT(ISERROR(SEARCH("show",C23)))</formula>
+    <cfRule type="containsText" dxfId="62" priority="1336" operator="containsText" text="show">
+      <formula>NOT(ISERROR(SEARCH("show",C26)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1 D23:D1048576">
-    <cfRule type="containsText" dxfId="49" priority="1801" operator="containsText" text="EN PROGRESO">
+  <conditionalFormatting sqref="D1 D26:D1048576">
+    <cfRule type="containsText" dxfId="61" priority="1813" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="48" priority="1802" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="60" priority="1814" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="47" priority="1803" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="59" priority="1815" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="46" priority="1804" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="58" priority="1816" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="45" priority="237" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="57" priority="249" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="44" priority="229" operator="containsText" text="NO APLICA">
+    <cfRule type="containsText" dxfId="56" priority="241" operator="containsText" text="NO APLICA">
       <formula>NOT(ISERROR(SEARCH("NO APLICA",D1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="containsText" dxfId="43" priority="1883" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="55" priority="1895" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="42" priority="1762" operator="containsText" text="PENDIENTE">
+    <cfRule type="containsText" dxfId="54" priority="1774" operator="containsText" text="PENDIENTE">
       <formula>NOT(ISERROR(SEARCH("PENDIENTE",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="41" priority="1767" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="53" priority="1779" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="40" priority="1886" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="52" priority="1898" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="39" priority="1887" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="51" priority="1899" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="38" priority="1888" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="50" priority="1900" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="1894" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="1906" stopIfTrue="1" operator="equal">
       <formula>"OPEN"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="1895" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="1907" stopIfTrue="1" operator="equal">
       <formula>"CLOSED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="1896" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="1908" stopIfTrue="1" operator="equal">
       <formula>"IN PROGRESS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D14">
-    <cfRule type="containsText" dxfId="34" priority="35" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="46" priority="47" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D23:D1048576">
-    <cfRule type="containsText" dxfId="33" priority="1530" operator="containsText" text="CERRADO">
-      <formula>NOT(ISERROR(SEARCH("CERRADO",D23)))</formula>
+  <conditionalFormatting sqref="D26:D1048576">
+    <cfRule type="containsText" dxfId="45" priority="1542" operator="containsText" text="CERRADO">
+      <formula>NOT(ISERROR(SEARCH("CERRADO",D26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="32" priority="1327" operator="containsText" text="PENDIENTE">
-      <formula>NOT(ISERROR(SEARCH("PENDIENTE",D23)))</formula>
+    <cfRule type="containsText" dxfId="44" priority="1339" operator="containsText" text="PENDIENTE">
+      <formula>NOT(ISERROR(SEARCH("PENDIENTE",D26)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15">
-    <cfRule type="containsText" dxfId="31" priority="29" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="43" priority="41" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="30" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="42" priority="42" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="29" priority="32" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="41" priority="44" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D15">
-    <cfRule type="containsText" dxfId="28" priority="31" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="40" priority="43" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16">
-    <cfRule type="containsText" dxfId="27" priority="25" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="39" priority="37" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C16)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="26" priority="26" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="38" priority="38" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C16)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="25" priority="28" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="37" priority="40" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C16)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D16">
-    <cfRule type="containsText" dxfId="24" priority="27" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="36" priority="39" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D16)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C17">
-    <cfRule type="containsText" dxfId="23" priority="21" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="35" priority="33" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C17)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="22" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="34" priority="34" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C17)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="24" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="33" priority="36" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C17)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D17">
-    <cfRule type="containsText" dxfId="20" priority="23" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="32" priority="35" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D17)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18">
-    <cfRule type="containsText" dxfId="19" priority="17" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="31" priority="29" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C18)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="18" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="30" priority="30" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C18)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="20" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="29" priority="32" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C18)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18">
-    <cfRule type="containsText" dxfId="16" priority="19" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="28" priority="31" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D18)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19">
-    <cfRule type="containsText" dxfId="15" priority="13" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="27" priority="25" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C19)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="14" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="26" priority="26" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C19)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="16" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="25" priority="28" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C19)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D19">
-    <cfRule type="containsText" dxfId="12" priority="15" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="24" priority="27" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D19)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C20">
-    <cfRule type="containsText" dxfId="11" priority="9" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="23" priority="21" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C20)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="10" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="22" priority="22" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C20)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="12" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="21" priority="24" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D20">
-    <cfRule type="containsText" dxfId="8" priority="11" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="20" priority="23" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C21">
-    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="19" priority="17" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C21)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="6" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="18" priority="18" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C21)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="8" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="17" priority="20" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C21)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D21">
-    <cfRule type="containsText" dxfId="4" priority="7" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="16" priority="19" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D21)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C22">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="15" priority="13" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C22)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="14" priority="14" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C22)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="13" priority="16" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C22)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D22">
+    <cfRule type="containsText" dxfId="12" priority="15" operator="containsText" text="ABIERTO">
+      <formula>NOT(ISERROR(SEARCH("ABIERTO",D22)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C23">
+    <cfRule type="containsText" dxfId="11" priority="9" operator="containsText" text="ALTO">
+      <formula>NOT(ISERROR(SEARCH("ALTO",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="10" operator="containsText" text="MEDIO">
+      <formula>NOT(ISERROR(SEARCH("MEDIO",C23)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="9" priority="12" operator="containsText" text="BAJA">
+      <formula>NOT(ISERROR(SEARCH("BAJA",C23)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D23">
+    <cfRule type="containsText" dxfId="8" priority="11" operator="containsText" text="ABIERTO">
+      <formula>NOT(ISERROR(SEARCH("ABIERTO",D23)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C24">
+    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="ALTO">
+      <formula>NOT(ISERROR(SEARCH("ALTO",C24)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="6" priority="6" operator="containsText" text="MEDIO">
+      <formula>NOT(ISERROR(SEARCH("MEDIO",C24)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="5" priority="8" operator="containsText" text="BAJA">
+      <formula>NOT(ISERROR(SEARCH("BAJA",C24)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D24">
+    <cfRule type="containsText" dxfId="4" priority="7" operator="containsText" text="ABIERTO">
+      <formula>NOT(ISERROR(SEARCH("ABIERTO",D24)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C25">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="ALTO">
+      <formula>NOT(ISERROR(SEARCH("ALTO",C25)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="MEDIO">
+      <formula>NOT(ISERROR(SEARCH("MEDIO",C25)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="BAJA">
+      <formula>NOT(ISERROR(SEARCH("BAJA",C25)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D25">
     <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D22)))</formula>
+      <formula>NOT(ISERROR(SEARCH("ABIERTO",D25)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2318:A1048576 A1:A1215" xr:uid="{00000000-0002-0000-0100-000003000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1 D23:D1048576" xr:uid="{00000000-0002-0000-0100-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1 D26:D1048576" xr:uid="{00000000-0002-0000-0100-000005000000}">
       <formula1>"EN PROGRESO, CERRADO, EN PRUEBA UAT, NO APLICA, ABIERTO, RE-ABIERTO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C22" xr:uid="{2EFE3990-CB5F-4D93-94A6-FF70142F2125}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C25" xr:uid="{2EFE3990-CB5F-4D93-94A6-FF70142F2125}">
       <formula1>"--------, ALTO, MEDIO, SHOWSTOPPER, BAJA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D22" xr:uid="{7C77CF05-9C90-43D6-9300-03C5452EAA1E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D25" xr:uid="{7C77CF05-9C90-43D6-9300-03C5452EAA1E}">
       <formula1>"--------, EN PROGRESO, CERRADO, EN PRUEBA UAT, NO APLICA, ABIERTO, RE-ABIERTO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16507,13 +17507,13 @@
           <x14:formula1>
             <xm:f>CBS!$E$2:$E$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E22</xm:sqref>
+          <xm:sqref>E2:E25</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F53AFC20-979E-4FAF-9E3F-A8EB434FE6B9}">
           <x14:formula1>
             <xm:f>CBS!$D$2:$D$3</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F22</xm:sqref>
+          <xm:sqref>F2:F25</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Update Copia de CheckList_Estatus-001-V.1.5DEV (1).xlsx
</commit_message>
<xml_diff>
--- a/validaciones_Y_ChecklistDeRequerimeintos/Copia de CheckList_Estatus-001-V.1.5DEV (1).xlsx
+++ b/validaciones_Y_ChecklistDeRequerimeintos/Copia de CheckList_Estatus-001-V.1.5DEV (1).xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ITZELPROYECTO\integradoraTeampoderoso\validaciones_Y_ChecklistDeRequerimeintos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\isrra\OneDrive\Documentos\GitHub\integradoraTeampoderoso\validaciones_Y_ChecklistDeRequerimeintos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49B5453A-FA3B-4AEF-8DE9-EB30EFC2F50E}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FCC8488-2147-47FA-BC59-82D1E7450BD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="586" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20640" windowHeight="11040" tabRatio="586" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFECTOS" sheetId="4" r:id="rId1"/>
     <sheet name="CBS" sheetId="6" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DEFECTOS!$A$1:$M$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DEFECTOS!$A$1:$M$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -648,535 +648,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
   </cellStyles>
-  <dxfs count="105">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="7" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="7" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="7" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="7" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="7" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="7" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="7" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="7" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="7" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="7" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="7" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="61">
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -2067,7 +1539,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1047751" y="6232070"/>
+          <a:off x="1074965" y="3605892"/>
           <a:ext cx="3950626" cy="1519246"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3465,22 +2937,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:ATS2317"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15" style="26" customWidth="1"/>
-    <col min="2" max="2" width="100.42578125" style="13" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" style="8" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" style="8" customWidth="1"/>
-    <col min="7" max="7" width="19.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" style="8" customWidth="1"/>
-    <col min="9" max="9" width="20.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="24.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5703125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="23.42578125" style="3" customWidth="1"/>
-    <col min="13" max="13" width="21.42578125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="100.44140625" style="13" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.88671875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="18.44140625" style="8" customWidth="1"/>
+    <col min="7" max="7" width="19.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.44140625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="20.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.5546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="23.44140625" style="3" customWidth="1"/>
+    <col min="13" max="13" width="21.44140625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1215" s="5" customFormat="1" ht="111" customHeight="1">
@@ -3524,7 +2997,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:1215" s="23" customFormat="1" ht="207.6" customHeight="1">
+    <row r="2" spans="1:1215" s="23" customFormat="1" ht="207.6" hidden="1" customHeight="1">
       <c r="A2" s="24" t="s">
         <v>30</v>
       </c>
@@ -4759,7 +4232,7 @@
       <c r="ATR2"/>
       <c r="ATS2"/>
     </row>
-    <row r="3" spans="1:1215" ht="343.5" customHeight="1">
+    <row r="3" spans="1:1215" ht="343.5" hidden="1" customHeight="1">
       <c r="A3" s="24" t="s">
         <v>31</v>
       </c>
@@ -4770,7 +4243,7 @@
         <v>14</v>
       </c>
       <c r="D3" s="34" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" s="29" t="s">
         <v>35</v>
@@ -4982,7 +4455,7 @@
       <c r="HB3" s="15"/>
       <c r="HC3" s="15"/>
     </row>
-    <row r="4" spans="1:1215" ht="217.15" customHeight="1">
+    <row r="4" spans="1:1215" ht="217.2" hidden="1" customHeight="1">
       <c r="A4" s="24" t="s">
         <v>32</v>
       </c>
@@ -4993,7 +4466,7 @@
         <v>14</v>
       </c>
       <c r="D4" s="34" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E4" s="29" t="s">
         <v>35</v>
@@ -5205,7 +4678,7 @@
       <c r="HB4" s="15"/>
       <c r="HC4" s="15"/>
     </row>
-    <row r="5" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="5" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A5" s="24" t="s">
         <v>33</v>
       </c>
@@ -5428,7 +4901,7 @@
       <c r="HB5" s="15"/>
       <c r="HC5" s="15"/>
     </row>
-    <row r="6" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="6" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A6" s="24" t="s">
         <v>33</v>
       </c>
@@ -5651,7 +5124,7 @@
       <c r="HB6" s="15"/>
       <c r="HC6" s="15"/>
     </row>
-    <row r="7" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="7" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A7" s="24" t="s">
         <v>33</v>
       </c>
@@ -5874,7 +5347,7 @@
       <c r="HB7" s="15"/>
       <c r="HC7" s="15"/>
     </row>
-    <row r="8" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="8" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A8" s="24" t="s">
         <v>33</v>
       </c>
@@ -6097,7 +5570,7 @@
       <c r="HB8" s="15"/>
       <c r="HC8" s="15"/>
     </row>
-    <row r="9" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="9" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A9" s="24" t="s">
         <v>33</v>
       </c>
@@ -6320,7 +5793,7 @@
       <c r="HB9" s="15"/>
       <c r="HC9" s="15"/>
     </row>
-    <row r="10" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="10" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A10" s="24" t="s">
         <v>33</v>
       </c>
@@ -6543,7 +6016,7 @@
       <c r="HB10" s="15"/>
       <c r="HC10" s="15"/>
     </row>
-    <row r="11" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="11" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A11" s="24" t="s">
         <v>33</v>
       </c>
@@ -6766,7 +6239,7 @@
       <c r="HB11" s="15"/>
       <c r="HC11" s="15"/>
     </row>
-    <row r="12" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="12" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A12" s="24" t="s">
         <v>33</v>
       </c>
@@ -6989,7 +6462,7 @@
       <c r="HB12" s="15"/>
       <c r="HC12" s="15"/>
     </row>
-    <row r="13" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="13" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A13" s="24" t="s">
         <v>33</v>
       </c>
@@ -7212,7 +6685,7 @@
       <c r="HB13" s="15"/>
       <c r="HC13" s="15"/>
     </row>
-    <row r="14" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="14" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A14" s="24" t="s">
         <v>33</v>
       </c>
@@ -7223,7 +6696,7 @@
         <v>14</v>
       </c>
       <c r="D14" s="34" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E14" s="29" t="s">
         <v>35</v>
@@ -7435,7 +6908,7 @@
       <c r="HB14" s="15"/>
       <c r="HC14" s="15"/>
     </row>
-    <row r="15" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="15" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A15" s="24" t="s">
         <v>33</v>
       </c>
@@ -7446,7 +6919,7 @@
         <v>14</v>
       </c>
       <c r="D15" s="34" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E15" s="29" t="s">
         <v>35</v>
@@ -7658,7 +7131,7 @@
       <c r="HB15" s="15"/>
       <c r="HC15" s="15"/>
     </row>
-    <row r="16" spans="1:1215" ht="277.14999999999998" customHeight="1">
+    <row r="16" spans="1:1215" ht="277.2" hidden="1" customHeight="1">
       <c r="A16" s="24" t="s">
         <v>33</v>
       </c>
@@ -7669,7 +7142,7 @@
         <v>14</v>
       </c>
       <c r="D16" s="34" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E16" s="29" t="s">
         <v>35</v>
@@ -7881,7 +7354,7 @@
       <c r="HB16" s="15"/>
       <c r="HC16" s="15"/>
     </row>
-    <row r="17" spans="1:211" ht="277.14999999999998" customHeight="1">
+    <row r="17" spans="1:211" ht="277.2" hidden="1" customHeight="1">
       <c r="A17" s="24" t="s">
         <v>33</v>
       </c>
@@ -7892,7 +7365,7 @@
         <v>14</v>
       </c>
       <c r="D17" s="34" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E17" s="29" t="s">
         <v>35</v>
@@ -8104,7 +7577,7 @@
       <c r="HB17" s="15"/>
       <c r="HC17" s="15"/>
     </row>
-    <row r="18" spans="1:211" ht="277.14999999999998" customHeight="1">
+    <row r="18" spans="1:211" ht="277.2" customHeight="1">
       <c r="A18" s="24" t="s">
         <v>33</v>
       </c>
@@ -8327,7 +7800,7 @@
       <c r="HB18" s="15"/>
       <c r="HC18" s="15"/>
     </row>
-    <row r="19" spans="1:211" ht="277.14999999999998" customHeight="1">
+    <row r="19" spans="1:211" ht="277.2" customHeight="1">
       <c r="A19" s="24" t="s">
         <v>33</v>
       </c>
@@ -8550,7 +8023,7 @@
       <c r="HB19" s="15"/>
       <c r="HC19" s="15"/>
     </row>
-    <row r="20" spans="1:211" ht="277.14999999999998" customHeight="1">
+    <row r="20" spans="1:211" ht="277.2" customHeight="1">
       <c r="A20" s="24" t="s">
         <v>33</v>
       </c>
@@ -8773,7 +8246,7 @@
       <c r="HB20" s="15"/>
       <c r="HC20" s="15"/>
     </row>
-    <row r="21" spans="1:211" ht="277.14999999999998" customHeight="1">
+    <row r="21" spans="1:211" ht="277.2" customHeight="1">
       <c r="A21" s="24" t="s">
         <v>33</v>
       </c>
@@ -8996,7 +8469,7 @@
       <c r="HB21" s="15"/>
       <c r="HC21" s="15"/>
     </row>
-    <row r="22" spans="1:211" ht="277.14999999999998" customHeight="1">
+    <row r="22" spans="1:211" ht="277.2" customHeight="1">
       <c r="A22" s="24" t="s">
         <v>33</v>
       </c>
@@ -9219,7 +8692,7 @@
       <c r="HB22" s="15"/>
       <c r="HC22" s="15"/>
     </row>
-    <row r="23" spans="1:211" ht="277.14999999999998" customHeight="1">
+    <row r="23" spans="1:211" ht="277.2" customHeight="1">
       <c r="A23" s="24" t="s">
         <v>33</v>
       </c>
@@ -9442,7 +8915,7 @@
       <c r="HB23" s="15"/>
       <c r="HC23" s="15"/>
     </row>
-    <row r="24" spans="1:211" ht="277.14999999999998" customHeight="1">
+    <row r="24" spans="1:211" ht="277.2" hidden="1" customHeight="1">
       <c r="A24" s="24" t="s">
         <v>33</v>
       </c>
@@ -9453,7 +8926,7 @@
         <v>14</v>
       </c>
       <c r="D24" s="34" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E24" s="29" t="s">
         <v>35</v>
@@ -9665,7 +9138,7 @@
       <c r="HB24" s="15"/>
       <c r="HC24" s="15"/>
     </row>
-    <row r="25" spans="1:211" ht="58.5" customHeight="1">
+    <row r="25" spans="1:211" ht="58.5" hidden="1" customHeight="1">
       <c r="A25" s="24" t="s">
         <v>33</v>
       </c>
@@ -9676,7 +9149,7 @@
         <v>14</v>
       </c>
       <c r="D25" s="34" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E25" s="29" t="s">
         <v>35</v>
@@ -15753,1736 +15226,1566 @@
     <row r="1980" spans="1:2">
       <c r="A1980" s="2"/>
     </row>
-    <row r="1981" spans="1:2" ht="12.75">
+    <row r="1981" spans="1:2" ht="13.2">
       <c r="A1981" s="2"/>
       <c r="B1981" s="2"/>
     </row>
-    <row r="1982" spans="1:2" ht="12.75">
+    <row r="1982" spans="1:2" ht="13.2">
       <c r="A1982" s="2"/>
       <c r="B1982" s="2"/>
     </row>
-    <row r="1983" spans="1:2" ht="12.75">
+    <row r="1983" spans="1:2" ht="13.2">
       <c r="A1983" s="2"/>
       <c r="B1983" s="2"/>
     </row>
-    <row r="1984" spans="1:2" ht="12.75">
+    <row r="1984" spans="1:2" ht="13.2">
       <c r="A1984" s="2"/>
       <c r="B1984" s="2"/>
     </row>
-    <row r="1985" spans="1:2" ht="12.75">
+    <row r="1985" spans="1:2" ht="13.2">
       <c r="A1985" s="2"/>
       <c r="B1985" s="2"/>
     </row>
-    <row r="1986" spans="1:2" ht="12.75">
+    <row r="1986" spans="1:2" ht="13.2">
       <c r="A1986" s="2"/>
       <c r="B1986" s="2"/>
     </row>
-    <row r="1987" spans="1:2" ht="12.75">
+    <row r="1987" spans="1:2" ht="13.2">
       <c r="A1987" s="2"/>
       <c r="B1987" s="2"/>
     </row>
-    <row r="1988" spans="1:2" ht="12.75">
+    <row r="1988" spans="1:2" ht="13.2">
       <c r="A1988" s="2"/>
       <c r="B1988" s="2"/>
     </row>
-    <row r="1989" spans="1:2" ht="12.75">
+    <row r="1989" spans="1:2" ht="13.2">
       <c r="A1989" s="2"/>
       <c r="B1989" s="2"/>
     </row>
-    <row r="1990" spans="1:2" ht="12.75">
+    <row r="1990" spans="1:2" ht="13.2">
       <c r="A1990" s="2"/>
       <c r="B1990" s="2"/>
     </row>
-    <row r="1991" spans="1:2" ht="12.75">
+    <row r="1991" spans="1:2" ht="13.2">
       <c r="A1991" s="2"/>
       <c r="B1991" s="2"/>
     </row>
-    <row r="1992" spans="1:2" ht="12.75">
+    <row r="1992" spans="1:2" ht="13.2">
       <c r="A1992" s="2"/>
       <c r="B1992" s="2"/>
     </row>
-    <row r="1993" spans="1:2" ht="12.75">
+    <row r="1993" spans="1:2" ht="13.2">
       <c r="A1993" s="2"/>
       <c r="B1993" s="2"/>
     </row>
-    <row r="1994" spans="1:2" ht="12.75">
+    <row r="1994" spans="1:2" ht="13.2">
       <c r="A1994" s="2"/>
       <c r="B1994" s="2"/>
     </row>
-    <row r="1995" spans="1:2" ht="12.75">
+    <row r="1995" spans="1:2" ht="13.2">
       <c r="A1995" s="2"/>
       <c r="B1995" s="2"/>
     </row>
-    <row r="1996" spans="1:2" ht="12.75">
+    <row r="1996" spans="1:2" ht="13.2">
       <c r="A1996" s="2"/>
       <c r="B1996" s="2"/>
     </row>
-    <row r="1997" spans="1:2" ht="12.75">
+    <row r="1997" spans="1:2" ht="13.2">
       <c r="A1997" s="2"/>
       <c r="B1997" s="2"/>
     </row>
-    <row r="1998" spans="1:2" ht="12.75">
+    <row r="1998" spans="1:2" ht="13.2">
       <c r="A1998" s="2"/>
       <c r="B1998" s="2"/>
     </row>
-    <row r="1999" spans="1:2" ht="12.75">
+    <row r="1999" spans="1:2" ht="13.2">
       <c r="A1999" s="2"/>
       <c r="B1999" s="2"/>
     </row>
-    <row r="2000" spans="1:2" ht="12.75">
+    <row r="2000" spans="1:2" ht="13.2">
       <c r="A2000" s="2"/>
       <c r="B2000" s="2"/>
     </row>
-    <row r="2001" spans="1:2" ht="12.75">
+    <row r="2001" spans="1:2" ht="13.2">
       <c r="A2001" s="2"/>
       <c r="B2001" s="2"/>
     </row>
-    <row r="2002" spans="1:2" ht="12.75">
+    <row r="2002" spans="1:2" ht="13.2">
       <c r="A2002" s="2"/>
       <c r="B2002" s="2"/>
     </row>
-    <row r="2003" spans="1:2" ht="12.75">
+    <row r="2003" spans="1:2" ht="13.2">
       <c r="A2003" s="2"/>
       <c r="B2003" s="2"/>
     </row>
-    <row r="2004" spans="1:2" ht="12.75">
+    <row r="2004" spans="1:2" ht="13.2">
       <c r="A2004" s="2"/>
       <c r="B2004" s="2"/>
     </row>
-    <row r="2005" spans="1:2" ht="12.75">
+    <row r="2005" spans="1:2" ht="13.2">
       <c r="A2005" s="2"/>
       <c r="B2005" s="2"/>
     </row>
-    <row r="2006" spans="1:2" ht="12.75">
+    <row r="2006" spans="1:2" ht="13.2">
       <c r="A2006" s="2"/>
       <c r="B2006" s="2"/>
     </row>
-    <row r="2007" spans="1:2" ht="12.75">
+    <row r="2007" spans="1:2" ht="13.2">
       <c r="A2007" s="2"/>
       <c r="B2007" s="2"/>
     </row>
-    <row r="2008" spans="1:2" ht="12.75">
+    <row r="2008" spans="1:2" ht="13.2">
       <c r="A2008" s="2"/>
       <c r="B2008" s="2"/>
     </row>
-    <row r="2009" spans="1:2" ht="12.75">
+    <row r="2009" spans="1:2" ht="13.2">
       <c r="A2009" s="2"/>
       <c r="B2009" s="2"/>
     </row>
-    <row r="2010" spans="1:2" ht="12.75">
+    <row r="2010" spans="1:2" ht="13.2">
       <c r="A2010" s="2"/>
       <c r="B2010" s="2"/>
     </row>
-    <row r="2011" spans="1:2" ht="12.75">
+    <row r="2011" spans="1:2" ht="13.2">
       <c r="A2011" s="2"/>
       <c r="B2011" s="2"/>
     </row>
-    <row r="2012" spans="1:2" ht="12.75">
+    <row r="2012" spans="1:2" ht="13.2">
       <c r="A2012" s="2"/>
       <c r="B2012" s="2"/>
     </row>
-    <row r="2013" spans="1:2" ht="12.75">
+    <row r="2013" spans="1:2" ht="13.2">
       <c r="A2013" s="2"/>
       <c r="B2013" s="2"/>
     </row>
-    <row r="2014" spans="1:2" ht="12.75">
+    <row r="2014" spans="1:2" ht="13.2">
       <c r="A2014" s="2"/>
       <c r="B2014" s="2"/>
     </row>
-    <row r="2015" spans="1:2" ht="12.75">
+    <row r="2015" spans="1:2" ht="13.2">
       <c r="A2015" s="2"/>
       <c r="B2015" s="2"/>
     </row>
-    <row r="2016" spans="1:2" ht="12.75">
+    <row r="2016" spans="1:2" ht="13.2">
       <c r="A2016" s="2"/>
       <c r="B2016" s="2"/>
     </row>
-    <row r="2017" spans="1:2" ht="12.75">
+    <row r="2017" spans="1:2" ht="13.2">
       <c r="A2017" s="2"/>
       <c r="B2017" s="2"/>
     </row>
-    <row r="2018" spans="1:2" ht="12.75">
+    <row r="2018" spans="1:2" ht="13.2">
       <c r="A2018" s="2"/>
       <c r="B2018" s="2"/>
     </row>
-    <row r="2019" spans="1:2" ht="12.75">
+    <row r="2019" spans="1:2" ht="13.2">
       <c r="A2019" s="2"/>
       <c r="B2019" s="2"/>
     </row>
-    <row r="2020" spans="1:2" ht="12.75">
+    <row r="2020" spans="1:2" ht="13.2">
       <c r="A2020" s="2"/>
       <c r="B2020" s="2"/>
     </row>
-    <row r="2021" spans="1:2" ht="12.75">
+    <row r="2021" spans="1:2" ht="13.2">
       <c r="A2021" s="2"/>
       <c r="B2021" s="2"/>
     </row>
-    <row r="2022" spans="1:2" ht="12.75">
+    <row r="2022" spans="1:2" ht="13.2">
       <c r="A2022" s="2"/>
       <c r="B2022" s="2"/>
     </row>
-    <row r="2023" spans="1:2" ht="12.75">
+    <row r="2023" spans="1:2" ht="13.2">
       <c r="A2023" s="2"/>
       <c r="B2023" s="2"/>
     </row>
-    <row r="2024" spans="1:2" ht="12.75">
+    <row r="2024" spans="1:2" ht="13.2">
       <c r="A2024" s="2"/>
       <c r="B2024" s="2"/>
     </row>
-    <row r="2025" spans="1:2" ht="12.75">
+    <row r="2025" spans="1:2" ht="13.2">
       <c r="A2025" s="2"/>
       <c r="B2025" s="2"/>
     </row>
-    <row r="2026" spans="1:2" ht="12.75">
+    <row r="2026" spans="1:2" ht="13.2">
       <c r="A2026" s="2"/>
       <c r="B2026" s="2"/>
     </row>
-    <row r="2027" spans="1:2" ht="12.75">
+    <row r="2027" spans="1:2" ht="13.2">
       <c r="A2027" s="2"/>
       <c r="B2027" s="2"/>
     </row>
-    <row r="2028" spans="1:2" ht="12.75">
+    <row r="2028" spans="1:2" ht="13.2">
       <c r="A2028" s="2"/>
       <c r="B2028" s="2"/>
     </row>
-    <row r="2029" spans="1:2" ht="12.75">
+    <row r="2029" spans="1:2" ht="13.2">
       <c r="A2029" s="2"/>
       <c r="B2029" s="2"/>
     </row>
-    <row r="2030" spans="1:2" ht="12.75">
+    <row r="2030" spans="1:2" ht="13.2">
       <c r="A2030" s="2"/>
       <c r="B2030" s="2"/>
     </row>
-    <row r="2031" spans="1:2" ht="12.75">
+    <row r="2031" spans="1:2" ht="13.2">
       <c r="A2031" s="2"/>
       <c r="B2031" s="2"/>
     </row>
-    <row r="2032" spans="1:2" ht="12.75">
+    <row r="2032" spans="1:2" ht="13.2">
       <c r="A2032" s="2"/>
       <c r="B2032" s="2"/>
     </row>
-    <row r="2033" spans="1:2" ht="12.75">
+    <row r="2033" spans="1:2" ht="13.2">
       <c r="A2033" s="2"/>
       <c r="B2033" s="2"/>
     </row>
-    <row r="2034" spans="1:2" ht="12.75">
+    <row r="2034" spans="1:2" ht="13.2">
       <c r="A2034" s="2"/>
       <c r="B2034" s="2"/>
     </row>
-    <row r="2035" spans="1:2" ht="12.75">
+    <row r="2035" spans="1:2" ht="13.2">
       <c r="A2035" s="2"/>
       <c r="B2035" s="2"/>
     </row>
-    <row r="2036" spans="1:2" ht="12.75">
+    <row r="2036" spans="1:2" ht="13.2">
       <c r="A2036" s="2"/>
       <c r="B2036" s="2"/>
     </row>
-    <row r="2037" spans="1:2" ht="12.75">
+    <row r="2037" spans="1:2" ht="13.2">
       <c r="A2037" s="2"/>
       <c r="B2037" s="2"/>
     </row>
-    <row r="2038" spans="1:2" ht="12.75">
+    <row r="2038" spans="1:2" ht="13.2">
       <c r="A2038" s="2"/>
       <c r="B2038" s="2"/>
     </row>
-    <row r="2039" spans="1:2" ht="12.75">
+    <row r="2039" spans="1:2" ht="13.2">
       <c r="A2039" s="2"/>
       <c r="B2039" s="2"/>
     </row>
-    <row r="2040" spans="1:2" ht="12.75">
+    <row r="2040" spans="1:2" ht="13.2">
       <c r="A2040" s="2"/>
       <c r="B2040" s="2"/>
     </row>
-    <row r="2041" spans="1:2" ht="12.75">
+    <row r="2041" spans="1:2" ht="13.2">
       <c r="A2041" s="2"/>
       <c r="B2041" s="2"/>
     </row>
-    <row r="2042" spans="1:2" ht="12.75">
+    <row r="2042" spans="1:2" ht="13.2">
       <c r="A2042" s="2"/>
       <c r="B2042" s="2"/>
     </row>
-    <row r="2043" spans="1:2" ht="12.75">
+    <row r="2043" spans="1:2" ht="13.2">
       <c r="A2043" s="2"/>
       <c r="B2043" s="2"/>
     </row>
-    <row r="2044" spans="1:2" ht="12.75">
+    <row r="2044" spans="1:2" ht="13.2">
       <c r="A2044" s="2"/>
       <c r="B2044" s="2"/>
     </row>
-    <row r="2045" spans="1:2" ht="12.75">
+    <row r="2045" spans="1:2" ht="13.2">
       <c r="A2045" s="2"/>
       <c r="B2045" s="2"/>
     </row>
-    <row r="2046" spans="1:2" ht="12.75">
+    <row r="2046" spans="1:2" ht="13.2">
       <c r="A2046" s="2"/>
       <c r="B2046" s="2"/>
     </row>
-    <row r="2047" spans="1:2" ht="12.75">
+    <row r="2047" spans="1:2" ht="13.2">
       <c r="A2047" s="2"/>
       <c r="B2047" s="2"/>
     </row>
-    <row r="2048" spans="1:2" ht="12.75">
+    <row r="2048" spans="1:2" ht="13.2">
       <c r="A2048" s="2"/>
       <c r="B2048" s="2"/>
     </row>
-    <row r="2049" spans="1:2" ht="12.75">
+    <row r="2049" spans="1:2" ht="13.2">
       <c r="A2049" s="2"/>
       <c r="B2049" s="2"/>
     </row>
-    <row r="2050" spans="1:2" ht="12.75">
+    <row r="2050" spans="1:2" ht="13.2">
       <c r="A2050" s="2"/>
       <c r="B2050" s="2"/>
     </row>
-    <row r="2051" spans="1:2" ht="12.75">
+    <row r="2051" spans="1:2" ht="13.2">
       <c r="A2051" s="2"/>
       <c r="B2051" s="2"/>
     </row>
-    <row r="2052" spans="1:2" ht="12.75">
+    <row r="2052" spans="1:2" ht="13.2">
       <c r="A2052" s="2"/>
       <c r="B2052" s="2"/>
     </row>
-    <row r="2053" spans="1:2" ht="12.75">
+    <row r="2053" spans="1:2" ht="13.2">
       <c r="A2053" s="2"/>
       <c r="B2053" s="2"/>
     </row>
-    <row r="2054" spans="1:2" ht="12.75">
+    <row r="2054" spans="1:2" ht="13.2">
       <c r="A2054" s="2"/>
       <c r="B2054" s="2"/>
     </row>
-    <row r="2055" spans="1:2" ht="12.75">
+    <row r="2055" spans="1:2" ht="13.2">
       <c r="A2055" s="2"/>
       <c r="B2055" s="2"/>
     </row>
-    <row r="2056" spans="1:2" ht="12.75">
+    <row r="2056" spans="1:2" ht="13.2">
       <c r="A2056" s="2"/>
       <c r="B2056" s="2"/>
     </row>
-    <row r="2057" spans="1:2" ht="12.75">
+    <row r="2057" spans="1:2" ht="13.2">
       <c r="A2057" s="2"/>
       <c r="B2057" s="2"/>
     </row>
-    <row r="2058" spans="1:2" ht="12.75">
+    <row r="2058" spans="1:2" ht="13.2">
       <c r="A2058" s="2"/>
       <c r="B2058" s="2"/>
     </row>
-    <row r="2059" spans="1:2" ht="12.75">
+    <row r="2059" spans="1:2" ht="13.2">
       <c r="A2059" s="2"/>
       <c r="B2059" s="2"/>
     </row>
-    <row r="2060" spans="1:2" ht="12.75">
+    <row r="2060" spans="1:2" ht="13.2">
       <c r="A2060" s="2"/>
       <c r="B2060" s="2"/>
     </row>
-    <row r="2061" spans="1:2" ht="12.75">
+    <row r="2061" spans="1:2" ht="13.2">
       <c r="A2061" s="2"/>
       <c r="B2061" s="2"/>
     </row>
-    <row r="2062" spans="1:2" ht="12.75">
+    <row r="2062" spans="1:2" ht="13.2">
       <c r="A2062" s="2"/>
       <c r="B2062" s="2"/>
     </row>
-    <row r="2063" spans="1:2" ht="12.75">
+    <row r="2063" spans="1:2" ht="13.2">
       <c r="A2063" s="2"/>
       <c r="B2063" s="2"/>
     </row>
-    <row r="2064" spans="1:2" ht="12.75">
+    <row r="2064" spans="1:2" ht="13.2">
       <c r="A2064" s="2"/>
       <c r="B2064" s="2"/>
     </row>
-    <row r="2065" spans="1:2" ht="12.75">
+    <row r="2065" spans="1:2" ht="13.2">
       <c r="A2065" s="2"/>
       <c r="B2065" s="2"/>
     </row>
-    <row r="2066" spans="1:2" ht="12.75">
+    <row r="2066" spans="1:2" ht="13.2">
       <c r="A2066" s="2"/>
       <c r="B2066" s="2"/>
     </row>
-    <row r="2067" spans="1:2" ht="12.75">
+    <row r="2067" spans="1:2" ht="13.2">
       <c r="A2067" s="2"/>
       <c r="B2067" s="2"/>
     </row>
-    <row r="2068" spans="1:2" ht="12.75">
+    <row r="2068" spans="1:2" ht="13.2">
       <c r="A2068" s="2"/>
       <c r="B2068" s="2"/>
     </row>
-    <row r="2069" spans="1:2" ht="12.75">
+    <row r="2069" spans="1:2" ht="13.2">
       <c r="A2069" s="2"/>
       <c r="B2069" s="2"/>
     </row>
-    <row r="2070" spans="1:2" ht="12.75">
+    <row r="2070" spans="1:2" ht="13.2">
       <c r="A2070" s="2"/>
       <c r="B2070" s="2"/>
     </row>
-    <row r="2071" spans="1:2" ht="12.75">
+    <row r="2071" spans="1:2" ht="13.2">
       <c r="A2071" s="2"/>
       <c r="B2071" s="2"/>
     </row>
-    <row r="2072" spans="1:2" ht="12.75">
+    <row r="2072" spans="1:2" ht="13.2">
       <c r="A2072" s="2"/>
       <c r="B2072" s="2"/>
     </row>
-    <row r="2073" spans="1:2" ht="12.75">
+    <row r="2073" spans="1:2" ht="13.2">
       <c r="A2073" s="2"/>
       <c r="B2073" s="2"/>
     </row>
-    <row r="2074" spans="1:2" ht="12.75">
+    <row r="2074" spans="1:2" ht="13.2">
       <c r="A2074" s="2"/>
       <c r="B2074" s="2"/>
     </row>
-    <row r="2075" spans="1:2" ht="12.75">
+    <row r="2075" spans="1:2" ht="13.2">
       <c r="A2075" s="2"/>
       <c r="B2075" s="2"/>
     </row>
-    <row r="2076" spans="1:2" ht="12.75">
+    <row r="2076" spans="1:2" ht="13.2">
       <c r="A2076" s="2"/>
       <c r="B2076" s="2"/>
     </row>
-    <row r="2077" spans="1:2" ht="12.75">
+    <row r="2077" spans="1:2" ht="13.2">
       <c r="A2077" s="2"/>
       <c r="B2077" s="2"/>
     </row>
-    <row r="2078" spans="1:2" ht="12.75">
+    <row r="2078" spans="1:2" ht="13.2">
       <c r="A2078" s="2"/>
       <c r="B2078" s="2"/>
     </row>
-    <row r="2079" spans="1:2" ht="12.75">
+    <row r="2079" spans="1:2" ht="13.2">
       <c r="A2079" s="2"/>
       <c r="B2079" s="2"/>
     </row>
-    <row r="2080" spans="1:2" ht="12.75">
+    <row r="2080" spans="1:2" ht="13.2">
       <c r="A2080" s="2"/>
       <c r="B2080" s="2"/>
     </row>
-    <row r="2081" spans="1:2" ht="12.75">
+    <row r="2081" spans="1:2" ht="13.2">
       <c r="A2081" s="2"/>
       <c r="B2081" s="2"/>
     </row>
-    <row r="2082" spans="1:2" ht="12.75">
+    <row r="2082" spans="1:2" ht="13.2">
       <c r="A2082" s="2"/>
       <c r="B2082" s="2"/>
     </row>
-    <row r="2083" spans="1:2" ht="12.75">
+    <row r="2083" spans="1:2" ht="13.2">
       <c r="A2083" s="2"/>
       <c r="B2083" s="2"/>
     </row>
-    <row r="2084" spans="1:2" ht="12.75">
+    <row r="2084" spans="1:2" ht="13.2">
       <c r="A2084" s="2"/>
       <c r="B2084" s="2"/>
     </row>
-    <row r="2085" spans="1:2" ht="12.75">
+    <row r="2085" spans="1:2" ht="13.2">
       <c r="A2085" s="2"/>
       <c r="B2085" s="2"/>
     </row>
-    <row r="2086" spans="1:2" ht="12.75">
+    <row r="2086" spans="1:2" ht="13.2">
       <c r="A2086" s="2"/>
       <c r="B2086" s="2"/>
     </row>
-    <row r="2087" spans="1:2" ht="12.75">
+    <row r="2087" spans="1:2" ht="13.2">
       <c r="A2087" s="2"/>
       <c r="B2087" s="2"/>
     </row>
-    <row r="2088" spans="1:2" ht="12.75">
+    <row r="2088" spans="1:2" ht="13.2">
       <c r="A2088" s="2"/>
       <c r="B2088" s="2"/>
     </row>
-    <row r="2089" spans="1:2" ht="12.75">
+    <row r="2089" spans="1:2" ht="13.2">
       <c r="A2089" s="2"/>
       <c r="B2089" s="2"/>
     </row>
-    <row r="2090" spans="1:2" ht="12.75">
+    <row r="2090" spans="1:2" ht="13.2">
       <c r="A2090" s="2"/>
       <c r="B2090" s="2"/>
     </row>
-    <row r="2091" spans="1:2" ht="12.75">
+    <row r="2091" spans="1:2" ht="13.2">
       <c r="A2091" s="2"/>
       <c r="B2091" s="2"/>
     </row>
-    <row r="2092" spans="1:2" ht="12.75">
+    <row r="2092" spans="1:2" ht="13.2">
       <c r="A2092" s="2"/>
       <c r="B2092" s="2"/>
     </row>
-    <row r="2093" spans="1:2" ht="12.75">
+    <row r="2093" spans="1:2" ht="13.2">
       <c r="A2093" s="2"/>
       <c r="B2093" s="2"/>
     </row>
-    <row r="2094" spans="1:2" ht="12.75">
+    <row r="2094" spans="1:2" ht="13.2">
       <c r="A2094" s="2"/>
       <c r="B2094" s="2"/>
     </row>
-    <row r="2095" spans="1:2" ht="12.75">
+    <row r="2095" spans="1:2" ht="13.2">
       <c r="A2095" s="2"/>
       <c r="B2095" s="2"/>
     </row>
-    <row r="2096" spans="1:2" ht="12.75">
+    <row r="2096" spans="1:2" ht="13.2">
       <c r="A2096" s="2"/>
       <c r="B2096" s="2"/>
     </row>
-    <row r="2097" spans="1:2" ht="12.75">
+    <row r="2097" spans="1:2" ht="13.2">
       <c r="A2097" s="2"/>
       <c r="B2097" s="2"/>
     </row>
-    <row r="2098" spans="1:2" ht="12.75">
+    <row r="2098" spans="1:2" ht="13.2">
       <c r="A2098" s="2"/>
       <c r="B2098" s="2"/>
     </row>
-    <row r="2099" spans="1:2" ht="12.75">
+    <row r="2099" spans="1:2" ht="13.2">
       <c r="A2099" s="2"/>
       <c r="B2099" s="2"/>
     </row>
-    <row r="2100" spans="1:2" ht="12.75">
+    <row r="2100" spans="1:2" ht="13.2">
       <c r="A2100" s="2"/>
       <c r="B2100" s="2"/>
     </row>
-    <row r="2101" spans="1:2" ht="12.75">
+    <row r="2101" spans="1:2" ht="13.2">
       <c r="A2101" s="2"/>
       <c r="B2101" s="2"/>
     </row>
-    <row r="2102" spans="1:2" ht="12.75">
+    <row r="2102" spans="1:2" ht="13.2">
       <c r="A2102" s="2"/>
       <c r="B2102" s="2"/>
     </row>
-    <row r="2103" spans="1:2" ht="12.75">
+    <row r="2103" spans="1:2" ht="13.2">
       <c r="A2103" s="2"/>
       <c r="B2103" s="2"/>
     </row>
-    <row r="2104" spans="1:2" ht="12.75">
+    <row r="2104" spans="1:2" ht="13.2">
       <c r="A2104" s="2"/>
       <c r="B2104" s="2"/>
     </row>
-    <row r="2105" spans="1:2" ht="12.75">
+    <row r="2105" spans="1:2" ht="13.2">
       <c r="A2105" s="2"/>
       <c r="B2105" s="2"/>
     </row>
-    <row r="2106" spans="1:2" ht="12.75">
+    <row r="2106" spans="1:2" ht="13.2">
       <c r="A2106" s="2"/>
       <c r="B2106" s="2"/>
     </row>
-    <row r="2107" spans="1:2" ht="12.75">
+    <row r="2107" spans="1:2" ht="13.2">
       <c r="A2107" s="2"/>
       <c r="B2107" s="2"/>
     </row>
-    <row r="2108" spans="1:2" ht="12.75">
+    <row r="2108" spans="1:2" ht="13.2">
       <c r="A2108" s="2"/>
       <c r="B2108" s="2"/>
     </row>
-    <row r="2109" spans="1:2" ht="12.75">
+    <row r="2109" spans="1:2" ht="13.2">
       <c r="A2109" s="2"/>
       <c r="B2109" s="2"/>
     </row>
-    <row r="2110" spans="1:2" ht="12.75">
+    <row r="2110" spans="1:2" ht="13.2">
       <c r="A2110" s="2"/>
       <c r="B2110" s="2"/>
     </row>
-    <row r="2111" spans="1:2" ht="12.75">
+    <row r="2111" spans="1:2" ht="13.2">
       <c r="A2111" s="2"/>
       <c r="B2111" s="2"/>
     </row>
-    <row r="2112" spans="1:2" ht="12.75">
+    <row r="2112" spans="1:2" ht="13.2">
       <c r="A2112" s="2"/>
       <c r="B2112" s="2"/>
     </row>
-    <row r="2113" spans="1:2" ht="12.75">
+    <row r="2113" spans="1:2" ht="13.2">
       <c r="A2113" s="2"/>
       <c r="B2113" s="2"/>
     </row>
-    <row r="2114" spans="1:2" ht="12.75">
+    <row r="2114" spans="1:2" ht="13.2">
       <c r="A2114" s="2"/>
       <c r="B2114" s="2"/>
     </row>
-    <row r="2115" spans="1:2" ht="12.75">
+    <row r="2115" spans="1:2" ht="13.2">
       <c r="A2115" s="2"/>
       <c r="B2115" s="2"/>
     </row>
-    <row r="2116" spans="1:2" ht="12.75">
+    <row r="2116" spans="1:2" ht="13.2">
       <c r="A2116" s="2"/>
       <c r="B2116" s="2"/>
     </row>
-    <row r="2117" spans="1:2" ht="12.75">
+    <row r="2117" spans="1:2" ht="13.2">
       <c r="A2117" s="2"/>
       <c r="B2117" s="2"/>
     </row>
-    <row r="2118" spans="1:2" ht="12.75">
+    <row r="2118" spans="1:2" ht="13.2">
       <c r="A2118" s="2"/>
       <c r="B2118" s="2"/>
     </row>
-    <row r="2119" spans="1:2" ht="12.75">
+    <row r="2119" spans="1:2" ht="13.2">
       <c r="A2119" s="2"/>
       <c r="B2119" s="2"/>
     </row>
-    <row r="2120" spans="1:2" ht="12.75">
+    <row r="2120" spans="1:2" ht="13.2">
       <c r="A2120" s="2"/>
       <c r="B2120" s="2"/>
     </row>
-    <row r="2121" spans="1:2" ht="12.75">
+    <row r="2121" spans="1:2" ht="13.2">
       <c r="A2121" s="2"/>
       <c r="B2121" s="2"/>
     </row>
-    <row r="2122" spans="1:2" ht="12.75">
+    <row r="2122" spans="1:2" ht="13.2">
       <c r="A2122" s="2"/>
       <c r="B2122" s="2"/>
     </row>
-    <row r="2123" spans="1:2" ht="12.75">
+    <row r="2123" spans="1:2" ht="13.2">
       <c r="A2123" s="2"/>
       <c r="B2123" s="2"/>
     </row>
-    <row r="2124" spans="1:2" ht="12.75">
+    <row r="2124" spans="1:2" ht="13.2">
       <c r="A2124" s="2"/>
       <c r="B2124" s="2"/>
     </row>
-    <row r="2125" spans="1:2" ht="12.75">
+    <row r="2125" spans="1:2" ht="13.2">
       <c r="A2125" s="2"/>
       <c r="B2125" s="2"/>
     </row>
-    <row r="2126" spans="1:2" ht="12.75">
+    <row r="2126" spans="1:2" ht="13.2">
       <c r="A2126" s="2"/>
       <c r="B2126" s="2"/>
     </row>
-    <row r="2127" spans="1:2" ht="12.75">
+    <row r="2127" spans="1:2" ht="13.2">
       <c r="A2127" s="2"/>
       <c r="B2127" s="2"/>
     </row>
-    <row r="2128" spans="1:2" ht="12.75">
+    <row r="2128" spans="1:2" ht="13.2">
       <c r="A2128" s="2"/>
       <c r="B2128" s="2"/>
     </row>
-    <row r="2129" spans="1:2" ht="12.75">
+    <row r="2129" spans="1:2" ht="13.2">
       <c r="A2129" s="2"/>
       <c r="B2129" s="2"/>
     </row>
-    <row r="2130" spans="1:2" ht="12.75">
+    <row r="2130" spans="1:2" ht="13.2">
       <c r="A2130" s="2"/>
       <c r="B2130" s="2"/>
     </row>
-    <row r="2131" spans="1:2" ht="12.75">
+    <row r="2131" spans="1:2" ht="13.2">
       <c r="A2131" s="2"/>
       <c r="B2131" s="2"/>
     </row>
-    <row r="2132" spans="1:2" ht="12.75">
+    <row r="2132" spans="1:2" ht="13.2">
       <c r="A2132" s="2"/>
       <c r="B2132" s="2"/>
     </row>
-    <row r="2133" spans="1:2" ht="12.75">
+    <row r="2133" spans="1:2" ht="13.2">
       <c r="A2133" s="2"/>
       <c r="B2133" s="2"/>
     </row>
-    <row r="2134" spans="1:2" ht="12.75">
+    <row r="2134" spans="1:2" ht="13.2">
       <c r="A2134" s="2"/>
       <c r="B2134" s="2"/>
     </row>
-    <row r="2135" spans="1:2" ht="12.75">
+    <row r="2135" spans="1:2" ht="13.2">
       <c r="A2135" s="2"/>
       <c r="B2135" s="2"/>
     </row>
-    <row r="2136" spans="1:2" ht="12.75">
+    <row r="2136" spans="1:2" ht="13.2">
       <c r="A2136" s="2"/>
       <c r="B2136" s="2"/>
     </row>
-    <row r="2137" spans="1:2" ht="12.75">
+    <row r="2137" spans="1:2" ht="13.2">
       <c r="A2137" s="2"/>
       <c r="B2137" s="2"/>
     </row>
-    <row r="2138" spans="1:2" ht="12.75">
+    <row r="2138" spans="1:2" ht="13.2">
       <c r="A2138" s="2"/>
       <c r="B2138" s="2"/>
     </row>
-    <row r="2139" spans="1:2" ht="12.75">
+    <row r="2139" spans="1:2" ht="13.2">
       <c r="A2139" s="2"/>
       <c r="B2139" s="2"/>
     </row>
-    <row r="2140" spans="1:2" ht="12.75">
+    <row r="2140" spans="1:2" ht="13.2">
       <c r="A2140" s="2"/>
       <c r="B2140" s="2"/>
     </row>
-    <row r="2141" spans="1:2" ht="12.75">
+    <row r="2141" spans="1:2" ht="13.2">
       <c r="A2141" s="2"/>
       <c r="B2141" s="2"/>
     </row>
-    <row r="2142" spans="1:2" ht="12.75">
+    <row r="2142" spans="1:2" ht="13.2">
       <c r="A2142" s="2"/>
       <c r="B2142" s="2"/>
     </row>
-    <row r="2143" spans="1:2" ht="12.75">
+    <row r="2143" spans="1:2" ht="13.2">
       <c r="A2143" s="2"/>
       <c r="B2143" s="2"/>
     </row>
-    <row r="2144" spans="1:2" ht="12.75">
+    <row r="2144" spans="1:2" ht="13.2">
       <c r="A2144" s="2"/>
       <c r="B2144" s="2"/>
     </row>
-    <row r="2145" spans="1:2" ht="12.75">
+    <row r="2145" spans="1:2" ht="13.2">
       <c r="A2145" s="2"/>
       <c r="B2145" s="2"/>
     </row>
-    <row r="2146" spans="1:2" ht="12.75">
+    <row r="2146" spans="1:2" ht="13.2">
       <c r="A2146" s="2"/>
       <c r="B2146" s="2"/>
     </row>
-    <row r="2147" spans="1:2" ht="12.75">
+    <row r="2147" spans="1:2" ht="13.2">
       <c r="A2147" s="2"/>
       <c r="B2147" s="2"/>
     </row>
-    <row r="2148" spans="1:2" ht="12.75">
+    <row r="2148" spans="1:2" ht="13.2">
       <c r="A2148" s="2"/>
       <c r="B2148" s="2"/>
     </row>
-    <row r="2149" spans="1:2" ht="12.75">
+    <row r="2149" spans="1:2" ht="13.2">
       <c r="A2149" s="2"/>
       <c r="B2149" s="2"/>
     </row>
-    <row r="2150" spans="1:2" ht="12.75">
+    <row r="2150" spans="1:2" ht="13.2">
       <c r="A2150" s="2"/>
       <c r="B2150" s="2"/>
     </row>
-    <row r="2151" spans="1:2" ht="12.75">
+    <row r="2151" spans="1:2" ht="13.2">
       <c r="A2151" s="2"/>
       <c r="B2151" s="2"/>
     </row>
-    <row r="2152" spans="1:2" ht="12.75">
+    <row r="2152" spans="1:2" ht="13.2">
       <c r="A2152" s="2"/>
       <c r="B2152" s="2"/>
     </row>
-    <row r="2153" spans="1:2" ht="12.75">
+    <row r="2153" spans="1:2" ht="13.2">
       <c r="A2153" s="2"/>
       <c r="B2153" s="2"/>
     </row>
-    <row r="2154" spans="1:2" ht="12.75">
+    <row r="2154" spans="1:2" ht="13.2">
       <c r="A2154" s="2"/>
       <c r="B2154" s="2"/>
     </row>
-    <row r="2155" spans="1:2" ht="12.75">
+    <row r="2155" spans="1:2" ht="13.2">
       <c r="A2155" s="2"/>
       <c r="B2155" s="2"/>
     </row>
-    <row r="2156" spans="1:2" ht="12.75">
+    <row r="2156" spans="1:2" ht="13.2">
       <c r="A2156" s="2"/>
       <c r="B2156" s="2"/>
     </row>
-    <row r="2157" spans="1:2" ht="12.75">
+    <row r="2157" spans="1:2" ht="13.2">
       <c r="A2157" s="2"/>
       <c r="B2157" s="2"/>
     </row>
-    <row r="2158" spans="1:2" ht="12.75">
+    <row r="2158" spans="1:2" ht="13.2">
       <c r="A2158" s="2"/>
       <c r="B2158" s="2"/>
     </row>
-    <row r="2159" spans="1:2" ht="12.75">
+    <row r="2159" spans="1:2" ht="13.2">
       <c r="A2159" s="2"/>
       <c r="B2159" s="2"/>
     </row>
-    <row r="2160" spans="1:2" ht="12.75">
+    <row r="2160" spans="1:2" ht="13.2">
       <c r="A2160" s="2"/>
       <c r="B2160" s="2"/>
     </row>
-    <row r="2161" spans="1:2" ht="12.75">
+    <row r="2161" spans="1:2" ht="13.2">
       <c r="A2161" s="2"/>
       <c r="B2161" s="2"/>
     </row>
-    <row r="2162" spans="1:2" ht="12.75">
+    <row r="2162" spans="1:2" ht="13.2">
       <c r="A2162" s="2"/>
       <c r="B2162" s="2"/>
     </row>
-    <row r="2163" spans="1:2" ht="12.75">
+    <row r="2163" spans="1:2" ht="13.2">
       <c r="A2163" s="2"/>
       <c r="B2163" s="2"/>
     </row>
-    <row r="2164" spans="1:2" ht="12.75">
+    <row r="2164" spans="1:2" ht="13.2">
       <c r="A2164" s="2"/>
       <c r="B2164" s="2"/>
     </row>
-    <row r="2165" spans="1:2" ht="12.75">
+    <row r="2165" spans="1:2" ht="13.2">
       <c r="A2165" s="2"/>
       <c r="B2165" s="2"/>
     </row>
-    <row r="2166" spans="1:2" ht="12.75">
+    <row r="2166" spans="1:2" ht="13.2">
       <c r="A2166" s="2"/>
       <c r="B2166" s="2"/>
     </row>
-    <row r="2167" spans="1:2" ht="12.75">
+    <row r="2167" spans="1:2" ht="13.2">
       <c r="A2167" s="2"/>
       <c r="B2167" s="2"/>
     </row>
-    <row r="2168" spans="1:2" ht="12.75">
+    <row r="2168" spans="1:2" ht="13.2">
       <c r="A2168" s="2"/>
       <c r="B2168" s="2"/>
     </row>
-    <row r="2169" spans="1:2" ht="12.75">
+    <row r="2169" spans="1:2" ht="13.2">
       <c r="A2169" s="2"/>
       <c r="B2169" s="2"/>
     </row>
-    <row r="2170" spans="1:2" ht="12.75">
+    <row r="2170" spans="1:2" ht="13.2">
       <c r="A2170" s="2"/>
       <c r="B2170" s="2"/>
     </row>
-    <row r="2171" spans="1:2" ht="12.75">
+    <row r="2171" spans="1:2" ht="13.2">
       <c r="A2171" s="2"/>
       <c r="B2171" s="2"/>
     </row>
-    <row r="2172" spans="1:2" ht="12.75">
+    <row r="2172" spans="1:2" ht="13.2">
       <c r="A2172" s="2"/>
       <c r="B2172" s="2"/>
     </row>
-    <row r="2173" spans="1:2" ht="12.75">
+    <row r="2173" spans="1:2" ht="13.2">
       <c r="A2173" s="2"/>
       <c r="B2173" s="2"/>
     </row>
-    <row r="2174" spans="1:2" ht="12.75">
+    <row r="2174" spans="1:2" ht="13.2">
       <c r="A2174" s="2"/>
       <c r="B2174" s="2"/>
     </row>
-    <row r="2175" spans="1:2" ht="12.75">
+    <row r="2175" spans="1:2" ht="13.2">
       <c r="A2175" s="2"/>
       <c r="B2175" s="2"/>
     </row>
-    <row r="2176" spans="1:2" ht="12.75">
+    <row r="2176" spans="1:2" ht="13.2">
       <c r="A2176" s="2"/>
       <c r="B2176" s="2"/>
     </row>
-    <row r="2177" spans="1:2" ht="12.75">
+    <row r="2177" spans="1:2" ht="13.2">
       <c r="A2177" s="2"/>
       <c r="B2177" s="2"/>
     </row>
-    <row r="2178" spans="1:2" ht="12.75">
+    <row r="2178" spans="1:2" ht="13.2">
       <c r="A2178" s="2"/>
       <c r="B2178" s="2"/>
     </row>
-    <row r="2179" spans="1:2" ht="12.75">
+    <row r="2179" spans="1:2" ht="13.2">
       <c r="A2179" s="2"/>
       <c r="B2179" s="2"/>
     </row>
-    <row r="2180" spans="1:2" ht="12.75">
+    <row r="2180" spans="1:2" ht="13.2">
       <c r="A2180" s="2"/>
       <c r="B2180" s="2"/>
     </row>
-    <row r="2181" spans="1:2" ht="12.75">
+    <row r="2181" spans="1:2" ht="13.2">
       <c r="A2181" s="2"/>
       <c r="B2181" s="2"/>
     </row>
-    <row r="2182" spans="1:2" ht="12.75">
+    <row r="2182" spans="1:2" ht="13.2">
       <c r="A2182" s="2"/>
       <c r="B2182" s="2"/>
     </row>
-    <row r="2183" spans="1:2" ht="12.75">
+    <row r="2183" spans="1:2" ht="13.2">
       <c r="A2183" s="2"/>
       <c r="B2183" s="2"/>
     </row>
-    <row r="2184" spans="1:2" ht="12.75">
+    <row r="2184" spans="1:2" ht="13.2">
       <c r="A2184" s="2"/>
       <c r="B2184" s="2"/>
     </row>
-    <row r="2185" spans="1:2" ht="12.75">
+    <row r="2185" spans="1:2" ht="13.2">
       <c r="A2185" s="2"/>
       <c r="B2185" s="2"/>
     </row>
-    <row r="2186" spans="1:2" ht="12.75">
+    <row r="2186" spans="1:2" ht="13.2">
       <c r="A2186" s="2"/>
       <c r="B2186" s="2"/>
     </row>
-    <row r="2187" spans="1:2" ht="12.75">
+    <row r="2187" spans="1:2" ht="13.2">
       <c r="A2187" s="2"/>
       <c r="B2187" s="2"/>
     </row>
-    <row r="2188" spans="1:2" ht="12.75">
+    <row r="2188" spans="1:2" ht="13.2">
       <c r="A2188" s="2"/>
       <c r="B2188" s="2"/>
     </row>
-    <row r="2189" spans="1:2" ht="12.75">
+    <row r="2189" spans="1:2" ht="13.2">
       <c r="A2189" s="2"/>
       <c r="B2189" s="2"/>
     </row>
-    <row r="2190" spans="1:2" ht="12.75">
+    <row r="2190" spans="1:2" ht="13.2">
       <c r="A2190" s="2"/>
       <c r="B2190" s="2"/>
     </row>
-    <row r="2191" spans="1:2" ht="12.75">
+    <row r="2191" spans="1:2" ht="13.2">
       <c r="A2191" s="2"/>
       <c r="B2191" s="2"/>
     </row>
-    <row r="2192" spans="1:2" ht="12.75">
+    <row r="2192" spans="1:2" ht="13.2">
       <c r="A2192" s="2"/>
       <c r="B2192" s="2"/>
     </row>
-    <row r="2193" spans="1:2" ht="12.75">
+    <row r="2193" spans="1:2" ht="13.2">
       <c r="A2193" s="2"/>
       <c r="B2193" s="2"/>
     </row>
-    <row r="2194" spans="1:2" ht="12.75">
+    <row r="2194" spans="1:2" ht="13.2">
       <c r="A2194" s="2"/>
       <c r="B2194" s="2"/>
     </row>
-    <row r="2195" spans="1:2" ht="12.75">
+    <row r="2195" spans="1:2" ht="13.2">
       <c r="A2195" s="2"/>
       <c r="B2195" s="2"/>
     </row>
-    <row r="2196" spans="1:2" ht="12.75">
+    <row r="2196" spans="1:2" ht="13.2">
       <c r="A2196" s="2"/>
       <c r="B2196" s="2"/>
     </row>
-    <row r="2197" spans="1:2" ht="12.75">
+    <row r="2197" spans="1:2" ht="13.2">
       <c r="A2197" s="2"/>
       <c r="B2197" s="2"/>
     </row>
-    <row r="2198" spans="1:2" ht="12.75">
+    <row r="2198" spans="1:2" ht="13.2">
       <c r="A2198" s="2"/>
       <c r="B2198" s="2"/>
     </row>
-    <row r="2199" spans="1:2" ht="12.75">
+    <row r="2199" spans="1:2" ht="13.2">
       <c r="A2199" s="2"/>
       <c r="B2199" s="2"/>
     </row>
-    <row r="2200" spans="1:2" ht="12.75">
+    <row r="2200" spans="1:2" ht="13.2">
       <c r="A2200" s="2"/>
       <c r="B2200" s="2"/>
     </row>
-    <row r="2201" spans="1:2" ht="12.75">
+    <row r="2201" spans="1:2" ht="13.2">
       <c r="A2201" s="2"/>
       <c r="B2201" s="2"/>
     </row>
-    <row r="2202" spans="1:2" ht="12.75">
+    <row r="2202" spans="1:2" ht="13.2">
       <c r="A2202" s="2"/>
       <c r="B2202" s="2"/>
     </row>
-    <row r="2203" spans="1:2" ht="12.75">
+    <row r="2203" spans="1:2" ht="13.2">
       <c r="A2203" s="2"/>
       <c r="B2203" s="2"/>
     </row>
-    <row r="2204" spans="1:2" ht="12.75">
+    <row r="2204" spans="1:2" ht="13.2">
       <c r="A2204" s="2"/>
       <c r="B2204" s="2"/>
     </row>
-    <row r="2205" spans="1:2" ht="12.75">
+    <row r="2205" spans="1:2" ht="13.2">
       <c r="A2205" s="2"/>
       <c r="B2205" s="2"/>
     </row>
-    <row r="2206" spans="1:2" ht="12.75">
+    <row r="2206" spans="1:2" ht="13.2">
       <c r="A2206" s="2"/>
       <c r="B2206" s="2"/>
     </row>
-    <row r="2207" spans="1:2" ht="12.75">
+    <row r="2207" spans="1:2" ht="13.2">
       <c r="A2207" s="2"/>
       <c r="B2207" s="2"/>
     </row>
-    <row r="2208" spans="1:2" ht="12.75">
+    <row r="2208" spans="1:2" ht="13.2">
       <c r="A2208" s="2"/>
       <c r="B2208" s="2"/>
     </row>
-    <row r="2209" spans="1:2" ht="12.75">
+    <row r="2209" spans="1:2" ht="13.2">
       <c r="A2209" s="2"/>
       <c r="B2209" s="2"/>
     </row>
-    <row r="2210" spans="1:2" ht="12.75">
+    <row r="2210" spans="1:2" ht="13.2">
       <c r="A2210" s="2"/>
       <c r="B2210" s="2"/>
     </row>
-    <row r="2211" spans="1:2" ht="12.75">
+    <row r="2211" spans="1:2" ht="13.2">
       <c r="A2211" s="2"/>
       <c r="B2211" s="2"/>
     </row>
-    <row r="2212" spans="1:2" ht="12.75">
+    <row r="2212" spans="1:2" ht="13.2">
       <c r="A2212" s="2"/>
       <c r="B2212" s="2"/>
     </row>
-    <row r="2213" spans="1:2" ht="12.75">
+    <row r="2213" spans="1:2" ht="13.2">
       <c r="A2213" s="2"/>
       <c r="B2213" s="2"/>
     </row>
-    <row r="2214" spans="1:2" ht="12.75">
+    <row r="2214" spans="1:2" ht="13.2">
       <c r="A2214" s="2"/>
       <c r="B2214" s="2"/>
     </row>
-    <row r="2215" spans="1:2" ht="12.75">
+    <row r="2215" spans="1:2" ht="13.2">
       <c r="A2215" s="2"/>
       <c r="B2215" s="2"/>
     </row>
-    <row r="2216" spans="1:2" ht="12.75">
+    <row r="2216" spans="1:2" ht="13.2">
       <c r="A2216" s="2"/>
       <c r="B2216" s="2"/>
     </row>
-    <row r="2217" spans="1:2" ht="12.75">
+    <row r="2217" spans="1:2" ht="13.2">
       <c r="A2217" s="2"/>
       <c r="B2217" s="2"/>
     </row>
-    <row r="2218" spans="1:2" ht="12.75">
+    <row r="2218" spans="1:2" ht="13.2">
       <c r="A2218" s="2"/>
       <c r="B2218" s="2"/>
     </row>
-    <row r="2219" spans="1:2" ht="12.75">
+    <row r="2219" spans="1:2" ht="13.2">
       <c r="A2219" s="2"/>
       <c r="B2219" s="2"/>
     </row>
-    <row r="2220" spans="1:2" ht="12.75">
+    <row r="2220" spans="1:2" ht="13.2">
       <c r="A2220" s="2"/>
       <c r="B2220" s="2"/>
     </row>
-    <row r="2221" spans="1:2" ht="12.75">
+    <row r="2221" spans="1:2" ht="13.2">
       <c r="A2221" s="2"/>
       <c r="B2221" s="2"/>
     </row>
-    <row r="2222" spans="1:2" ht="12.75">
+    <row r="2222" spans="1:2" ht="13.2">
       <c r="A2222" s="2"/>
       <c r="B2222" s="2"/>
     </row>
-    <row r="2223" spans="1:2" ht="12.75">
+    <row r="2223" spans="1:2" ht="13.2">
       <c r="A2223" s="2"/>
       <c r="B2223" s="2"/>
     </row>
-    <row r="2224" spans="1:2" ht="12.75">
+    <row r="2224" spans="1:2" ht="13.2">
       <c r="A2224" s="2"/>
       <c r="B2224" s="2"/>
     </row>
-    <row r="2225" spans="1:2" ht="12.75">
+    <row r="2225" spans="1:2" ht="13.2">
       <c r="A2225" s="2"/>
       <c r="B2225" s="2"/>
     </row>
-    <row r="2226" spans="1:2" ht="12.75">
+    <row r="2226" spans="1:2" ht="13.2">
       <c r="A2226" s="2"/>
       <c r="B2226" s="2"/>
     </row>
-    <row r="2227" spans="1:2" ht="12.75">
+    <row r="2227" spans="1:2" ht="13.2">
       <c r="A2227" s="2"/>
       <c r="B2227" s="2"/>
     </row>
-    <row r="2228" spans="1:2" ht="12.75">
+    <row r="2228" spans="1:2" ht="13.2">
       <c r="A2228" s="2"/>
       <c r="B2228" s="2"/>
     </row>
-    <row r="2229" spans="1:2" ht="12.75">
+    <row r="2229" spans="1:2" ht="13.2">
       <c r="A2229" s="2"/>
       <c r="B2229" s="2"/>
     </row>
-    <row r="2230" spans="1:2" ht="12.75">
+    <row r="2230" spans="1:2" ht="13.2">
       <c r="A2230" s="2"/>
       <c r="B2230" s="2"/>
     </row>
-    <row r="2231" spans="1:2" ht="12.75">
+    <row r="2231" spans="1:2" ht="13.2">
       <c r="A2231" s="2"/>
       <c r="B2231" s="2"/>
     </row>
-    <row r="2232" spans="1:2" ht="12.75">
+    <row r="2232" spans="1:2" ht="13.2">
       <c r="A2232" s="2"/>
       <c r="B2232" s="2"/>
     </row>
-    <row r="2233" spans="1:2" ht="12.75">
+    <row r="2233" spans="1:2" ht="13.2">
       <c r="A2233" s="2"/>
       <c r="B2233" s="2"/>
     </row>
-    <row r="2234" spans="1:2" ht="12.75">
+    <row r="2234" spans="1:2" ht="13.2">
       <c r="A2234" s="2"/>
       <c r="B2234" s="2"/>
     </row>
-    <row r="2235" spans="1:2" ht="12.75">
+    <row r="2235" spans="1:2" ht="13.2">
       <c r="A2235" s="2"/>
       <c r="B2235" s="2"/>
     </row>
-    <row r="2236" spans="1:2" ht="12.75">
+    <row r="2236" spans="1:2" ht="13.2">
       <c r="A2236" s="2"/>
       <c r="B2236" s="2"/>
     </row>
-    <row r="2237" spans="1:2" ht="12.75">
+    <row r="2237" spans="1:2" ht="13.2">
       <c r="A2237" s="2"/>
       <c r="B2237" s="2"/>
     </row>
-    <row r="2238" spans="1:2" ht="12.75">
+    <row r="2238" spans="1:2" ht="13.2">
       <c r="A2238" s="2"/>
       <c r="B2238" s="2"/>
     </row>
-    <row r="2239" spans="1:2" ht="12.75">
+    <row r="2239" spans="1:2" ht="13.2">
       <c r="A2239" s="2"/>
       <c r="B2239" s="2"/>
     </row>
-    <row r="2240" spans="1:2" ht="12.75">
+    <row r="2240" spans="1:2" ht="13.2">
       <c r="A2240" s="2"/>
       <c r="B2240" s="2"/>
     </row>
-    <row r="2241" spans="1:2" ht="12.75">
+    <row r="2241" spans="1:2" ht="13.2">
       <c r="A2241" s="2"/>
       <c r="B2241" s="2"/>
     </row>
-    <row r="2242" spans="1:2" ht="12.75">
+    <row r="2242" spans="1:2" ht="13.2">
       <c r="A2242" s="2"/>
       <c r="B2242" s="2"/>
     </row>
-    <row r="2243" spans="1:2" ht="12.75">
+    <row r="2243" spans="1:2" ht="13.2">
       <c r="A2243" s="2"/>
       <c r="B2243" s="2"/>
     </row>
-    <row r="2244" spans="1:2" ht="12.75">
+    <row r="2244" spans="1:2" ht="13.2">
       <c r="A2244" s="2"/>
       <c r="B2244" s="2"/>
     </row>
-    <row r="2245" spans="1:2" ht="12.75">
+    <row r="2245" spans="1:2" ht="13.2">
       <c r="A2245" s="2"/>
       <c r="B2245" s="2"/>
     </row>
-    <row r="2246" spans="1:2" ht="12.75">
+    <row r="2246" spans="1:2" ht="13.2">
       <c r="A2246" s="2"/>
       <c r="B2246" s="2"/>
     </row>
-    <row r="2247" spans="1:2" ht="12.75">
+    <row r="2247" spans="1:2" ht="13.2">
       <c r="A2247" s="2"/>
       <c r="B2247" s="2"/>
     </row>
-    <row r="2248" spans="1:2" ht="12.75">
+    <row r="2248" spans="1:2" ht="13.2">
       <c r="A2248" s="2"/>
       <c r="B2248" s="2"/>
     </row>
-    <row r="2249" spans="1:2" ht="12.75">
+    <row r="2249" spans="1:2" ht="13.2">
       <c r="A2249" s="2"/>
       <c r="B2249" s="2"/>
     </row>
-    <row r="2250" spans="1:2" ht="12.75">
+    <row r="2250" spans="1:2" ht="13.2">
       <c r="A2250" s="2"/>
       <c r="B2250" s="2"/>
     </row>
-    <row r="2251" spans="1:2" ht="12.75">
+    <row r="2251" spans="1:2" ht="13.2">
       <c r="A2251" s="2"/>
       <c r="B2251" s="2"/>
     </row>
-    <row r="2252" spans="1:2" ht="12.75">
+    <row r="2252" spans="1:2" ht="13.2">
       <c r="A2252" s="2"/>
       <c r="B2252" s="2"/>
     </row>
-    <row r="2253" spans="1:2" ht="12.75">
+    <row r="2253" spans="1:2" ht="13.2">
       <c r="A2253" s="2"/>
       <c r="B2253" s="2"/>
     </row>
-    <row r="2254" spans="1:2" ht="12.75">
+    <row r="2254" spans="1:2" ht="13.2">
       <c r="A2254" s="2"/>
       <c r="B2254" s="2"/>
     </row>
-    <row r="2255" spans="1:2" ht="12.75">
+    <row r="2255" spans="1:2" ht="13.2">
       <c r="A2255" s="2"/>
       <c r="B2255" s="2"/>
     </row>
-    <row r="2256" spans="1:2" ht="12.75">
+    <row r="2256" spans="1:2" ht="13.2">
       <c r="A2256" s="2"/>
       <c r="B2256" s="2"/>
     </row>
-    <row r="2257" spans="1:2" ht="12.75">
+    <row r="2257" spans="1:2" ht="13.2">
       <c r="A2257" s="2"/>
       <c r="B2257" s="2"/>
     </row>
-    <row r="2258" spans="1:2" ht="12.75">
+    <row r="2258" spans="1:2" ht="13.2">
       <c r="A2258" s="2"/>
       <c r="B2258" s="2"/>
     </row>
-    <row r="2259" spans="1:2" ht="12.75">
+    <row r="2259" spans="1:2" ht="13.2">
       <c r="A2259" s="2"/>
       <c r="B2259" s="2"/>
     </row>
-    <row r="2260" spans="1:2" ht="12.75">
+    <row r="2260" spans="1:2" ht="13.2">
       <c r="A2260" s="2"/>
       <c r="B2260" s="2"/>
     </row>
-    <row r="2261" spans="1:2" ht="12.75">
+    <row r="2261" spans="1:2" ht="13.2">
       <c r="A2261" s="2"/>
       <c r="B2261" s="2"/>
     </row>
-    <row r="2262" spans="1:2" ht="12.75">
+    <row r="2262" spans="1:2" ht="13.2">
       <c r="A2262" s="2"/>
       <c r="B2262" s="2"/>
     </row>
-    <row r="2263" spans="1:2" ht="12.75">
+    <row r="2263" spans="1:2" ht="13.2">
       <c r="A2263" s="2"/>
       <c r="B2263" s="2"/>
     </row>
-    <row r="2264" spans="1:2" ht="12.75">
+    <row r="2264" spans="1:2" ht="13.2">
       <c r="A2264" s="2"/>
       <c r="B2264" s="2"/>
     </row>
-    <row r="2265" spans="1:2" ht="12.75">
+    <row r="2265" spans="1:2" ht="13.2">
       <c r="A2265" s="2"/>
       <c r="B2265" s="2"/>
     </row>
-    <row r="2266" spans="1:2" ht="12.75">
+    <row r="2266" spans="1:2" ht="13.2">
       <c r="A2266" s="2"/>
       <c r="B2266" s="2"/>
     </row>
-    <row r="2267" spans="1:2" ht="12.75">
+    <row r="2267" spans="1:2" ht="13.2">
       <c r="A2267" s="2"/>
       <c r="B2267" s="2"/>
     </row>
-    <row r="2268" spans="1:2" ht="12.75">
+    <row r="2268" spans="1:2" ht="13.2">
       <c r="A2268" s="2"/>
       <c r="B2268" s="2"/>
     </row>
-    <row r="2269" spans="1:2" ht="12.75">
+    <row r="2269" spans="1:2" ht="13.2">
       <c r="A2269" s="2"/>
       <c r="B2269" s="2"/>
     </row>
-    <row r="2270" spans="1:2" ht="12.75">
+    <row r="2270" spans="1:2" ht="13.2">
       <c r="A2270" s="2"/>
       <c r="B2270" s="2"/>
     </row>
-    <row r="2271" spans="1:2" ht="12.75">
+    <row r="2271" spans="1:2" ht="13.2">
       <c r="A2271" s="2"/>
       <c r="B2271" s="2"/>
     </row>
-    <row r="2272" spans="1:2" ht="12.75">
+    <row r="2272" spans="1:2" ht="13.2">
       <c r="A2272" s="2"/>
       <c r="B2272" s="2"/>
     </row>
-    <row r="2273" spans="1:2" ht="12.75">
+    <row r="2273" spans="1:2" ht="13.2">
       <c r="A2273" s="2"/>
       <c r="B2273" s="2"/>
     </row>
-    <row r="2274" spans="1:2" ht="12.75">
+    <row r="2274" spans="1:2" ht="13.2">
       <c r="A2274" s="2"/>
       <c r="B2274" s="2"/>
     </row>
-    <row r="2275" spans="1:2" ht="12.75">
+    <row r="2275" spans="1:2" ht="13.2">
       <c r="A2275" s="2"/>
       <c r="B2275" s="2"/>
     </row>
-    <row r="2276" spans="1:2" ht="12.75">
+    <row r="2276" spans="1:2" ht="13.2">
       <c r="A2276" s="2"/>
       <c r="B2276" s="2"/>
     </row>
-    <row r="2277" spans="1:2" ht="12.75">
+    <row r="2277" spans="1:2" ht="13.2">
       <c r="A2277" s="2"/>
       <c r="B2277" s="2"/>
     </row>
-    <row r="2278" spans="1:2" ht="12.75">
+    <row r="2278" spans="1:2" ht="13.2">
       <c r="A2278" s="2"/>
       <c r="B2278" s="2"/>
     </row>
-    <row r="2279" spans="1:2" ht="12.75">
+    <row r="2279" spans="1:2" ht="13.2">
       <c r="A2279" s="2"/>
       <c r="B2279" s="2"/>
     </row>
-    <row r="2280" spans="1:2" ht="12.75">
+    <row r="2280" spans="1:2" ht="13.2">
       <c r="A2280" s="2"/>
       <c r="B2280" s="2"/>
     </row>
-    <row r="2281" spans="1:2" ht="12.75">
+    <row r="2281" spans="1:2" ht="13.2">
       <c r="A2281" s="2"/>
       <c r="B2281" s="2"/>
     </row>
-    <row r="2282" spans="1:2" ht="12.75">
+    <row r="2282" spans="1:2" ht="13.2">
       <c r="A2282" s="2"/>
       <c r="B2282" s="2"/>
     </row>
-    <row r="2283" spans="1:2" ht="12.75">
+    <row r="2283" spans="1:2" ht="13.2">
       <c r="A2283" s="2"/>
       <c r="B2283" s="2"/>
     </row>
-    <row r="2284" spans="1:2" ht="12.75">
+    <row r="2284" spans="1:2" ht="13.2">
       <c r="A2284" s="2"/>
       <c r="B2284" s="2"/>
     </row>
-    <row r="2285" spans="1:2" ht="12.75">
+    <row r="2285" spans="1:2" ht="13.2">
       <c r="A2285" s="2"/>
       <c r="B2285" s="2"/>
     </row>
-    <row r="2286" spans="1:2" ht="12.75">
+    <row r="2286" spans="1:2" ht="13.2">
       <c r="A2286" s="2"/>
       <c r="B2286" s="2"/>
     </row>
-    <row r="2287" spans="1:2" ht="12.75">
+    <row r="2287" spans="1:2" ht="13.2">
       <c r="A2287" s="2"/>
       <c r="B2287" s="2"/>
     </row>
-    <row r="2288" spans="1:2" ht="12.75">
+    <row r="2288" spans="1:2" ht="13.2">
       <c r="A2288" s="2"/>
       <c r="B2288" s="2"/>
     </row>
-    <row r="2289" spans="1:2" ht="12.75">
+    <row r="2289" spans="1:2" ht="13.2">
       <c r="A2289" s="2"/>
       <c r="B2289" s="2"/>
     </row>
-    <row r="2290" spans="1:2" ht="12.75">
+    <row r="2290" spans="1:2" ht="13.2">
       <c r="A2290" s="2"/>
       <c r="B2290" s="2"/>
     </row>
-    <row r="2291" spans="1:2" ht="12.75">
+    <row r="2291" spans="1:2" ht="13.2">
       <c r="A2291" s="2"/>
       <c r="B2291" s="2"/>
     </row>
-    <row r="2292" spans="1:2" ht="12.75">
+    <row r="2292" spans="1:2" ht="13.2">
       <c r="A2292" s="2"/>
       <c r="B2292" s="2"/>
     </row>
-    <row r="2293" spans="1:2" ht="12.75">
+    <row r="2293" spans="1:2" ht="13.2">
       <c r="A2293" s="2"/>
       <c r="B2293" s="2"/>
     </row>
-    <row r="2294" spans="1:2" ht="12.75">
+    <row r="2294" spans="1:2" ht="13.2">
       <c r="A2294" s="2"/>
       <c r="B2294" s="2"/>
     </row>
-    <row r="2295" spans="1:2" ht="12.75">
+    <row r="2295" spans="1:2" ht="13.2">
       <c r="A2295" s="2"/>
       <c r="B2295" s="2"/>
     </row>
-    <row r="2296" spans="1:2" ht="12.75">
+    <row r="2296" spans="1:2" ht="13.2">
       <c r="A2296" s="2"/>
       <c r="B2296" s="2"/>
     </row>
-    <row r="2297" spans="1:2" ht="12.75">
+    <row r="2297" spans="1:2" ht="13.2">
       <c r="A2297" s="2"/>
       <c r="B2297" s="2"/>
     </row>
-    <row r="2298" spans="1:2" ht="12.75">
+    <row r="2298" spans="1:2" ht="13.2">
       <c r="A2298" s="2"/>
       <c r="B2298" s="2"/>
     </row>
-    <row r="2299" spans="1:2" ht="12.75">
+    <row r="2299" spans="1:2" ht="13.2">
       <c r="A2299" s="2"/>
       <c r="B2299" s="2"/>
     </row>
-    <row r="2300" spans="1:2" ht="12.75">
+    <row r="2300" spans="1:2" ht="13.2">
       <c r="A2300" s="2"/>
       <c r="B2300" s="2"/>
     </row>
-    <row r="2301" spans="1:2" ht="12.75">
+    <row r="2301" spans="1:2" ht="13.2">
       <c r="A2301" s="2"/>
       <c r="B2301" s="2"/>
     </row>
-    <row r="2302" spans="1:2" ht="12.75">
+    <row r="2302" spans="1:2" ht="13.2">
       <c r="A2302" s="2"/>
       <c r="B2302" s="2"/>
     </row>
-    <row r="2303" spans="1:2" ht="12.75">
+    <row r="2303" spans="1:2" ht="13.2">
       <c r="A2303" s="2"/>
       <c r="B2303" s="2"/>
     </row>
-    <row r="2304" spans="1:2" ht="12.75">
+    <row r="2304" spans="1:2" ht="13.2">
       <c r="A2304" s="2"/>
       <c r="B2304" s="2"/>
     </row>
-    <row r="2305" spans="1:2" ht="12.75">
+    <row r="2305" spans="1:2" ht="13.2">
       <c r="A2305" s="2"/>
       <c r="B2305" s="2"/>
     </row>
-    <row r="2306" spans="1:2" ht="12.75">
+    <row r="2306" spans="1:2" ht="13.2">
       <c r="A2306" s="2"/>
       <c r="B2306" s="2"/>
     </row>
-    <row r="2307" spans="1:2" ht="12.75">
+    <row r="2307" spans="1:2" ht="13.2">
       <c r="A2307" s="2"/>
       <c r="B2307" s="2"/>
     </row>
-    <row r="2308" spans="1:2" ht="12.75">
+    <row r="2308" spans="1:2" ht="13.2">
       <c r="A2308" s="2"/>
       <c r="B2308" s="2"/>
     </row>
-    <row r="2309" spans="1:2" ht="12.75">
+    <row r="2309" spans="1:2" ht="13.2">
       <c r="A2309" s="2"/>
       <c r="B2309" s="2"/>
     </row>
-    <row r="2310" spans="1:2" ht="12.75">
+    <row r="2310" spans="1:2" ht="13.2">
       <c r="A2310" s="2"/>
       <c r="B2310" s="2"/>
     </row>
-    <row r="2311" spans="1:2" ht="12.75">
+    <row r="2311" spans="1:2" ht="13.2">
       <c r="A2311" s="2"/>
       <c r="B2311" s="2"/>
     </row>
-    <row r="2312" spans="1:2" ht="12.75">
+    <row r="2312" spans="1:2" ht="13.2">
       <c r="A2312" s="2"/>
       <c r="B2312" s="2"/>
     </row>
-    <row r="2313" spans="1:2" ht="12.75">
+    <row r="2313" spans="1:2" ht="13.2">
       <c r="A2313" s="2"/>
       <c r="B2313" s="2"/>
     </row>
-    <row r="2314" spans="1:2" ht="12.75">
+    <row r="2314" spans="1:2" ht="13.2">
       <c r="A2314" s="2"/>
       <c r="B2314" s="2"/>
     </row>
-    <row r="2315" spans="1:2" ht="12.75">
+    <row r="2315" spans="1:2" ht="13.2">
       <c r="A2315" s="2"/>
       <c r="B2315" s="2"/>
     </row>
-    <row r="2316" spans="1:2" ht="12.75">
+    <row r="2316" spans="1:2" ht="13.2">
       <c r="A2316" s="2"/>
       <c r="B2316" s="2"/>
     </row>
-    <row r="2317" spans="1:2" ht="12.75">
+    <row r="2317" spans="1:2" ht="13.2">
       <c r="A2317" s="2"/>
       <c r="B2317" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M14" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:M25" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="ABIERTO"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="A1">
-    <cfRule type="containsText" dxfId="104" priority="757" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="60" priority="757" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="103" priority="762" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="59" priority="762" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",A1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="763" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="763" stopIfTrue="1" operator="equal">
       <formula>"OPEN"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="101" priority="755" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="57" priority="755" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="100" priority="756" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="56" priority="756" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",A1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="99" priority="764" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="764" stopIfTrue="1" operator="equal">
       <formula>"CLOSED"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="98" priority="758" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="54" priority="758" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="97" priority="759" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="53" priority="759" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",A1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="765" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="765" stopIfTrue="1" operator="equal">
       <formula>"IN PROGRESS"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="95" priority="761" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="51" priority="761" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1 D1 D26:D1048576">
-    <cfRule type="containsText" dxfId="94" priority="760" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="50" priority="760" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="containsText" dxfId="93" priority="408" operator="containsText" text="PENDIENTE">
+    <cfRule type="containsText" dxfId="49" priority="408" operator="containsText" text="PENDIENTE">
       <formula>NOT(ISERROR(SEARCH("PENDIENTE",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1">
-    <cfRule type="containsText" dxfId="92" priority="1792" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="48" priority="1792" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="91" priority="1791" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="47" priority="1791" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="90" priority="1790" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="46" priority="1790" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="89" priority="1793" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="45" priority="1793" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="88" priority="1789" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="44" priority="1789" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="87" priority="1788" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="43" priority="1788" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="86" priority="1794" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="42" priority="1794" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",B1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="85" priority="1795" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="41" priority="1795" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",B1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="1796" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="1796" stopIfTrue="1" operator="equal">
       <formula>"OPEN"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="1797" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="1797" stopIfTrue="1" operator="equal">
       <formula>"CLOSED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="1798" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="1798" stopIfTrue="1" operator="equal">
       <formula>"IN PROGRESS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="containsText" dxfId="81" priority="382" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="37" priority="382" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="80" priority="384" operator="containsText" text="SHOWSTOPPER">
+    <cfRule type="containsText" dxfId="36" priority="384" operator="containsText" text="SHOWSTOPPER">
       <formula>NOT(ISERROR(SEARCH("SHOWSTOPPER",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="79" priority="385" operator="containsText" text="show">
+    <cfRule type="containsText" dxfId="35" priority="385" operator="containsText" text="show">
       <formula>NOT(ISERROR(SEARCH("show",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="78" priority="386" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="34" priority="386" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="77" priority="387" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="33" priority="387" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="76" priority="1901" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="32" priority="1901" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="75" priority="1896" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="31" priority="1896" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="74" priority="1897" operator="containsText" text="Showstopper ">
+    <cfRule type="containsText" dxfId="30" priority="1897" operator="containsText" text="Showstopper ">
       <formula>NOT(ISERROR(SEARCH("Showstopper ",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="73" priority="1902" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="29" priority="1902" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="1903" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="1903" stopIfTrue="1" operator="equal">
       <formula>"Medio"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="71" priority="1904" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="1904" stopIfTrue="1" operator="equal">
       <formula>"Bajo"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="1905" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="1905" stopIfTrue="1" operator="equal">
       <formula>"Alto"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C14">
-    <cfRule type="containsText" dxfId="69" priority="46" operator="containsText" text="MEDIO">
+  <conditionalFormatting sqref="C2:C25">
+    <cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="68" priority="48" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="24" priority="4" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="67" priority="45" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="23" priority="1" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C26:C1048576">
-    <cfRule type="containsText" dxfId="66" priority="1337" operator="containsText" text="MEDIO">
+    <cfRule type="containsText" dxfId="22" priority="1337" operator="containsText" text="MEDIO">
       <formula>NOT(ISERROR(SEARCH("MEDIO",C26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="65" priority="1338" operator="containsText" text="ALTO">
+    <cfRule type="containsText" dxfId="21" priority="1338" operator="containsText" text="ALTO">
       <formula>NOT(ISERROR(SEARCH("ALTO",C26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="64" priority="1333" operator="containsText" text="BAJA">
+    <cfRule type="containsText" dxfId="20" priority="1333" operator="containsText" text="BAJA">
       <formula>NOT(ISERROR(SEARCH("BAJA",C26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="63" priority="1335" operator="containsText" text="SHOWSTOPPER">
+    <cfRule type="containsText" dxfId="19" priority="1335" operator="containsText" text="SHOWSTOPPER">
       <formula>NOT(ISERROR(SEARCH("SHOWSTOPPER",C26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="62" priority="1336" operator="containsText" text="show">
+    <cfRule type="containsText" dxfId="18" priority="1336" operator="containsText" text="show">
       <formula>NOT(ISERROR(SEARCH("show",C26)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1 D26:D1048576">
-    <cfRule type="containsText" dxfId="61" priority="1813" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="17" priority="1813" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="60" priority="1814" operator="containsText" text="EN PROGRESO">
+    <cfRule type="containsText" dxfId="16" priority="1814" operator="containsText" text="EN PROGRESO">
       <formula>NOT(ISERROR(SEARCH("EN PROGRESO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="59" priority="1815" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="15" priority="1815" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="58" priority="1816" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="14" priority="1816" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="57" priority="249" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="13" priority="249" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="56" priority="241" operator="containsText" text="NO APLICA">
+    <cfRule type="containsText" dxfId="12" priority="241" operator="containsText" text="NO APLICA">
       <formula>NOT(ISERROR(SEARCH("NO APLICA",D1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="containsText" dxfId="55" priority="1895" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="11" priority="1895" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="54" priority="1774" operator="containsText" text="PENDIENTE">
+    <cfRule type="containsText" dxfId="10" priority="1774" operator="containsText" text="PENDIENTE">
       <formula>NOT(ISERROR(SEARCH("PENDIENTE",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="53" priority="1779" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="9" priority="1779" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="52" priority="1898" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="8" priority="1898" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="51" priority="1899" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="7" priority="1899" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="50" priority="1900" operator="containsText" text="ABIERTO">
+    <cfRule type="containsText" dxfId="6" priority="1900" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="1906" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="1906" stopIfTrue="1" operator="equal">
       <formula>"OPEN"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="1907" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="1907" stopIfTrue="1" operator="equal">
       <formula>"CLOSED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="1908" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="1908" stopIfTrue="1" operator="equal">
       <formula>"IN PROGRESS"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D14">
-    <cfRule type="containsText" dxfId="46" priority="47" operator="containsText" text="ABIERTO">
+  <conditionalFormatting sqref="D2:D25">
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",D2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D26:D1048576">
-    <cfRule type="containsText" dxfId="45" priority="1542" operator="containsText" text="CERRADO">
+    <cfRule type="containsText" dxfId="1" priority="1542" operator="containsText" text="CERRADO">
       <formula>NOT(ISERROR(SEARCH("CERRADO",D26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="44" priority="1339" operator="containsText" text="PENDIENTE">
+    <cfRule type="containsText" dxfId="0" priority="1339" operator="containsText" text="PENDIENTE">
       <formula>NOT(ISERROR(SEARCH("PENDIENTE",D26)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C15">
-    <cfRule type="containsText" dxfId="43" priority="41" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="42" priority="42" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="41" priority="44" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C15)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D15">
-    <cfRule type="containsText" dxfId="40" priority="43" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D15)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C16">
-    <cfRule type="containsText" dxfId="39" priority="37" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C16)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="38" priority="38" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C16)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="37" priority="40" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C16)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D16">
-    <cfRule type="containsText" dxfId="36" priority="39" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D16)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C17">
-    <cfRule type="containsText" dxfId="35" priority="33" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C17)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="34" priority="34" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C17)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="33" priority="36" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C17)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D17">
-    <cfRule type="containsText" dxfId="32" priority="35" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D17)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C18">
-    <cfRule type="containsText" dxfId="31" priority="29" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C18)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="30" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C18)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="29" priority="32" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C18)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D18">
-    <cfRule type="containsText" dxfId="28" priority="31" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D18)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C19">
-    <cfRule type="containsText" dxfId="27" priority="25" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C19)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="26" priority="26" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C19)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="25" priority="28" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C19)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D19">
-    <cfRule type="containsText" dxfId="24" priority="27" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D19)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C20">
-    <cfRule type="containsText" dxfId="23" priority="21" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C20)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="22" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C20)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="24" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C20)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D20">
-    <cfRule type="containsText" dxfId="20" priority="23" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D20)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C21">
-    <cfRule type="containsText" dxfId="19" priority="17" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C21)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="18" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C21)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="20" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C21)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D21">
-    <cfRule type="containsText" dxfId="16" priority="19" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D21)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C22">
-    <cfRule type="containsText" dxfId="15" priority="13" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C22)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="14" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C22)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="16" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C22)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D22">
-    <cfRule type="containsText" dxfId="12" priority="15" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D22)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C23">
-    <cfRule type="containsText" dxfId="11" priority="9" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C23)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="10" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C23)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="12" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C23)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D23">
-    <cfRule type="containsText" dxfId="8" priority="11" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D23)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C24">
-    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C24)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="6" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C24)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="8" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C24)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D24">
-    <cfRule type="containsText" dxfId="4" priority="7" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D24)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C25">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="ALTO">
-      <formula>NOT(ISERROR(SEARCH("ALTO",C25)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="MEDIO">
-      <formula>NOT(ISERROR(SEARCH("MEDIO",C25)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="BAJA">
-      <formula>NOT(ISERROR(SEARCH("BAJA",C25)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D25">
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="ABIERTO">
-      <formula>NOT(ISERROR(SEARCH("ABIERTO",D25)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
@@ -17524,12 +16827,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02A2ABB5-42B5-497D-950A-71A244302DF4}">
   <dimension ref="B1:J19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2"/>
   <cols>
-    <col min="2" max="2" width="24.42578125" customWidth="1"/>
-    <col min="3" max="3" width="31.42578125" customWidth="1"/>
-    <col min="4" max="4" width="46.42578125" customWidth="1"/>
-    <col min="5" max="5" width="26.42578125" customWidth="1"/>
+    <col min="2" max="2" width="24.44140625" customWidth="1"/>
+    <col min="3" max="3" width="31.44140625" customWidth="1"/>
+    <col min="4" max="4" width="46.44140625" customWidth="1"/>
+    <col min="5" max="5" width="26.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:10" s="1" customFormat="1" ht="55.35" customHeight="1">

</xml_diff>